<commit_message>
Mark sample lead source as Landing Page
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -514,7 +514,11 @@
 Tolong bantu cek harga dan stocknya ya Kak!</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 30 leads WA batch (1-4 Sept 2026, Landing Page & Meta Ads)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -520,6 +520,1070 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1800-5181</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Andrejazz</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Daihatsu
+Tipe Mobil: Sirion
+Tahun Mobil: 2013
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9618-9434</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Deden Kosasih</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-7437-5250</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ifandi rizal</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-7629-9939</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>💥⭐🔄🌟⭐</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6270-0088</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Mang Se</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-3943-9242</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>mAs koko_ituaku</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7460-7432</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Ahmad "AcHiL" Nurdiansyah</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7685-311</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>rusmawane3</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>01:10</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-5329-1400</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Dokter Michael</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1969-5362</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Aguskowo</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>01:36</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1156-8273</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Arkanul otoluwa</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>02:20</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5299-1759</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>zuka</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>01:42</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare pagi  bos  mantel</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4066-9930</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hanny Maanari</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>04:31</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-2787-3675</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Mas'ud</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>04:51</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-5621-1212</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Edwin</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Klo innova reborn hrga brp? (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-916-681</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>imamsayogo</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Klo buat mbl lancer Sl Th 82 ada kah.... (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4540-3041</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Imanuel Tandi</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4249-8171</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Farid</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>00:48</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6212-6777</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Oberlin Sahat Hisar Lubis</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>04:39</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1155-3672</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ferisandrea48</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4424-0572</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>04:40</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4555-2228</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>45RUL T4N3T3 🗡️</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>06:05</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brv</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6014-1085</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Parwata</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8820-5736</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Andy</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: honda
+Tipe Mobil: mobilio
+Tahun Mobil: 2018
+Nama Penerima: andy geby
+Alamat Penerima: jln.barukang 2, kecamatan ujing tanah, kelurahan pattingaloang, makasar
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3079-5658</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>altaf jaya</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-8316-2228</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>suparman zeal</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>04:31</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3792-4503</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Bambang Gd Ariawan</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3323-3329</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Dodi Syaputra</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>04:43</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6444-0944</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>prayitno</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>00:56</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3385-3739</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Wawan</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 14 more leads WA batch (1 & 3 Sept 2026, Meta Ads)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1584,6 +1584,496 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8696-1101</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1899-2637</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>budhiprabowoprabowo</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>06:17</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6161-1976</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Akheng</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-2224-5163</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>komjenbudigunawan123</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4248-0355</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>4770"YS</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4047-3277</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Anita</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9958-4921</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Pak</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0611-3635</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Eddy Mardiyanto</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-4652-7333</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>ZuLk@rN@iN BiN Z@iN@L</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>15:31</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat mobil grandmax</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3865-6020</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Elisabethkrova</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8825-7140</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>00:55</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Mlm cover ya berapa (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-9270-6460</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Putu Krisnanda</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>+62 881-5629-460</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>MFuady92</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-1097-6907</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Yusman Zein</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 6-10 of leads WA (1-3 Sept 2026, Meta Ads & Landing Page)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2074,6 +2074,3177 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-3313-3304</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Humaidi</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2200-0529</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Yohana Kolibu</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-4833-209</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>OEGENG</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3942-4446</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Momang D' Mori</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4312-2381</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Suratno</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>06:46</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5818-8259</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>wh9999812</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>05:43</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Beli / Tie mobil rush terbaru (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3059-6655</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Evelyn Sriwanti</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9450-866</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Ungki</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-2282-8162</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Iman Rajiman</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-5259-0999</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Jamal Raditya Shaqueena</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2917-972</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Just Do It</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-1677-1577</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>HANDJOJO</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-3976-6763</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>arisubawa</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-5720-4695</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Geepsoon</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-0020-6889</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Mas Danie</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>22:34</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8281-9193</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>SUGIYANTO</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4249-6930</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Jik Red</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? / Regulel untuk Mobil Xenia th 2014</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-0576-5023</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Mey Mey.</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9156-4766</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Bundahrio</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>01:08</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2239-0307</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Rudi</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1041-5077</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>MUHAMMAD RUSDI SELIAN, SE</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>02:39</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-5507-7701</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>De Bagas</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak (pesan terpotong di screenshot)</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2396-8989</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Des Fadli</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3808-4245</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Melvis Umbu Meha</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>04:35</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7961-7855</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>kang tralis &amp; kang plapon</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-4357-5882</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Sapto Firmansis</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-7701-9517</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Nurhaida</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9451-9914</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Sarip</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>08:05</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare hrga</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-2108-9070</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>05:23</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? (tanggal perlu dikonfirmasi, terpotong di screenshot)</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3128-1335</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>I~1</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2172-4827</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Dorce Kaitana</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>21:29</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8121-8261</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Rudy SC</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-7903-2979</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>zuLsalim</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>00:04</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (pesan sama dikirim ulang)</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7762-7117</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Im@</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-4363-1391</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>zainudinkoriah</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-599-191</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Budi G Pro</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this? Utk outdoor mbl LC VX200</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7523-3213</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Eug</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>00:07</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8869-8330</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Rismon Hanandua (Mon)</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-5974-555</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Fiki Astriyadi</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4145-1171</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>husenalii8679</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-0789-9123</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Nurul</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-0493-0894</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>harjonotri32</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>21:29</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-1466-877</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Arinanda</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>21:47</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-4107-32176</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>dailapasasandra</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-4191-4566</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Eko Maryanto</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>04:56</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-2438-6106</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>IRVAN</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5864-5541</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>sutimin benakat123</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4282-6836</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>putra kembar</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>04:21</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Cek harga utk mobil toyota rush 2024 (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5283-0613</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2438-3002</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>BUNG.KOTEKA</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1243-1856</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Merr</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>10:41</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-6158-11900</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Dewu</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6475-505</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>ilhamfamly89@gmail.com</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>01:47</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4596-6659</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Rusli Nangka</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-1017-4087</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>daimron89</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3971-8025</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>ALEXA</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>08:53</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>+62 881-0381-94355</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>dani</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>+62 888-2632-026</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Glemboh Nur</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-6026-5516</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>putusuwija81</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2187-8169</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Jro Nana</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-2277-0575</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>èdMön Lámáwàtò</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>00:09</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8402-6565</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Mr Dolphin</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>02:40</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5537-1166</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Zaenal</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5776-6635</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>N.HERY TETUKO</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7858-4925</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Agus Supriadi</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Tokonya dmna? (tidak pakai CTA template, tidak ada label iklan)</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Sumber tidak teridentifikasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-0033-52964</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>David Danials Batik</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>05:05</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0541-8883</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Tom Bali (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare / Untuk type Toyota Rush 2016, berpa?</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-0003-32802</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>FEY❤️</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-8014-7006</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>Tri Yuwono Oeding</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: toyota
+Tipe Mobil: sienta
+Tahun Mobil: 2016
+Nama Penerima: Tri Yuwono
+Alamat Penerima: Jl. Kebantenan 3, Rt.02/05 No.37 Semper Timur, Cilincing Jakarta Utara
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-6031-9669</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Batiar</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7382-6868</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Raulina</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2069-3878</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Prazentio Fathybetara</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4744-2975</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Nancy Lasabuda</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>05:56</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-8339-994</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>Nasi Gemuk Pakai Telor</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Halo untuk mobil chery tiggo 9 csh berapa ya? (video ad, tidak pakai CTA template standar)</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7677-9427</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>r sigit n</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-0828-1790</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>AHMAD WUJUD</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>07:42</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Ted (pesan tidak jelas/terpotong)</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6591-7171</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Purnomo</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare harga bos</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-8006-1616</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Oma</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5904-2254</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>nelly ilma</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4589-3096</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Ketut Witana</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-0677-2559</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Imam Bonjol</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-8802-4677</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Id Maryam</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4354-8187</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>RSL (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4148-5209</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Apriliano Grasia Boli Sug</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-2032-8111</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Ummu Rachsal</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4393-9500</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>jefrylahamendu084</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5579-0911</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>andika</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>10:41</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Harga brpa ? (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8079-4647</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Bambang Purwadi</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>(nomor tidak terlihat - kontak tersimpan 'adhy')</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>adhy</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5493-7313</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Nelson</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Meta Ads - Facebook</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Standardize Sumber/Keterangan taxonomy (Facebook/Instagram - Whatsapp, Landing Page V2)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3015,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram (Video)</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3582,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram (Video)</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Perlu dicek</t>
         </is>
       </c>
     </row>
@@ -4212,7 +4212,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Sumber tidak teridentifikasi</t>
+          <t>Perlu dicek</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Landing Page V2</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Perlu dicek</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Perlu dicek</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Perlu dicek</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook (Video)</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Instagram</t>
+          <t>Instagram - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads - Facebook</t>
+          <t>Facebook - Whatsapp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Label ambiguous-origin leads with standard CTA as plain Whatsapp source
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Perlu dicek</t>
+          <t>Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Perlu dicek</t>
+          <t>Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Perlu dicek</t>
+          <t>Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Perlu dicek</t>
+          <t>Whatsapp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Label generic-Iklan-card leads as Meta - Whatsapp
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -4926,7 +4926,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Whatsapp</t>
+          <t>Meta - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Whatsapp</t>
+          <t>Meta - Whatsapp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Relabel standard-CTA leads without visible ad card as Meta - Whatsapp
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Whatsapp</t>
+          <t>Meta - Whatsapp</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Whatsapp</t>
+          <t>Meta - Whatsapp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add batch 11 of leads WA (1-7 Sept 2026, Meta Ads & Landing Page V2)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5245,6 +5245,510 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1945-454</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>^~^</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9677-9321</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Rahmat</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil Calia hrg brp</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4737-5128</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Edy Resubun</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7379-7867</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Muliono Tohir</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5170-8471</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Asmar Siahaan</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-4106-9049</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Anton Wibowo</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-3117-961</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Septian Christianto</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2146-2520</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Wil</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>15:32</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3714-9078</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>isrofifirman85 (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8858-2442</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Hasbieaffan (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4054-3996</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Anif Makbul</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1811-4445</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Samila Ali</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>19:38</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4522-0818</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Loren</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9500-2441</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>_KUS MLP_</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>08:46</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 12-13 of leads WA (1-5 Sept 2026, Meta Ads incl. video ads)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5749,6 +5749,1056 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7068-2409</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Lainnya (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3021-2877</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2566-6014</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>samsiralang35</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4526-7517</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Karyono</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>05:25</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-1323-3691</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Sensei Cukman</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-3626-1670</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>M. Kurniyanto</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-7918-280</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Dilah</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Spill price untuk mobil avanza (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5568-3979</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5331-5182</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>antoksugianto2122</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>02:48</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1805-9704</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Sibgadinda</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4160-6778</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>Rahim Afen</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3854-9998</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>Mj_shukur</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>02:19</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4692-5511</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>Isran Malik S.Pd</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5418-7080</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Moh Hamim Tohari</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0539-3814</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Putu Srie</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-1446-435</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Agus Laskar</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>00:34</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5888-1787</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>Zero Computer (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>Ada Link Shopee/ Tokopedia (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-8257-6522</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>PortakTambunan</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>22:51</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3278-51546</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-7722-8082</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>Hj.Darmalailis Lbs.</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4794-4349</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>TOMIINDA</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4720-6798</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Fauzi</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7782-5320</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Dodol (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5601-4191</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>haji tonny</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-5653-7129</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>GUNK</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>19:13</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5990-3185</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>~ADR~</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4720-1123</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>Faizal Burhan</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>05:04</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-418-731</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Syahrir</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>05:19</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9659-6252</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Sartika Lubis</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8500-2627</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>B IBRAHIM</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 15-16 of leads WA (2, 4, 6-7 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G180"/>
+  <dimension ref="A1:G210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6799,6 +6799,1070 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-1435-8077</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>DL8</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9419-4514</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>ASM</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3666-0878</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Sura</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4212-3252</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>SulHam</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>17:06</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-7550-7507</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>Adhi Kharisma Putra</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-3300-5545</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Apong</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>19:31</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1002-4789</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>agnes</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8607-2059</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>chasyning (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-596-300</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Y Budi Sulistioadi</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare untuk Toyota Kijan Innova 2011</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5016-058</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>05:24</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2180-1149</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>D D</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat mobil pickup ss 2017 ada?</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-0941-0199</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>WA khusus Bantuan, GBU 😇</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7393-8555</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Rahmat Marzuki Nst</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3020-7036</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Rozaly</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5345-1330</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>dadiserigar</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6633-5665</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Andrian Kaifan</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3377-4523</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Wjy</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>06:56</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-1788-4380</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>B4CHT14R</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6005-0881</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>Bona</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7857-6558</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>henh99611</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1181-3137</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>Heri.S</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8944-2969</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Adi Prasetyo</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-9388-7359</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>NRS Footwear Designer</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>21:41</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2557-8812</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Deni Irawan 1112724</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>06:37</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-4345-0390</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Icha Store</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>21:42</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-7809-4538</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>SAMUEL SIMANJUNTAK</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>21:57</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Brpaan kak cover mobil nya ? (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>+62 898-3701-445</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>mama adni</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-7795-8775</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>Ryan R.</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-2190-6331</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>Neng Emput</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>22:46</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk Brio th 2015 diharga berapa ka dan Setok ready ngk</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6212-8988</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Pilosofi</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>23:12</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 17-18 of leads WA, dedup against prior batches (1-7 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G210"/>
+  <dimension ref="A1:G223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7863,6 +7863,482 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-2660-0987</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>G.O</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>23:51</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: BMW
+Tipe Mobil: 330i
+Tahun Mobil: 2021
+Nama Penerima: Geryn
+Alamat Penerima: PIK 2
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4881-6660</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Taufik Palenga</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>05:11</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau konsultasi Cover Mobil.
+Merk Mobil: Suzuki
+Tipe Mobil: X4 Over
+Tahun Mobil: 2012
+Nama Penerima: Taufik
+Alamat Penerima:
+Tipe Cover: Reguler berapa, Eksekutive brp....mhn info
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4071-6580</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Heru</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4600-9870</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>01:13</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3679-4004</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>kurawa084</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>07:39</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (pesan dikirim 2x, jam kedua 08:13)</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4047-3757</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Purru</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>00:32</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>Daerah mana, cek harga (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-2471-8184</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Budi idol</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>00:21</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3736-9489</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>John M Benggu</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-0018-9726</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Danik</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-8330-2434</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Yogie</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3077-0168</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>pausmarsel</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga kak</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0370-5185</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Made Suasta</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Info harga</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3820-0041</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Komang Sulatra</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare, harganya?</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 19 of leads WA (4, 6-7 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G223"/>
+  <dimension ref="A1:G234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8339,6 +8339,391 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4187-8834</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Rio Ucup Nainggolan</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>+1 (202) 705-3175</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Wira</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8037-0473</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>RMtef</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4289-8999</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Bapak Sumiran</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Xpander Cross (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7193-7596</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>ramonindra04</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>17:57</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1086-6737</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Enza Fachreza</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>17:19</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-6133-0834</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Suanda Dik$a</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>05:27</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1393-4858</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Yudha_MD</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5715-8060</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Reny Aprillia</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Apa harga nya 299rb</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-6218-3999</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>kitaponsel896</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5018-3314</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Abdu</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Untuk mobil kayla 2026 ada gak</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 20, 22-23 of leads WA (5-7 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8724,6 +8724,1091 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9733-3685</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>xaveclaus</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4611-4188</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Salman S</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Cek harga cover</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7067-3317</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Pak Reni Sihombing@15Pro</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek harga &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-3796-9390</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Malik Plaza Toyota Green Garden (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat Agya berapa</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2836-8733</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>Yakin kpd Allah SWT</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>04:25</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-8935-3763</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>defrihardian05</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4676-9235</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>ery indra</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk Daihatsu Xenia tahun 2007</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4584-8321</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>A. Ismail</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1650-7025</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>John Kheng</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9264-1032</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Yan's pelafon</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>18:19</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4708-5708</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Novi Hartanto</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7410-4476</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Syamsurizal</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-0681-1085</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Fahmi Yusuf</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4359-9631</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Moko/umming</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>+44 7761 928122</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Nanang</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>Selamat siang (tidak pakai CTA template, tanpa label iklan)</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-315-899</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Hey There</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>+62 897-5637-970</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>Murli Soemaryono</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>06:07</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8765-6454</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>saparuddindjuraidj837</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (pesan dikirim ulang jam 11:55)</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3933-6009</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>Jichoya 👪</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3141-1882</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Akara</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>22:54</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7351-5593</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>mmukti193@gmail.com</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>07:54</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-5330-0245</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>PS. J.B Piris. S.Th</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5851-9848</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>alexsandersalama48 (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8944-4908</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4013-7918</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>Ros</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2760-0765</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Dedy Damanhuri</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2916-5823</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>Agus</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3977-4961</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Ngh Asin</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-0688-0330</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>Syahar</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-161-828</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Ichsan Suharsono</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-1574-2599</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>Aris Riskandar (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 27-31 of leads WA (1, 3, 5-8 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9809,6 +9809,4017 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="2" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9933-2838</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Joshua</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>18:13</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3828-6667</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>Fijayku</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>+62 887-4374-49817</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Toko kelontongan (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8211-7276</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>Freddy Yohanes</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>20:29</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2510-9628</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>.SalokOoo</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-9686-8858</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-9562-9084</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Andi K</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3331-3740</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>Xxx (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-3493-6636</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Darat</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>22:49</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-5009-0072</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>Jalal Assegaf</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9016-9991</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>bang rian ganteng d w</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>06:03</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2637-7622</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>Edy Gondrong</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare .Cek Harga</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-4221-3661</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>🤝</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1925-6684</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Teguh Gunawan</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-2637-319</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Gemifar</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3610-4717</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>Dwi Septari</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8266-2282</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>deri</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>23:31</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: honda
+Tipe Mobil: CR-V gen 3
+Tahun Mobil: 2012
+Nama Penerima: Deri
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-2730-5850</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>Dyk (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>09:37</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8453-4450</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>Aldi.V</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-2882-3602</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>Agus Wijayanto Nugroho</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk Nissan Serena c24</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-1041-344</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>wahidhanft</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cari untuk mobil sigra</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-1975-3282</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>Defin las</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5572-2811</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Jimran</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-3962-6675</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>fendy</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare P</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5888-306</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>indkhan01</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada u/mobil Toyota Yaris</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9020-1186</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>Korah Deisy Ngau</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>04:26</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1606-639</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>hmd</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>07:16</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7365-6908</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>Ilham</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>06:58</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-4993-322</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>miiillaaaa</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3139-3501</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>Mahmoed Faza</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G295" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3701-3100</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>Paskalis</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk avanza tipe E tahun 2017</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-8058-7117</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>Ikhwan Nasution</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G297" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4459-9034</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>sunartirante617</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek hrg,bisa cod kah</t>
+        </is>
+      </c>
+      <c r="G298" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6979-9119</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>JOKO PURNOMO</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G299" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7573-7374</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>Mhd Fadli</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G300" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9991-1777</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>Said Umar</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-3399-2795</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>Unity Of Fashion (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3360-4049</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>Budi Santoso</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>14:49</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Sarung mobil Ertiga warna putih 2018</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-7917-0844</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>Aviz</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7007-5700</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>Polis Patola</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3288-3188</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>Hendy</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4168-6858</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>Taufik Nur</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>05:41</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-5555-0616</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Hn.Syahpoetra</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Toyota
+Tipe Mobil: all New rush TRD sportivo
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2860-5530</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>hermaniusaja</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>+62 898-1693-966</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Rezky Adelia</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>Halo kk (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3262-92369</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>Fiqram</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Tiktok ada?</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8822-1755</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>Benz</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7267-3333</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>🇵🇸 Mahdi Karunia 🇵🇸</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>05:59</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-6404-311</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>Subur Harsoyo</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brp harganya mobil Ertiga COVERNYA</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2888-6348</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>Calon.arang12</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>01:17</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1854-8383</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Suratin_TS_AB Jatibaru</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G316" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6358-7745</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>Ilham Rezki</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1823-3799</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>disuhardi185</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8164-3311</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>Suas</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>18:09</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2132-7805</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>yoyontaryana</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>Kl buat honda pred ada ga (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G320" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7507-192</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>Yusma SE</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>09:08</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek harga</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3484-88562</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>El Musytari</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G322" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-1399-9960</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>Nono G</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare maaf lokasi dr mana</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-4721-0849</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>Komang Andyana</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>20:29</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brp cover mobilnya pak (nomor sudah tidak aktif di WA)</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8725-6511</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>Chand</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G325" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4305-6435</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>U.Elly Batpoty</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3658-0084</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>MK</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>23:13</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1791-4152</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>Zainul</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-6457-0896</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>Datuk Riyo</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>07:39</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4682-6020</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>Sudirman Haris</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9211-3292</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>03:36</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Untuk honda oddessey brp kak</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-1908-017</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>Esta</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>04:44</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa harga promo utk warna...</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4002-3142</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>jamespandoy06</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>04:33</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1012-0779</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Tara</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>06:06</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4674-5447</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>Subardi Al Sobri</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>06:07</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Daihatsu
+Tipe Mobil: Terrios
+Tahun Mobil: 2019
+Nama Penerima: Subardi
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1886-1164</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>Tonce</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>06:29</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utk mbl Nissan Terano S1</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7816-6663</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>M Dhefin Al Fatih</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Selambu mbl kah ini? Untuk Fortuner berapa hrgnya?</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7116-0007</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>PAK UWO DEN..</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>10:41</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek harga bos . Untuk mobil Avanza ada bos... berapa harga ?</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9248-3467</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>sashuke kenjiro nagata</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>08:16</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utk inova reborn harga brp Ada foto / video</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-217-497</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Iman Fathurrohman</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G340" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4742-7995</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>AGUESS deluga babah</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1590-0100</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>Ava Eleana (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>08:53</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harganya brapa</t>
+        </is>
+      </c>
+      <c r="G342" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9603-6199</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>YSM</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G343" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-9026-5434</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>Irwan</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G344" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-2245-0980</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>Raffasya</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>09:29</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>Cek harga buat zigra (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-3355-2506</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>Gop_il</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G346" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7166-0453</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>Jerry kontu</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G347" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-5049-4005</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>La Rusia, S.Sos</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G348" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1692-0347</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>puterabalam</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr">
+        <is>
+          <t>Brp hrga untuk Toyota new rush (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G349" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4510-7704</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>drsngatiran</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G350" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-8686-683</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>Arief Wibowo</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G351" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-5800-7930</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>Firman Chou</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat vw golf mk 6 brpa kk?</t>
+        </is>
+      </c>
+      <c r="G352" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4139-3254</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>imank</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G353" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-4175-2776</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>lalu zul akhyar</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G354" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3725-3138</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>Herman🐊</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G355" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2504-0009</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>Kim Byeong Ho</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G356" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1678-6963</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>sigiwibisono73@gmail.com</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G357" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8988-0125</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>Abi Azzam</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G358" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-4714-7941</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>sakunabfredianus</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G359" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5736-6855</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>Aurel INK Production</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G360" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8722-8318</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>English teacher</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>02:05</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G361" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-2426-6106</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>slow (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Toyota
+Tipe Mobil: Vios Gen 3
+Tahun Mobil: 2015
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G362" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3451-6768</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>Dicky</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3954-5646</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>Mega Purnama</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1856-2775</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>rifqi ainur</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: chevrolet
+Tipe Mobil: trax
+Tahun Mobil: 2018
+Nama Penerima: rifqi
+Alamat Penerima: jakarta timur
+Tipe Cover: (Reguler)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7285-4422</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>Igustibagus</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga dulu berapa.. Mm</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-5874-4171</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>Dwi Agung Wibowo</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>13:09</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Toyota
+Tipe Mobil: Yaris
+Tahun Mobil: 2011
+Nama Penerima: Agung
+Alamat Penerima: Terban GK 5/32C RT.01 RW.01 Yogyakarta 55223
+Tipe Cover: Premium (3 ly)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-1904-0983</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>Andri Pratama</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk mobil xenia R sporty 2017 Harga berpa ya ka</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3823-0788</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>Pelita (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil nav 1 THN 2013 Harga</t>
+        </is>
+      </c>
+      <c r="G369" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-4104-4490</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>Mr Zippo</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G370" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1002-2500</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G371" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9398-6624</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>Bahtiar Lau</t>
+        </is>
+      </c>
+      <c r="E372" s="2" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G372" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2385-0857</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>Dani Modeong</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9290-7383</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>pakfuadndalem</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: expander
+Tipe Mobil:suv
+Tahun Mobil:2023
+Nama Penerima:fuad
+Alamat Penerima:semarang
+Tipe Cover: (Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4297-7727</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>abdulbahar1966</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare harga</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9687-9196</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>Nikma Nasir</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-220-403</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>Felipe F</t>
+        </is>
+      </c>
+      <c r="E377" s="2" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G377" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5038-8889</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>Charles Rauwiyanto</t>
+        </is>
+      </c>
+      <c r="E378" s="2" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G378" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 33-35 of leads WA (1, 6-9 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G378"/>
+  <dimension ref="A1:G430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13820,6 +13820,1847 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" s="2" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8778-3719</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>herpinasimanjuntak</t>
+        </is>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t>05:56</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G379" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5599-9981</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>⻌ⱍ⻌⨚⻌</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G380" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4232-2358</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>homy interior (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t>07:23</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada berapa type ya di undercover</t>
+        </is>
+      </c>
+      <c r="G381" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-0117-8808</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>Sandi</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau bli di tempat boleh? (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G382" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7028-5378</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>yopitanuarta78</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga berapa ?</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2077-5345</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>Humaidi Abu Uwais</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G384" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4227-6164</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>Eka Pratiwi</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1772-5188</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>Eko Pije Budi Santosa</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>05:20</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9998-4172</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>Erwin Kesuma Dg Mallongi</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapaan untuk brio</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3344-2345</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>M. Syaiful Qomari Als Ali</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>02:33</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4727-6101</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>IGusti Ngurah Japa</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>09:01</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare untuk mobil Toyota Raize....apakah ada petunjuk pemakaiannya, ada larangan? Dan apakah bisa outdor?</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9997-7721</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>Ones Sopanyo</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Mobil parkir di luar</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5334-2881</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>Marimin</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4049-6983</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>Dwi Budiarti</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9990-2906</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>DR. LA ISMEID, S.Pd, M.Pd</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8452-4167</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>samuellamber948</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek harga untuk oto Avanza 2015 kk.</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1272-6341</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>xxxxx (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G395" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="B396" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-9927-2271</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>RAHMAT rahmat</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G396" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="n">
+        <v>396</v>
+      </c>
+      <c r="B397" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-1115-2980</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>Supri</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: New Ertiga
+Tipe Mobil: GL
+Tahun Mobil: 2018
+Nama Penerima: Supriyanto
+Alamat Penerima: jl. Kakap Kp. Pencikan Barat 209 Kelurahan Dadapsari. Semarang Utara. SEMARANG
+Tipe Cover: (Reguler)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G397" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-5611-029</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>Ronald</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utk suzuki All new swift th. 2013 brp harganya</t>
+        </is>
+      </c>
+      <c r="G398" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="n">
+        <v>398</v>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-252-566</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="B400" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-6143-0966</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>Heru</t>
+        </is>
+      </c>
+      <c r="E400" s="2" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G400" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B401" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-6739-5604</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>Safna</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="inlineStr">
+        <is>
+          <t>Hallo kak / Ada cover civic lx gaa yaa (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G401" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="n">
+        <v>401</v>
+      </c>
+      <c r="B402" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8693-4532</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>Abduronta</t>
+        </is>
+      </c>
+      <c r="E402" s="2" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G402" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="n">
+        <v>402</v>
+      </c>
+      <c r="B403" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-427-448</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>Sepril</t>
+        </is>
+      </c>
+      <c r="E403" s="2" t="inlineStr">
+        <is>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G403" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="n">
+        <v>403</v>
+      </c>
+      <c r="B404" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C404" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5096-4632</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>idul</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G404" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="n">
+        <v>404</v>
+      </c>
+      <c r="B405" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-9272-5748</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>Henri</t>
+        </is>
+      </c>
+      <c r="E405" s="2" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada link shoppynya kak</t>
+        </is>
+      </c>
+      <c r="G405" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="n">
+        <v>405</v>
+      </c>
+      <c r="B406" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3378-5202</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>Duwi</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G406" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="n">
+        <v>406</v>
+      </c>
+      <c r="B407" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C407" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-5905-0617</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>Jro Mk Istri Tripitasih</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G407" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="n">
+        <v>407</v>
+      </c>
+      <c r="B408" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C408" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-6757-6364</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>Ahmad Riadi</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Apakah water proof</t>
+        </is>
+      </c>
+      <c r="G408" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="n">
+        <v>408</v>
+      </c>
+      <c r="B409" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4768-0557</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>imron</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr">
+        <is>
+          <t>Kl ke kaltim broa gan (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G409" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="n">
+        <v>409</v>
+      </c>
+      <c r="B410" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1713-1166</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>Hadikusuma</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cover mobil BRV brp</t>
+        </is>
+      </c>
+      <c r="G410" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="n">
+        <v>410</v>
+      </c>
+      <c r="B411" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C411" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7352-1037</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>☽</t>
+        </is>
+      </c>
+      <c r="E411" s="2" t="inlineStr">
+        <is>
+          <t>07:38</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G411" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="n">
+        <v>411</v>
+      </c>
+      <c r="B412" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8005-8568</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>Hry</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G412" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="n">
+        <v>412</v>
+      </c>
+      <c r="B413" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6673-4554</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>m.sanusi</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>06:54</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G413" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="B414" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8885-8343</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>Monica</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G414" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="n">
+        <v>414</v>
+      </c>
+      <c r="B415" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-3596-619</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>wibisonosonic (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>01:53</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G415" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="n">
+        <v>415</v>
+      </c>
+      <c r="B416" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-1454-617</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>BUNDA AEO</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ini harganya 300 ya?</t>
+        </is>
+      </c>
+      <c r="G416" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="n">
+        <v>416</v>
+      </c>
+      <c r="B417" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3028-7220</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>Ainul Yaqin</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G417" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="n">
+        <v>417</v>
+      </c>
+      <c r="B418" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-5854-5336</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>rahmat Kartolo</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>23:51</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:  Mobilio
+Tipe Mobil: E
+Tahun Mobil: 2014
+Nama Penerima: Rahmat
+Alamat Penerima : Perum putra kelana jaya blok C5 no 3 bengkong sadai batam
+Tipe Cover: (Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G418" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="n">
+        <v>418</v>
+      </c>
+      <c r="B419" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-0773-7995</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>Fredy Dwi Saputra</t>
+        </is>
+      </c>
+      <c r="E419" s="2" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="inlineStr">
+        <is>
+          <t>Cek sarung mobil avansa taun 2009 (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G419" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="B420" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-7601-3371</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>Amran</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak! ada shopee kak q?</t>
+        </is>
+      </c>
+      <c r="G420" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="B421" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6171-3875</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>Ongky Sanjaya</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G421" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="n">
+        <v>421</v>
+      </c>
+      <c r="B422" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-2944-1565</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>Madi</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G422" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="n">
+        <v>422</v>
+      </c>
+      <c r="B423" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1407-6465</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>EvanParulian</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk tipe honda wrv rs berapa harganya</t>
+        </is>
+      </c>
+      <c r="G423" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="n">
+        <v>423</v>
+      </c>
+      <c r="B424" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-1858-185</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>TRIOJEGAJE</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>16:18</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G424" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="n">
+        <v>424</v>
+      </c>
+      <c r="B425" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-2137-0385</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>CharunTelkomsel</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G425" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="B426" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3220-2860</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>tonny widhiono</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G426" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="B427" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3959-3556</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>nurmasugiarto</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Lokasi</t>
+        </is>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="n">
+        <v>427</v>
+      </c>
+      <c r="B428" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1074-8481</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>Muh.sahidin</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>09:48</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G428" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="n">
+        <v>428</v>
+      </c>
+      <c r="B429" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-5847-5252</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>camelia</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G429" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="n">
+        <v>429</v>
+      </c>
+      <c r="B430" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-4703-8578</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>Gondhez Sutedjo</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G430" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 36-37 of leads WA (5, 8-10 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G430"/>
+  <dimension ref="A1:G447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -15661,6 +15661,601 @@
         </is>
       </c>
     </row>
+    <row r="431">
+      <c r="A431" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="B431" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-5707-1622</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>Ajez</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>05:51</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G431" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="n">
+        <v>431</v>
+      </c>
+      <c r="B432" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5961-9170</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>MR</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Apakah buat premio hiace / Cover untuk hiace premio ready kah</t>
+        </is>
+      </c>
+      <c r="G432" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="B433" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9282-5442</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>Momong Vano</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak / Cover BYD atto 1 ready gak (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G433" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="n">
+        <v>433</v>
+      </c>
+      <c r="B434" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1089-4852</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>Didi</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G434" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="n">
+        <v>434</v>
+      </c>
+      <c r="B435" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4315-8842</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>Usman</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>04:33</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G435" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="n">
+        <v>435</v>
+      </c>
+      <c r="B436" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-2440-2595</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>bobby prakoso</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat Terios 2016 ada tdk ya?</t>
+        </is>
+      </c>
+      <c r="G436" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="n">
+        <v>436</v>
+      </c>
+      <c r="B437" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2180-6412</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>eyang Abas /Anita rias</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>03:39</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada buat mbl taruna thn2003</t>
+        </is>
+      </c>
+      <c r="G437" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="n">
+        <v>437</v>
+      </c>
+      <c r="B438" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5469-7759</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>KettyMumu</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G438" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="n">
+        <v>438</v>
+      </c>
+      <c r="B439" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8376-6650</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>02:46</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G439" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="n">
+        <v>439</v>
+      </c>
+      <c r="B440" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C440" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-6051-0046</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>أصمعي هدايت البنتني</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G440" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="B441" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3471-19486</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>Bunda Lela</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>20:13</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G441" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="n">
+        <v>441</v>
+      </c>
+      <c r="B442" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6803-9539</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>Andi Kiswanto</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G442" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="n">
+        <v>442</v>
+      </c>
+      <c r="B443" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C443" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1511-5078</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>mufaizahizah31</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>22:02</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="n">
+        <v>443</v>
+      </c>
+      <c r="B444" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6631-0063</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>00:57</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="n">
+        <v>444</v>
+      </c>
+      <c r="B445" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9217-0456</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>Yakob Sanjati</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G445" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="n">
+        <v>445</v>
+      </c>
+      <c r="B446" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2523-6653</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>Iskandar</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G446" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="n">
+        <v>446</v>
+      </c>
+      <c r="B447" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7452-9202</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>aidilputraindra</t>
+        </is>
+      </c>
+      <c r="E447" s="2" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G447" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 40-42 of leads WA (3, 7-11 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G447"/>
+  <dimension ref="A1:G520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -16256,6 +16256,2596 @@
         </is>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="B448" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C448" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5015-1073</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>ridaassaragih</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Hrg brp</t>
+        </is>
+      </c>
+      <c r="G448" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="n">
+        <v>448</v>
+      </c>
+      <c r="B449" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7821-1080</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="E449" s="2" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil Toyota calya</t>
+        </is>
+      </c>
+      <c r="G449" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="n">
+        <v>449</v>
+      </c>
+      <c r="B450" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C450" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9810-5522</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>Fadly</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek</t>
+        </is>
+      </c>
+      <c r="G450" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="B451" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1140-734</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>Anto</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="n">
+        <v>451</v>
+      </c>
+      <c r="B452" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6201-3294</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>Riki Riwanto</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G452" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="n">
+        <v>452</v>
+      </c>
+      <c r="B453" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-5268-6051</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>Ramli</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="n">
+        <v>453</v>
+      </c>
+      <c r="B454" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-1364-5779</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>andreyanto28</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat Avanza 2025</t>
+        </is>
+      </c>
+      <c r="G454" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="n">
+        <v>454</v>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-7126-8353</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>Reza Ismail Abdul Rahman</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G455" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="n">
+        <v>455</v>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-3055-5333</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr">
+        <is>
+          <t>misi / bisa liat contoh cover mobil-nya (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G456" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="n">
+        <v>456</v>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1987-8999</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>Hendra</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Honda civic turbo. 2018</t>
+        </is>
+      </c>
+      <c r="G457" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="n">
+        <v>457</v>
+      </c>
+      <c r="B458" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-8524-3488</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>Gunadi Jasum (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G458" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="n">
+        <v>458</v>
+      </c>
+      <c r="B459" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5009-7122</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>Delce Baware</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>15:17</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G459" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="n">
+        <v>459</v>
+      </c>
+      <c r="B460" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-1042-3496</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>Pak Roni</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G460" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="n">
+        <v>460</v>
+      </c>
+      <c r="B461" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4360-8980</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>Ucu</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>12:16</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>Cek hrga (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G461" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="n">
+        <v>461</v>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7153-9699</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>CANDRA.R</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Yg indoor brp hrgnya</t>
+        </is>
+      </c>
+      <c r="G462" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="n">
+        <v>462</v>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3739-4642</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>Lionelgian84</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="n">
+        <v>463</v>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-0595-9483</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>hbh</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: nissan
+Tipe Mobil: serena c24
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:sepatan kab tangerang
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G464" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="n">
+        <v>464</v>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3309-8109</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>Rembrand</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="n">
+        <v>465</v>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-3351-46871</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>Noldi Seran</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>05:58</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="n">
+        <v>466</v>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1569-9416</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>Supriadi Pae Kembar</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>Cek harga untuk cover nya kak (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="n">
+        <v>467</v>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4616-5385</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G468" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7078-9393</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>Inayah</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>19:34</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="n">
+        <v>469</v>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4103-8463</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>Hery Suyatno</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>18:57</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek hrg</t>
+        </is>
+      </c>
+      <c r="G470" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="B471" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4777-9482</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>Batara Hutabarat_17</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G471" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="n">
+        <v>471</v>
+      </c>
+      <c r="B472" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4182-4962</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>Wahida Ibrahim</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek aja dl</t>
+        </is>
+      </c>
+      <c r="G472" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="n">
+        <v>472</v>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-2676-456</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>Intus</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>05:10</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Yg ekonomis dalam nya halus versi...</t>
+        </is>
+      </c>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="n">
+        <v>473</v>
+      </c>
+      <c r="B474" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0601-2973</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>Yan (Zenko) (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G474" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="n">
+        <v>474</v>
+      </c>
+      <c r="B475" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C475" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9790-8758</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>51_70ko_pr@n</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G475" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="n">
+        <v>475</v>
+      </c>
+      <c r="B476" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-7922-6280</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>hanif</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G476" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="n">
+        <v>476</v>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1686-5348</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>CABUKO</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="n">
+        <v>477</v>
+      </c>
+      <c r="B478" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4510-1383</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>giantorokris904</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>19:03</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G478" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="n">
+        <v>478</v>
+      </c>
+      <c r="B479" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C479" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2142-2563</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>Teh Ani</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G479" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="n">
+        <v>479</v>
+      </c>
+      <c r="B480" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1975-7171</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>HM.Agus Mulyana</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>19:34</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G480" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="B481" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C481" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4692-9599</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>kakek kubu Alit</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk mobil Terios cek harga</t>
+        </is>
+      </c>
+      <c r="G481" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="B482" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9235-8848</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>BRAVO</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G482" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="n">
+        <v>482</v>
+      </c>
+      <c r="B483" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7721-1925</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>Sefri Nahak</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G483" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="n">
+        <v>483</v>
+      </c>
+      <c r="B484" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4111-3331</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>Matt Lamato</t>
+        </is>
+      </c>
+      <c r="E484" s="2" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G484" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="n">
+        <v>484</v>
+      </c>
+      <c r="B485" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-7505-3469</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>thoriq</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G485" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="n">
+        <v>485</v>
+      </c>
+      <c r="B486" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4084-2438</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>meketisonrumbrapukmeki</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G486" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="n">
+        <v>486</v>
+      </c>
+      <c r="B487" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5917-1788</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>Sampir</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="n">
+        <v>487</v>
+      </c>
+      <c r="B488" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-1558-5491</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>Samsul Arifin</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G488" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="n">
+        <v>488</v>
+      </c>
+      <c r="B489" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-9613-8451</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>ewiill</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="n">
+        <v>489</v>
+      </c>
+      <c r="B490" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3935-4400</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>MOEH SYUKUR</t>
+        </is>
+      </c>
+      <c r="E490" s="2" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="F490" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G490" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="n">
+        <v>490</v>
+      </c>
+      <c r="B491" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-332-921</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>🐝</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G491" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="n">
+        <v>491</v>
+      </c>
+      <c r="B492" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8469-0144</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>Fariz Mahesa</t>
+        </is>
+      </c>
+      <c r="E492" s="2" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="F492" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G492" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="n">
+        <v>492</v>
+      </c>
+      <c r="B493" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1094-8048</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>Andry H.</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G493" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="B494" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9256-4724</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>jenggot Rsi</t>
+        </is>
+      </c>
+      <c r="E494" s="2" t="inlineStr">
+        <is>
+          <t>08:39</t>
+        </is>
+      </c>
+      <c r="F494" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa pak harganya</t>
+        </is>
+      </c>
+      <c r="G494" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="n">
+        <v>494</v>
+      </c>
+      <c r="B495" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-7514-9775</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>ok emoji</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G495" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="n">
+        <v>495</v>
+      </c>
+      <c r="B496" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1626-1565</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>Ranto Ketaren (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>12:11</t>
+        </is>
+      </c>
+      <c r="F496" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G496" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="n">
+        <v>496</v>
+      </c>
+      <c r="B497" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C497" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-2678-6754</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>colepalmer (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>07:53</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Destinator
+Tipe Mobil:
+Tahun Mobil: 2026
+Nama Penerima: Andi
+Alamat Penerima: Bogor
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G497" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="n">
+        <v>497</v>
+      </c>
+      <c r="B498" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8863-8518</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>Jasmin Parenrengi</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G498" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="n">
+        <v>498</v>
+      </c>
+      <c r="B499" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-1419-2868</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>Suwartini</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="inlineStr">
+        <is>
+          <t>Ada buat mobil sienta kah (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G499" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="n">
+        <v>499</v>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5314-2299</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>Gitut Castrow</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: toyota
+Tipe Mobil: innova lama
+Tahun Mobil:2009
+Nama Penerima: gitut
+Alamat Penerima: alamanda regency E19/15 tambun utara
+Tipe Cover: (Reguler/Exclusive) kalo bisa yg premium.
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G500" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="B501" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7561-9045</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>Agunan Butar-Butar</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>22:14</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil Toyota Innova Grand</t>
+        </is>
+      </c>
+      <c r="G501" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="n">
+        <v>501</v>
+      </c>
+      <c r="B502" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-1352-4387</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>TerCinta (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="F502" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Masih ada ya....?</t>
+        </is>
+      </c>
+      <c r="G502" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="n">
+        <v>502</v>
+      </c>
+      <c r="B503" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C503" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7455-0009</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>aldinoerda77</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>17:28</t>
+        </is>
+      </c>
+      <c r="F503" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G503" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="n">
+        <v>503</v>
+      </c>
+      <c r="B504" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4174-2286</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>Tatan</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="F504" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada mobil panter</t>
+        </is>
+      </c>
+      <c r="G504" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="B505" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C505" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9301-0001</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>Silas Ong</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
+      <c r="F505" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G505" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="n">
+        <v>505</v>
+      </c>
+      <c r="B506" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-5917-9388</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="F506" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G506" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="n">
+        <v>506</v>
+      </c>
+      <c r="B507" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-7244-8099</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>Yukensi</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="F507" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G507" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="n">
+        <v>507</v>
+      </c>
+      <c r="B508" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7754-5256</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>Abu kashafa (Dika)</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="F508" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G508" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="n">
+        <v>508</v>
+      </c>
+      <c r="B509" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9989-7563</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>Hampri</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="F509" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G509" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="n">
+        <v>509</v>
+      </c>
+      <c r="B510" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4422-3514</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>yermiamia01</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="F510" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G510" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="B511" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C511" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-4275-1911</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>Guritafw</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>18:28</t>
+        </is>
+      </c>
+      <c r="F511" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G511" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="n">
+        <v>511</v>
+      </c>
+      <c r="B512" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-7755-4888</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>M Jubaidi Yusuf</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="F512" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G512" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="n">
+        <v>512</v>
+      </c>
+      <c r="B513" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6020-7835</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>wulapaulus11</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="F513" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G513" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="n">
+        <v>513</v>
+      </c>
+      <c r="B514" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-4643-0874</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>Ibrahim Abdullah</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="F514" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G514" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="n">
+        <v>514</v>
+      </c>
+      <c r="B515" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-5120-8899</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>Samuel Christopher</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="F515" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G515" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="n">
+        <v>515</v>
+      </c>
+      <c r="B516" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9981-0085</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>Deck Dept</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G516" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="n">
+        <v>516</v>
+      </c>
+      <c r="B517" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7336-3107</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>Azna</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="F517" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G517" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="n">
+        <v>517</v>
+      </c>
+      <c r="B518" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9284-6260</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>Firmansyah</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="F518" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: wuling
+Tipe Mobil: almaz
+Tahun Mobil: 2019
+Nama Penerima: firman
+Alamat Penerima: cakung
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G518" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="n">
+        <v>518</v>
+      </c>
+      <c r="B519" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4057-5431</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>arsan</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="F519" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G519" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="n">
+        <v>519</v>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6503-5145</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G520" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Status column for flagging repeat-return customers
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G520"/>
+  <dimension ref="A1:H520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,6 +476,11 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sumber/Keterangan</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add batch 43 of leads WA (9, 12 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H520"/>
+  <dimension ref="A1:H535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -567,6 +568,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -602,6 +604,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -637,6 +640,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -672,6 +676,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -707,6 +712,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -742,6 +748,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -777,6 +784,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -812,6 +820,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -847,6 +856,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -882,6 +892,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -917,6 +928,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -952,6 +964,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -987,6 +1000,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1022,6 +1036,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1057,6 +1072,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1092,6 +1108,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1127,6 +1144,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1162,6 +1180,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1197,6 +1216,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1232,6 +1252,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1267,6 +1288,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1302,6 +1324,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1337,6 +1360,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1379,6 +1403,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1414,6 +1439,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1449,6 +1475,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1484,6 +1511,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1519,6 +1547,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1554,6 +1583,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1589,6 +1619,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1624,6 +1655,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1659,6 +1691,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1694,6 +1727,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1729,6 +1763,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1764,6 +1799,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1799,6 +1835,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1834,6 +1871,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1869,6 +1907,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1904,6 +1943,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1939,6 +1979,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1974,6 +2015,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2009,6 +2051,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2044,6 +2087,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2079,6 +2123,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2114,6 +2159,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2149,6 +2195,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2184,6 +2231,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2219,6 +2267,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2254,6 +2303,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2289,6 +2339,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2324,6 +2375,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2359,6 +2411,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2394,6 +2447,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2429,6 +2483,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2464,6 +2519,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2499,6 +2555,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2534,6 +2591,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2569,6 +2627,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2604,6 +2663,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2639,6 +2699,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -2674,6 +2735,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2709,6 +2771,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2744,6 +2807,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -2779,6 +2843,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2814,6 +2879,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2849,6 +2915,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -2884,6 +2951,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -2919,6 +2987,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -2954,6 +3023,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -2989,6 +3059,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3024,6 +3095,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3059,6 +3131,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3094,6 +3167,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3129,6 +3203,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3164,6 +3239,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3199,6 +3275,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3234,6 +3311,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3276,6 +3354,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -3311,6 +3390,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -3346,6 +3426,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -3381,6 +3462,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -3416,6 +3498,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -3451,6 +3534,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -3486,6 +3570,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -3521,6 +3606,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -3556,6 +3642,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -3591,6 +3678,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -3626,6 +3714,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -3661,6 +3750,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -3696,6 +3786,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -3731,6 +3822,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3766,6 +3858,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -3801,6 +3894,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -3836,6 +3930,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -3871,6 +3966,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -3906,6 +4002,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -3941,6 +4038,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -3976,6 +4074,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -4011,6 +4110,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -4046,6 +4146,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -4081,6 +4182,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -4116,6 +4218,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -4151,6 +4254,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -4186,6 +4290,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -4221,6 +4326,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -4256,6 +4362,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -4291,6 +4398,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -4326,6 +4434,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -4361,6 +4470,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -4403,6 +4513,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -4438,6 +4549,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -4473,6 +4585,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -4515,6 +4628,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -4550,6 +4664,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -4585,6 +4700,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -4620,6 +4736,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -4655,6 +4772,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -4690,6 +4808,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -4725,6 +4844,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -4760,6 +4880,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -4795,6 +4916,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -4830,6 +4952,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -4865,6 +4988,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -4900,6 +5024,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -4935,6 +5060,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -4970,6 +5096,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -5005,6 +5132,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -5040,6 +5168,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
@@ -5075,6 +5204,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -5110,6 +5240,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
@@ -5145,6 +5276,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
@@ -5180,6 +5312,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
@@ -5215,6 +5348,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -5250,6 +5384,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
@@ -5285,6 +5420,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
@@ -5320,6 +5456,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
@@ -5355,6 +5492,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
@@ -5390,6 +5528,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
@@ -5432,6 +5571,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
@@ -5467,6 +5607,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -5502,6 +5643,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -5537,6 +5679,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -5572,6 +5715,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -5607,6 +5751,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
@@ -5649,6 +5794,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -5684,6 +5830,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
@@ -5719,6 +5866,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -5754,6 +5902,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -5789,6 +5938,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -5824,6 +5974,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n">
@@ -5859,6 +6010,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -5894,6 +6046,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
@@ -5929,6 +6082,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -5964,6 +6118,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -5999,6 +6154,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
@@ -6034,6 +6190,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
@@ -6069,6 +6226,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -6104,6 +6262,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
@@ -6139,6 +6298,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
@@ -6174,6 +6334,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n">
@@ -6209,6 +6370,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
@@ -6244,6 +6406,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
@@ -6279,6 +6442,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
@@ -6314,6 +6478,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
@@ -6349,6 +6514,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
@@ -6384,6 +6550,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
@@ -6419,6 +6586,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
@@ -6454,6 +6622,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
@@ -6489,6 +6658,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
@@ -6524,6 +6694,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
@@ -6559,6 +6730,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -6594,6 +6766,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
@@ -6629,6 +6802,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -6664,6 +6838,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
@@ -6699,6 +6874,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
@@ -6734,6 +6910,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
@@ -6769,6 +6946,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
@@ -6804,6 +6982,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
@@ -6839,6 +7018,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -6874,6 +7054,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
@@ -6909,6 +7090,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -6951,6 +7133,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n">
@@ -6986,6 +7169,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -7021,6 +7205,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
@@ -7063,6 +7248,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
@@ -7098,6 +7284,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
@@ -7133,6 +7320,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
@@ -7168,6 +7356,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
@@ -7203,6 +7392,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
@@ -7238,6 +7428,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
@@ -7273,6 +7464,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -7308,6 +7500,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
@@ -7343,6 +7536,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
@@ -7378,6 +7572,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -7413,6 +7608,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -7448,6 +7644,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
@@ -7483,6 +7680,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
@@ -7518,6 +7716,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
@@ -7553,6 +7752,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
@@ -7588,6 +7788,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
@@ -7623,6 +7824,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
@@ -7658,6 +7860,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
@@ -7693,6 +7896,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
@@ -7728,6 +7932,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
@@ -7763,6 +7968,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
@@ -7798,6 +8004,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
@@ -7833,6 +8040,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
@@ -7868,6 +8076,7 @@
           <t>Meta - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
@@ -7910,6 +8119,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n">
@@ -7952,6 +8162,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
@@ -7987,6 +8198,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
@@ -8029,6 +8241,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n">
@@ -8064,6 +8277,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
@@ -8099,6 +8313,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
@@ -8134,6 +8349,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n">
@@ -8169,6 +8385,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n">
@@ -8204,6 +8421,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
@@ -8239,6 +8457,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
@@ -8274,6 +8493,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
@@ -8309,6 +8529,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
@@ -8344,6 +8565,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
@@ -8379,6 +8601,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
@@ -8414,6 +8637,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
@@ -8449,6 +8673,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
@@ -8484,6 +8709,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
@@ -8519,6 +8745,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
@@ -8554,6 +8781,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
@@ -8589,6 +8817,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
@@ -8624,6 +8853,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
@@ -8659,6 +8889,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
@@ -8694,6 +8925,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
@@ -8729,6 +8961,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
@@ -8764,6 +8997,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
@@ -8799,6 +9033,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
@@ -8834,6 +9069,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n">
@@ -8869,6 +9105,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n">
@@ -8904,6 +9141,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n">
@@ -8939,6 +9177,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n">
@@ -8974,6 +9213,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n">
@@ -9009,6 +9249,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n">
@@ -9044,6 +9285,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n">
@@ -9079,6 +9321,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n">
@@ -9114,6 +9357,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n">
@@ -9149,6 +9393,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n">
@@ -9184,6 +9429,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n">
@@ -9219,6 +9465,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n">
@@ -9254,6 +9501,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n">
@@ -9289,6 +9537,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n">
@@ -9324,6 +9573,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n">
@@ -9359,6 +9609,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n">
@@ -9394,6 +9645,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n">
@@ -9429,6 +9681,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n">
@@ -9464,6 +9717,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n">
@@ -9499,6 +9753,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n">
@@ -9534,6 +9789,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n">
@@ -9569,6 +9825,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n">
@@ -9604,6 +9861,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n">
@@ -9639,6 +9897,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n">
@@ -9674,6 +9933,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H261" s="2" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n">
@@ -9709,6 +9969,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H262" s="2" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n">
@@ -9744,6 +10005,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H263" s="2" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n">
@@ -9779,6 +10041,7 @@
           <t>Meta - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H264" s="2" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n">
@@ -9814,6 +10077,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H265" s="2" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n">
@@ -9849,6 +10113,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H266" s="2" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n">
@@ -9884,6 +10149,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H267" s="2" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n">
@@ -9919,6 +10185,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H268" s="2" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n">
@@ -9954,6 +10221,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H269" s="2" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n">
@@ -9989,6 +10257,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H270" s="2" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n">
@@ -10024,6 +10293,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n">
@@ -10059,6 +10329,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H272" s="2" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n">
@@ -10094,6 +10365,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H273" s="2" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n">
@@ -10129,6 +10401,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H274" s="2" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n">
@@ -10164,6 +10437,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H275" s="2" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n">
@@ -10199,6 +10473,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H276" s="2" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n">
@@ -10234,6 +10509,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H277" s="2" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n">
@@ -10269,6 +10545,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H278" s="2" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n">
@@ -10304,6 +10581,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H279" s="2" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n">
@@ -10339,6 +10617,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H280" s="2" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n">
@@ -10374,6 +10653,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H281" s="2" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n">
@@ -10416,6 +10696,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H282" s="2" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n">
@@ -10451,6 +10732,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H283" s="2" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n">
@@ -10486,6 +10768,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H284" s="2" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n">
@@ -10521,6 +10804,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H285" s="2" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n">
@@ -10556,6 +10840,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H286" s="2" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n">
@@ -10591,6 +10876,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H287" s="2" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n">
@@ -10626,6 +10912,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H288" s="2" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n">
@@ -10661,6 +10948,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H289" s="2" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n">
@@ -10696,6 +10984,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H290" s="2" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n">
@@ -10731,6 +11020,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H291" s="2" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n">
@@ -10773,6 +11063,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H292" s="2" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n">
@@ -10808,6 +11099,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H293" s="2" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n">
@@ -10843,6 +11135,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H294" s="2" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n">
@@ -10878,6 +11171,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H295" s="2" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n">
@@ -10913,6 +11207,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H296" s="2" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n">
@@ -10948,6 +11243,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H297" s="2" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n">
@@ -10983,6 +11279,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H298" s="2" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n">
@@ -11018,6 +11315,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n">
@@ -11053,6 +11351,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H300" s="2" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n">
@@ -11088,6 +11387,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H301" s="2" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="n">
@@ -11123,6 +11423,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H302" s="2" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="n">
@@ -11158,6 +11459,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H303" s="2" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="n">
@@ -11193,6 +11495,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H304" s="2" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="n">
@@ -11228,6 +11531,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H305" s="2" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="n">
@@ -11263,6 +11567,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H306" s="2" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="n">
@@ -11298,6 +11603,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H307" s="2" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="n">
@@ -11340,6 +11646,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H308" s="2" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="n">
@@ -11375,6 +11682,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H309" s="2" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="n">
@@ -11410,6 +11718,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H310" s="2" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="n">
@@ -11445,6 +11754,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H311" s="2" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="n">
@@ -11480,6 +11790,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H312" s="2" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="n">
@@ -11515,6 +11826,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H313" s="2" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="n">
@@ -11550,6 +11862,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H314" s="2" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="n">
@@ -11585,6 +11898,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H315" s="2" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="n">
@@ -11620,6 +11934,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H316" s="2" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="n">
@@ -11655,6 +11970,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H317" s="2" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="n">
@@ -11690,6 +12006,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H318" s="2" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="n">
@@ -11725,6 +12042,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H319" s="2" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="n">
@@ -11760,6 +12078,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H320" s="2" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="n">
@@ -11795,6 +12114,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H321" s="2" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="n">
@@ -11830,6 +12150,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H322" s="2" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="n">
@@ -11865,6 +12186,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H323" s="2" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="2" t="n">
@@ -11900,6 +12222,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H324" s="2" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="n">
@@ -11935,6 +12258,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H325" s="2" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="n">
@@ -11970,6 +12294,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H326" s="2" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="n">
@@ -12005,6 +12330,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H327" s="2" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="n">
@@ -12040,6 +12366,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H328" s="2" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="n">
@@ -12075,6 +12402,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H329" s="2" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="n">
@@ -12110,6 +12438,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H330" s="2" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="n">
@@ -12145,6 +12474,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H331" s="2" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="n">
@@ -12180,6 +12510,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H332" s="2" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="n">
@@ -12215,6 +12546,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H333" s="2" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="n">
@@ -12250,6 +12582,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H334" s="2" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="n">
@@ -12292,6 +12625,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H335" s="2" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="n">
@@ -12327,6 +12661,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H336" s="2" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="n">
@@ -12362,6 +12697,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H337" s="2" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="n">
@@ -12397,6 +12733,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H338" s="2" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="n">
@@ -12432,6 +12769,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H339" s="2" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="n">
@@ -12467,6 +12805,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H340" s="2" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="n">
@@ -12502,6 +12841,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H341" s="2" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="n">
@@ -12537,6 +12877,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H342" s="2" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="n">
@@ -12572,6 +12913,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H343" s="2" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="2" t="n">
@@ -12607,6 +12949,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H344" s="2" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="n">
@@ -12642,6 +12985,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H345" s="2" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="n">
@@ -12677,6 +13021,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H346" s="2" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n">
@@ -12712,6 +13057,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H347" s="2" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n">
@@ -12747,6 +13093,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H348" s="2" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n">
@@ -12782,6 +13129,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H349" s="2" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n">
@@ -12817,6 +13165,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H350" s="2" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n">
@@ -12852,6 +13201,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H351" s="2" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n">
@@ -12887,6 +13237,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H352" s="2" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n">
@@ -12922,6 +13273,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H353" s="2" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n">
@@ -12957,6 +13309,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H354" s="2" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n">
@@ -12992,6 +13345,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H355" s="2" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n">
@@ -13027,6 +13381,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H356" s="2" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n">
@@ -13062,6 +13417,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H357" s="2" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n">
@@ -13097,6 +13453,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H358" s="2" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="n">
@@ -13132,6 +13489,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H359" s="2" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n">
@@ -13167,6 +13525,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H360" s="2" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n">
@@ -13202,6 +13561,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H361" s="2" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n">
@@ -13244,6 +13604,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H362" s="2" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n">
@@ -13279,6 +13640,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H363" s="2" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n">
@@ -13314,6 +13676,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H364" s="2" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="n">
@@ -13356,6 +13719,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H365" s="2" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="n">
@@ -13391,6 +13755,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H366" s="2" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n">
@@ -13433,6 +13798,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H367" s="2" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n">
@@ -13468,6 +13834,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H368" s="2" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n">
@@ -13503,6 +13870,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H369" s="2" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n">
@@ -13538,6 +13906,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H370" s="2" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n">
@@ -13573,6 +13942,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H371" s="2" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n">
@@ -13608,6 +13978,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H372" s="2" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n">
@@ -13643,6 +14014,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H373" s="2" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n">
@@ -13685,6 +14057,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H374" s="2" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n">
@@ -13720,6 +14093,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H375" s="2" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n">
@@ -13755,6 +14129,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H376" s="2" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n">
@@ -13790,6 +14165,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H377" s="2" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n">
@@ -13825,6 +14201,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H378" s="2" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n">
@@ -13860,6 +14237,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H379" s="2" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n">
@@ -13895,6 +14273,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H380" s="2" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n">
@@ -13930,6 +14309,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H381" s="2" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n">
@@ -13965,6 +14345,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H382" s="2" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n">
@@ -14000,6 +14381,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H383" s="2" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n">
@@ -14035,6 +14417,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H384" s="2" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n">
@@ -14070,6 +14453,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H385" s="2" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="n">
@@ -14105,6 +14489,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H386" s="2" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="n">
@@ -14140,6 +14525,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H387" s="2" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="n">
@@ -14175,6 +14561,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H388" s="2" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="n">
@@ -14210,6 +14597,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H389" s="2" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="n">
@@ -14245,6 +14633,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H390" s="2" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="n">
@@ -14280,6 +14669,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H391" s="2" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n">
@@ -14315,6 +14705,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H392" s="2" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n">
@@ -14350,6 +14741,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H393" s="2" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n">
@@ -14385,6 +14777,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H394" s="2" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n">
@@ -14420,6 +14813,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H395" s="2" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n">
@@ -14455,6 +14849,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H396" s="2" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n">
@@ -14497,6 +14892,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H397" s="2" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n">
@@ -14532,6 +14928,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H398" s="2" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n">
@@ -14567,6 +14964,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H399" s="2" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n">
@@ -14602,6 +15000,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H400" s="2" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n">
@@ -14637,6 +15036,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H401" s="2" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n">
@@ -14672,6 +15072,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H402" s="2" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n">
@@ -14707,6 +15108,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H403" s="2" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n">
@@ -14742,6 +15144,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H404" s="2" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n">
@@ -14777,6 +15180,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H405" s="2" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n">
@@ -14812,6 +15216,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H406" s="2" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n">
@@ -14847,6 +15252,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H407" s="2" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n">
@@ -14882,6 +15288,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H408" s="2" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n">
@@ -14917,6 +15324,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H409" s="2" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n">
@@ -14952,6 +15360,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H410" s="2" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n">
@@ -14987,6 +15396,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H411" s="2" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n">
@@ -15022,6 +15432,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H412" s="2" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n">
@@ -15057,6 +15468,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H413" s="2" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n">
@@ -15092,6 +15504,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H414" s="2" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n">
@@ -15127,6 +15540,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H415" s="2" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n">
@@ -15162,6 +15576,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H416" s="2" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n">
@@ -15197,6 +15612,7 @@
           <t>Instagram - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H417" s="2" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n">
@@ -15239,6 +15655,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H418" s="2" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n">
@@ -15274,6 +15691,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H419" s="2" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n">
@@ -15316,6 +15734,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H420" s="2" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n">
@@ -15351,6 +15770,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H421" s="2" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n">
@@ -15386,6 +15806,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H422" s="2" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n">
@@ -15421,6 +15842,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H423" s="2" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n">
@@ -15456,6 +15878,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H424" s="2" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n">
@@ -15491,6 +15914,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H425" s="2" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n">
@@ -15526,6 +15950,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H426" s="2" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n">
@@ -15561,6 +15986,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H427" s="2" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n">
@@ -15596,6 +16022,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H428" s="2" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n">
@@ -15631,6 +16058,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H429" s="2" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n">
@@ -15666,6 +16094,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H430" s="2" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n">
@@ -15701,6 +16130,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H431" s="2" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n">
@@ -15736,6 +16166,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H432" s="2" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n">
@@ -15771,6 +16202,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H433" s="2" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n">
@@ -15806,6 +16238,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H434" s="2" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n">
@@ -15841,6 +16274,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H435" s="2" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n">
@@ -15876,6 +16310,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H436" s="2" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n">
@@ -15911,6 +16346,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H437" s="2" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n">
@@ -15946,6 +16382,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H438" s="2" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n">
@@ -15981,6 +16418,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H439" s="2" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n">
@@ -16016,6 +16454,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H440" s="2" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n">
@@ -16051,6 +16490,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H441" s="2" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n">
@@ -16086,6 +16526,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H442" s="2" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n">
@@ -16121,6 +16562,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H443" s="2" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n">
@@ -16156,6 +16598,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H444" s="2" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n">
@@ -16191,6 +16634,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H445" s="2" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n">
@@ -16226,6 +16670,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H446" s="2" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n">
@@ -16261,6 +16706,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H447" s="2" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n">
@@ -16296,6 +16742,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H448" s="2" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n">
@@ -16331,6 +16778,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H449" s="2" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n">
@@ -16366,6 +16814,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H450" s="2" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n">
@@ -16401,6 +16850,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H451" s="2" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n">
@@ -16436,6 +16886,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H452" s="2" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n">
@@ -16471,6 +16922,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H453" s="2" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n">
@@ -16506,6 +16958,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H454" s="2" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n">
@@ -16541,6 +16994,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H455" s="2" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n">
@@ -16576,6 +17030,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H456" s="2" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n">
@@ -16611,6 +17066,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H457" s="2" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n">
@@ -16646,6 +17102,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H458" s="2" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n">
@@ -16681,6 +17138,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H459" s="2" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n">
@@ -16716,6 +17174,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H460" s="2" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n">
@@ -16751,6 +17210,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H461" s="2" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n">
@@ -16786,6 +17246,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H462" s="2" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n">
@@ -16821,6 +17282,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H463" s="2" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n">
@@ -16863,6 +17325,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H464" s="2" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n">
@@ -16898,6 +17361,7 @@
           <t>Meta - Whatsapp</t>
         </is>
       </c>
+      <c r="H465" s="2" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n">
@@ -16933,6 +17397,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H466" s="2" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n">
@@ -16968,6 +17433,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H467" s="2" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n">
@@ -17003,6 +17469,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H468" s="2" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n">
@@ -17038,6 +17505,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H469" s="2" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n">
@@ -17073,6 +17541,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H470" s="2" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n">
@@ -17108,6 +17577,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H471" s="2" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n">
@@ -17143,6 +17613,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H472" s="2" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n">
@@ -17178,6 +17649,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H473" s="2" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n">
@@ -17213,6 +17685,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H474" s="2" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n">
@@ -17248,6 +17721,7 @@
           <t>Whatsapp</t>
         </is>
       </c>
+      <c r="H475" s="2" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n">
@@ -17283,6 +17757,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H476" s="2" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n">
@@ -17318,6 +17793,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H477" s="2" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n">
@@ -17353,6 +17829,7 @@
           <t>Facebook - Whatsapp (Video)</t>
         </is>
       </c>
+      <c r="H478" s="2" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n">
@@ -17388,6 +17865,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H479" s="2" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n">
@@ -17423,6 +17901,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H480" s="2" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n">
@@ -17458,6 +17937,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H481" s="2" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="2" t="n">
@@ -17493,6 +17973,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H482" s="2" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="2" t="n">
@@ -17528,6 +18009,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H483" s="2" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="2" t="n">
@@ -17563,6 +18045,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H484" s="2" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="2" t="n">
@@ -17605,6 +18088,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H485" s="2" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="2" t="n">
@@ -17640,6 +18124,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H486" s="2" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="2" t="n">
@@ -17675,6 +18160,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H487" s="2" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="2" t="n">
@@ -17710,6 +18196,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H488" s="2" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n">
@@ -17745,6 +18232,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H489" s="2" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n">
@@ -17780,6 +18268,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H490" s="2" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n">
@@ -17815,6 +18304,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H491" s="2" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n">
@@ -17850,6 +18340,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H492" s="2" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n">
@@ -17885,6 +18376,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H493" s="2" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="2" t="n">
@@ -17920,6 +18412,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H494" s="2" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="2" t="n">
@@ -17955,6 +18448,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H495" s="2" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="n">
@@ -17990,6 +18484,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H496" s="2" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="2" t="n">
@@ -18032,6 +18527,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H497" s="2" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="2" t="n">
@@ -18067,6 +18563,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H498" s="2" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="2" t="n">
@@ -18102,6 +18599,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H499" s="2" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="2" t="n">
@@ -18144,6 +18642,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H500" s="2" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="2" t="n">
@@ -18179,6 +18678,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H501" s="2" t="n"/>
     </row>
     <row r="502">
       <c r="A502" s="2" t="n">
@@ -18214,6 +18714,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H502" s="2" t="n"/>
     </row>
     <row r="503">
       <c r="A503" s="2" t="n">
@@ -18249,6 +18750,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H503" s="2" t="n"/>
     </row>
     <row r="504">
       <c r="A504" s="2" t="n">
@@ -18284,6 +18786,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H504" s="2" t="n"/>
     </row>
     <row r="505">
       <c r="A505" s="2" t="n">
@@ -18319,6 +18822,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H505" s="2" t="n"/>
     </row>
     <row r="506">
       <c r="A506" s="2" t="n">
@@ -18354,6 +18858,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H506" s="2" t="n"/>
     </row>
     <row r="507">
       <c r="A507" s="2" t="n">
@@ -18389,6 +18894,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H507" s="2" t="n"/>
     </row>
     <row r="508">
       <c r="A508" s="2" t="n">
@@ -18424,6 +18930,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H508" s="2" t="n"/>
     </row>
     <row r="509">
       <c r="A509" s="2" t="n">
@@ -18459,6 +18966,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H509" s="2" t="n"/>
     </row>
     <row r="510">
       <c r="A510" s="2" t="n">
@@ -18494,6 +19002,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H510" s="2" t="n"/>
     </row>
     <row r="511">
       <c r="A511" s="2" t="n">
@@ -18529,6 +19038,7 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H511" s="2" t="n"/>
     </row>
     <row r="512">
       <c r="A512" s="2" t="n">
@@ -18564,6 +19074,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H512" s="2" t="n"/>
     </row>
     <row r="513">
       <c r="A513" s="2" t="n">
@@ -18599,6 +19110,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H513" s="2" t="n"/>
     </row>
     <row r="514">
       <c r="A514" s="2" t="n">
@@ -18634,6 +19146,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H514" s="2" t="n"/>
     </row>
     <row r="515">
       <c r="A515" s="2" t="n">
@@ -18669,6 +19182,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H515" s="2" t="n"/>
     </row>
     <row r="516">
       <c r="A516" s="2" t="n">
@@ -18704,6 +19218,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H516" s="2" t="n"/>
     </row>
     <row r="517">
       <c r="A517" s="2" t="n">
@@ -18739,6 +19254,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H517" s="2" t="n"/>
     </row>
     <row r="518">
       <c r="A518" s="2" t="n">
@@ -18781,6 +19297,7 @@
           <t>Landing Page V2</t>
         </is>
       </c>
+      <c r="H518" s="2" t="n"/>
     </row>
     <row r="519">
       <c r="A519" s="2" t="n">
@@ -18816,6 +19333,7 @@
           <t>Facebook - Whatsapp</t>
         </is>
       </c>
+      <c r="H519" s="2" t="n"/>
     </row>
     <row r="520">
       <c r="A520" s="2" t="n">
@@ -18851,6 +19369,547 @@
           <t>Instagram - Whatsapp</t>
         </is>
       </c>
+      <c r="H520" s="2" t="n"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="n">
+        <v>520</v>
+      </c>
+      <c r="B521" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1863-2112</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>em</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="F521" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G521" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H521" s="2" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="n">
+        <v>521</v>
+      </c>
+      <c r="B522" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5643-9841</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>Dheepina.U</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G522" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H522" s="2" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="n">
+        <v>522</v>
+      </c>
+      <c r="B523" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5910-1167</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>Wanwanhilwana</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>19:13</t>
+        </is>
+      </c>
+      <c r="F523" s="2" t="inlineStr">
+        <is>
+          <t>Saya mau tanya harga penutup mobil nisan mach berapa? (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G523" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H523" s="2" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="n">
+        <v>523</v>
+      </c>
+      <c r="B524" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4006-2224</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>CIYI</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G524" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H524" s="2" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="n">
+        <v>524</v>
+      </c>
+      <c r="B525" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-3518-1761</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>JUNAIDI ANTI GALAO</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="F525" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G525" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H525" s="2" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="n">
+        <v>525</v>
+      </c>
+      <c r="B526" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6419-3339</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>jimi</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="F526" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G526" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H526" s="2" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="n">
+        <v>526</v>
+      </c>
+      <c r="B527" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C527" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8441-9999</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>Andi</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F527" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat Inova</t>
+        </is>
+      </c>
+      <c r="G527" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H527" s="2" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="n">
+        <v>527</v>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5424-3900</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>Rin@</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G528" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H528" s="2" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="B529" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-8074-6550</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>faizalrachman</t>
+        </is>
+      </c>
+      <c r="E529" s="2" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="F529" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G529" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H529" s="2" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="n">
+        <v>529</v>
+      </c>
+      <c r="B530" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8443-6092</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>Rafidal</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="F530" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G530" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H530" s="2" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="n">
+        <v>530</v>
+      </c>
+      <c r="B531" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4519-8732</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>dewaat81</t>
+        </is>
+      </c>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="F531" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G531" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H531" s="2" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="n">
+        <v>531</v>
+      </c>
+      <c r="B532" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2645-5521</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>Herlina</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="F532" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ini nempel ga ya k Mobil?</t>
+        </is>
+      </c>
+      <c r="G532" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H532" s="2" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="n">
+        <v>532</v>
+      </c>
+      <c r="B533" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C533" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3923-0108</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>Brigadir g ADC23+</t>
+        </is>
+      </c>
+      <c r="E533" s="2" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="F533" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brpa harganya</t>
+        </is>
+      </c>
+      <c r="G533" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H533" s="2" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="n">
+        <v>533</v>
+      </c>
+      <c r="B534" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-4393-6664</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>Joizpuccaka</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="F534" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G534" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H534" s="2" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="n">
+        <v>534</v>
+      </c>
+      <c r="B535" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C535" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4773-5817</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>❤️ EBEN PHILIP ESTER ❤️</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="F535" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G535" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H535" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add batch 44 of leads WA (11-12 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H535"/>
+  <dimension ref="A1:H550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -19911,6 +19911,546 @@
       </c>
       <c r="H535" s="2" t="inlineStr"/>
     </row>
+    <row r="536">
+      <c r="A536" s="2" t="n">
+        <v>535</v>
+      </c>
+      <c r="B536" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C536" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-6658-416</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>Jek</t>
+        </is>
+      </c>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="F536" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G536" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H536" s="2" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="n">
+        <v>536</v>
+      </c>
+      <c r="B537" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C537" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4575-8564</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>Munip Ismail</t>
+        </is>
+      </c>
+      <c r="E537" s="2" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="F537" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G537" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H537" s="2" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="n">
+        <v>537</v>
+      </c>
+      <c r="B538" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C538" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3699-9525</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>I Gusti Ngurah Adnyana</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="F538" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untk Avanza ada</t>
+        </is>
+      </c>
+      <c r="G538" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H538" s="2" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="n">
+        <v>538</v>
+      </c>
+      <c r="B539" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9805-3600</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>Farisal Dg Rowa</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="F539" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G539" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H539" s="2" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="n">
+        <v>539</v>
+      </c>
+      <c r="B540" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C540" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3941-7088</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>emi tjeunfin</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="F540" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G540" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H540" s="2" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="B541" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C541" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-2550-7106</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>Luklukretnaningsih</t>
+        </is>
+      </c>
+      <c r="E541" s="2" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="F541" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa kak harganya</t>
+        </is>
+      </c>
+      <c r="G541" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H541" s="2" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="n">
+        <v>541</v>
+      </c>
+      <c r="B542" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C542" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-654-705</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>Reynold</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="F542" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G542" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H542" s="2" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="n">
+        <v>542</v>
+      </c>
+      <c r="B543" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C543" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-0006-45161</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>Dhion P</t>
+        </is>
+      </c>
+      <c r="E543" s="2" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="F543" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G543" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H543" s="2" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="n">
+        <v>543</v>
+      </c>
+      <c r="B544" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C544" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8201-0158</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>Mas Iswanto</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="F544" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G544" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H544" s="2" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="n">
+        <v>544</v>
+      </c>
+      <c r="B545" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C545" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3757-8006</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>Marthen Marten</t>
+        </is>
+      </c>
+      <c r="E545" s="2" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="F545" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Bahan dr kain atau terpal ya</t>
+        </is>
+      </c>
+      <c r="G545" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H545" s="2" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="n">
+        <v>545</v>
+      </c>
+      <c r="B546" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C546" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4192-9714</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>ishak</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="inlineStr">
+        <is>
+          <t>21:53</t>
+        </is>
+      </c>
+      <c r="F546" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G546" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H546" s="2" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="n">
+        <v>546</v>
+      </c>
+      <c r="B547" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3014-7761</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>Ridho Rochman (od)</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="F547" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G547" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H547" s="2" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="n">
+        <v>547</v>
+      </c>
+      <c r="B548" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-2934-1184</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>Agil Mawahib</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F548" s="2" t="inlineStr">
+        <is>
+          <t>permisi kak / cover mobil jazzgk5 berapa ya (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G548" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H548" s="2" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="n">
+        <v>548</v>
+      </c>
+      <c r="B549" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-3365-3085</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>Banuartha</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="F549" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cover untuk honda jazz ada</t>
+        </is>
+      </c>
+      <c r="G549" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H549" s="2" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="n">
+        <v>549</v>
+      </c>
+      <c r="B550" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-5701-973</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>Jalal</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berpa hrga cover jika COD sampai lombok Ntb</t>
+        </is>
+      </c>
+      <c r="G550" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H550" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batches 45-46 of leads WA (4, 10-12 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H550"/>
+  <dimension ref="A1:H580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -20451,6 +20451,1114 @@
       </c>
       <c r="H550" s="2" t="inlineStr"/>
     </row>
+    <row r="551">
+      <c r="A551" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="B551" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3501-0506</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>Dedy</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G551" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="n">
+        <v>551</v>
+      </c>
+      <c r="B552" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-4918-2824</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>Pan Juna</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak! Kalo buat susuki splash brp?</t>
+        </is>
+      </c>
+      <c r="G552" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H552" s="2" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="n">
+        <v>552</v>
+      </c>
+      <c r="B553" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5659-1578</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>daltonalpenos</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Wulling confero DB</t>
+        </is>
+      </c>
+      <c r="G553" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H553" s="2" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="n">
+        <v>553</v>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-6621-7036</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>Kallo Chandra,S.Sos</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G554" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H554" s="2" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="n">
+        <v>554</v>
+      </c>
+      <c r="B555" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1791-972</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>💕HeCla Sulcata💕</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat new ertiga 2023</t>
+        </is>
+      </c>
+      <c r="G555" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H555" s="2" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="n">
+        <v>555</v>
+      </c>
+      <c r="B556" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-3244-0553</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>Yudi</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="inlineStr">
+        <is>
+          <t>Cek mahar buat Agiya Thun 2017 / Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G556" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H556" s="2" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="n">
+        <v>556</v>
+      </c>
+      <c r="B557" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C557" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9671-9415</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>Van_da</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="F557" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G557" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H557" s="2" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="n">
+        <v>557</v>
+      </c>
+      <c r="B558" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7051-7612</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>Iman</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>12:16</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cover unyuk mobil Rush thn 2025 brp harga nya</t>
+        </is>
+      </c>
+      <c r="G558" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H558" s="2" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="n">
+        <v>558</v>
+      </c>
+      <c r="B559" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C559" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4730-1239</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>Kristino Sumedi</t>
+        </is>
+      </c>
+      <c r="E559" s="2" t="inlineStr">
+        <is>
+          <t>01:44</t>
+        </is>
+      </c>
+      <c r="F559" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G559" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H559" s="2" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="n">
+        <v>559</v>
+      </c>
+      <c r="B560" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C560" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-731-841</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Koko</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>04:40</t>
+        </is>
+      </c>
+      <c r="F560" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare ini beneran 299 rb</t>
+        </is>
+      </c>
+      <c r="G560" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H560" s="2" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="B561" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C561" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4305-9648</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>nama Sy Ibu Nanie</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="inlineStr">
+        <is>
+          <t>07:33</t>
+        </is>
+      </c>
+      <c r="F561" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa harganya harganya Ada sarung mobil sigra</t>
+        </is>
+      </c>
+      <c r="G561" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H561" s="2" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="n">
+        <v>561</v>
+      </c>
+      <c r="B562" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>+62 897-0399-961</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>Jeffry Julius Santosa</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="F562" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil: aion ut
+Tahun Mobil: 2026
+Nama Penerima: Jeffry
+Alamat Penerima: Jl. Let. Kol. Isdiman no. 114 A, Bancar, Purbalingga
+Tipe Cover: Reguler
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G562" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H562" s="2" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="n">
+        <v>562</v>
+      </c>
+      <c r="B563" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-3361-3299</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>Juliana Balo</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="F563" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ayla brp</t>
+        </is>
+      </c>
+      <c r="G563" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H563" s="2" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="n">
+        <v>563</v>
+      </c>
+      <c r="B564" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-1801-064</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>Suhadi</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="F564" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: Byd
+Tipe Mobil: Sealoin 7
+Tahun Mobil: 2025
+Nama Penerima:
+Alamat  Jl. Pluit karang indah 1 no 35. (Block P 8 Utara 35. Muara karang , Pluit, Jakarta Utara. Penerima: Suhadi  A.T.
+Tipe Cover: yg 3 layer  Diatas reguler. (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G564" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H564" s="2" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="n">
+        <v>564</v>
+      </c>
+      <c r="B565" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C565" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-5216-777</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>Endro Susanto (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E565" s="2" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="F565" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G565" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H565" s="2" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="n">
+        <v>565</v>
+      </c>
+      <c r="B566" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6810-2223</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>Doan</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="F566" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G566" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H566" s="2" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="n">
+        <v>566</v>
+      </c>
+      <c r="B567" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C567" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0353-6060</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>Munawir Haris</t>
+        </is>
+      </c>
+      <c r="E567" s="2" t="inlineStr">
+        <is>
+          <t>17:19</t>
+        </is>
+      </c>
+      <c r="F567" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G567" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H567" s="2" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="n">
+        <v>567</v>
+      </c>
+      <c r="B568" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-6690-330</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>Afmi Yarsi</t>
+        </is>
+      </c>
+      <c r="E568" s="2" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="F568" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G568" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H568" s="2" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="n">
+        <v>568</v>
+      </c>
+      <c r="B569" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-4148-741</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>OmBepe741</t>
+        </is>
+      </c>
+      <c r="E569" s="2" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="F569" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G569" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H569" s="2" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="n">
+        <v>569</v>
+      </c>
+      <c r="B570" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-3925-0487</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>you yeng</t>
+        </is>
+      </c>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F570" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G570" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H570" s="2" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="B571" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C571" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-3761-2420</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>idoy (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E571" s="2" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="F571" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G571" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H571" s="2" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="n">
+        <v>571</v>
+      </c>
+      <c r="B572" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9859-6991</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>Abdul Hadi</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="F572" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G572" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H572" s="2" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="n">
+        <v>572</v>
+      </c>
+      <c r="B573" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-8115-9752</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>Ahmad kader</t>
+        </is>
+      </c>
+      <c r="E573" s="2" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="F573" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G573" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H573" s="2" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="n">
+        <v>573</v>
+      </c>
+      <c r="B574" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8141-8681</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>19:33</t>
+        </is>
+      </c>
+      <c r="F574" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G574" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H574" s="2" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="n">
+        <v>574</v>
+      </c>
+      <c r="B575" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C575" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9343-8488</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>Desmon Sasikome</t>
+        </is>
+      </c>
+      <c r="E575" s="2" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="F575" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G575" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H575" s="2" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="B576" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8750-8606</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>Dudun</t>
+        </is>
+      </c>
+      <c r="E576" s="2" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="F576" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G576" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H576" s="2" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="n">
+        <v>576</v>
+      </c>
+      <c r="B577" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C577" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4200-631</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>Mhila Mh</t>
+        </is>
+      </c>
+      <c r="E577" s="2" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="F577" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Rush</t>
+        </is>
+      </c>
+      <c r="G577" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H577" s="2" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="n">
+        <v>577</v>
+      </c>
+      <c r="B578" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6698-6950</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>Juniarman Simanjuntak</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="F578" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G578" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H578" s="2" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="n">
+        <v>578</v>
+      </c>
+      <c r="B579" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8882-7878</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>Imran Rasul</t>
+        </is>
+      </c>
+      <c r="E579" s="2" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="F579" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G579" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H579" s="2" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="n">
+        <v>579</v>
+      </c>
+      <c r="B580" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C580" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3929-8717</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>arispadji12</t>
+        </is>
+      </c>
+      <c r="E580" s="2" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="F580" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G580" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H580" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 47 of leads WA (12 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H580"/>
+  <dimension ref="A1:H587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -21559,6 +21559,265 @@
       </c>
       <c r="H580" s="2" t="inlineStr"/>
     </row>
+    <row r="581">
+      <c r="A581" s="2" t="n">
+        <v>580</v>
+      </c>
+      <c r="B581" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C581" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-4000-0627</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>Jefry</t>
+        </is>
+      </c>
+      <c r="E581" s="2" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="F581" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G581" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H581" s="2" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="n">
+        <v>581</v>
+      </c>
+      <c r="B582" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-6404-1883</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>Indah</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="F582" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G582" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H582" s="2" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="n">
+        <v>582</v>
+      </c>
+      <c r="B583" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C583" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6364-5992</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>EdyeGinting</t>
+        </is>
+      </c>
+      <c r="E583" s="2" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="F583" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G583" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H583" s="2" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="n">
+        <v>583</v>
+      </c>
+      <c r="B584" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-8177-767</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>Jansen</t>
+        </is>
+      </c>
+      <c r="E584" s="2" t="inlineStr">
+        <is>
+          <t>04:40</t>
+        </is>
+      </c>
+      <c r="F584" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G584" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H584" s="2" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="n">
+        <v>584</v>
+      </c>
+      <c r="B585" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C585" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9280-2364</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="E585" s="2" t="inlineStr">
+        <is>
+          <t>05:10</t>
+        </is>
+      </c>
+      <c r="F585" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G585" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H585" s="2" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="n">
+        <v>585</v>
+      </c>
+      <c r="B586" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-1638-0043</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>Bang</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="F586" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G586" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H586" s="2" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="n">
+        <v>586</v>
+      </c>
+      <c r="B587" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-143-508</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>Mountnear (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="F587" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G587" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H587" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 48 of leads WA (1, 13-18 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H587"/>
+  <dimension ref="A1:H600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -21818,6 +21818,474 @@
       </c>
       <c r="H587" s="2" t="inlineStr"/>
     </row>
+    <row r="588">
+      <c r="A588" s="2" t="n">
+        <v>587</v>
+      </c>
+      <c r="B588" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4939-6545</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>Cia Liem Augusta</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>02:12</t>
+        </is>
+      </c>
+      <c r="F588" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G588" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H588" s="2" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="n">
+        <v>588</v>
+      </c>
+      <c r="B589" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C589" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-1354-1664</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>Eko Purwanto</t>
+        </is>
+      </c>
+      <c r="E589" s="2" t="inlineStr">
+        <is>
+          <t>22:29</t>
+        </is>
+      </c>
+      <c r="F589" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G589" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H589" s="2" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="n">
+        <v>589</v>
+      </c>
+      <c r="B590" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-2248-0623</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>Taswin, L.😍</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="F590" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G590" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H590" s="2" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="n">
+        <v>590</v>
+      </c>
+      <c r="B591" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C591" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9681-7775</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>I Wayan Taker</t>
+        </is>
+      </c>
+      <c r="E591" s="2" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="F591" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil Rush GR Sport 2026</t>
+        </is>
+      </c>
+      <c r="G591" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H591" s="2" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="n">
+        <v>591</v>
+      </c>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5131-4689</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>Willy</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="F592" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G592" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H592" s="2" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="n">
+        <v>592</v>
+      </c>
+      <c r="B593" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7484-1840</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>batammmm33</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="F593" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa</t>
+        </is>
+      </c>
+      <c r="G593" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H593" s="2" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="n">
+        <v>593</v>
+      </c>
+      <c r="B594" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2139-3098</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>cef fian</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="F594" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G594" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H594" s="2" t="inlineStr"/>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="n">
+        <v>594</v>
+      </c>
+      <c r="B595" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C595" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-6393-9277</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>Fajar P.</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="F595" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G595" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H595" s="2" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="n">
+        <v>595</v>
+      </c>
+      <c r="B596" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C596" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7588-6792</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>SITOR SITUMORANG</t>
+        </is>
+      </c>
+      <c r="E596" s="2" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="F596" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G596" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H596" s="2" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="n">
+        <v>596</v>
+      </c>
+      <c r="B597" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C597" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5399-3774</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>Efren</t>
+        </is>
+      </c>
+      <c r="E597" s="2" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="F597" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G597" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H597" s="2" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="n">
+        <v>597</v>
+      </c>
+      <c r="B598" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-2586-1334</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>Siswoto</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="F598" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G598" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H598" s="2" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="n">
+        <v>598</v>
+      </c>
+      <c r="B599" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C599" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-6849-4678</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="E599" s="2" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="F599" s="2" t="inlineStr">
+        <is>
+          <t>Price list (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G599" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H599" s="2" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="n">
+        <v>599</v>
+      </c>
+      <c r="B600" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-5259-3563</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>Tarajuh</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="F600" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G600" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H600" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 49 of leads WA (16-17 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H600"/>
+  <dimension ref="A1:H613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -22286,6 +22286,474 @@
       </c>
       <c r="H600" s="2" t="inlineStr"/>
     </row>
+    <row r="601">
+      <c r="A601" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="B601" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C601" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3768-7911</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E601" s="2" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="F601" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G601" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H601" s="2" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="n">
+        <v>601</v>
+      </c>
+      <c r="B602" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6755-8955</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>Hasbi Rukman</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="F602" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G602" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H602" s="2" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="n">
+        <v>602</v>
+      </c>
+      <c r="B603" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6202-1984</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>Sibuk. (Tinggalkan Pesan)</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="F603" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G603" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H603" s="2" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="n">
+        <v>603</v>
+      </c>
+      <c r="B604" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-2338-3309</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>RizqyRA</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="F604" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G604" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H604" s="2" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="n">
+        <v>604</v>
+      </c>
+      <c r="B605" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6813-4891</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>Samsudin</t>
+        </is>
+      </c>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="F605" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G605" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H605" s="2" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="n">
+        <v>605</v>
+      </c>
+      <c r="B606" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4220-2423</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>🙏</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="F606" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare mobil Terios 2019 ada?</t>
+        </is>
+      </c>
+      <c r="G606" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H606" s="2" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="n">
+        <v>606</v>
+      </c>
+      <c r="B607" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5656-6794</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>nurul kesya 077</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="F607" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brp harga Avanza velox bos, ku</t>
+        </is>
+      </c>
+      <c r="G607" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H607" s="2" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="n">
+        <v>607</v>
+      </c>
+      <c r="B608" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-7388-2798</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Abduh</t>
+        </is>
+      </c>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="F608" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G608" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H608" s="2" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="n">
+        <v>608</v>
+      </c>
+      <c r="B609" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C609" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-2688-5261</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="E609" s="2" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="F609" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Untuk xpander 2022 dikisaran harga brpa ya kak?</t>
+        </is>
+      </c>
+      <c r="G609" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H609" s="2" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="n">
+        <v>609</v>
+      </c>
+      <c r="B610" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4728-4005</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>RommyCfranS</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="F610" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G610" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H610" s="2" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="n">
+        <v>610</v>
+      </c>
+      <c r="B611" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C611" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-6460-4555</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>Azhar Budi</t>
+        </is>
+      </c>
+      <c r="E611" s="2" t="inlineStr">
+        <is>
+          <t>20:12</t>
+        </is>
+      </c>
+      <c r="F611" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Admin. Berapa harga selimut mobil</t>
+        </is>
+      </c>
+      <c r="G611" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H611" s="2" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="n">
+        <v>611</v>
+      </c>
+      <c r="B612" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C612" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-7104-786</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>.yadi</t>
+        </is>
+      </c>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="F612" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G612" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H612" s="2" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="n">
+        <v>612</v>
+      </c>
+      <c r="B613" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C613" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-2802-1985</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>Nanda Saputra</t>
+        </is>
+      </c>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t>18:13</t>
+        </is>
+      </c>
+      <c r="F613" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G613" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H613" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 50 of leads WA (15, 17-18 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H613"/>
+  <dimension ref="A1:H629"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -22754,6 +22754,582 @@
       </c>
       <c r="H613" s="2" t="inlineStr"/>
     </row>
+    <row r="614">
+      <c r="A614" s="2" t="n">
+        <v>613</v>
+      </c>
+      <c r="B614" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C614" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5077-7017</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>dewi</t>
+        </is>
+      </c>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="F614" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G614" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H614" s="2" t="inlineStr"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="n">
+        <v>614</v>
+      </c>
+      <c r="B615" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C615" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5710-2328</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>raconoldy</t>
+        </is>
+      </c>
+      <c r="E615" s="2" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="F615" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G615" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H615" s="2" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="n">
+        <v>615</v>
+      </c>
+      <c r="B616" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C616" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6759-5886</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>✍</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="F616" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G616" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H616" s="2" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="n">
+        <v>616</v>
+      </c>
+      <c r="B617" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C617" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3884-0867</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>Kornelis Subir</t>
+        </is>
+      </c>
+      <c r="E617" s="2" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="F617" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G617" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H617" s="2" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="n">
+        <v>617</v>
+      </c>
+      <c r="B618" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C618" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-2535-6885</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>Nuryanto</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>16:33</t>
+        </is>
+      </c>
+      <c r="F618" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G618" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H618" s="2" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="n">
+        <v>618</v>
+      </c>
+      <c r="B619" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C619" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7408-9152</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="F619" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G619" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H619" s="2" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="n">
+        <v>619</v>
+      </c>
+      <c r="B620" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9693-8627</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>Vedy</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="F620" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G620" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H620" s="2" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="n">
+        <v>620</v>
+      </c>
+      <c r="B621" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2345-8824</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>azam mokoagow</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="F621" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G621" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H621" s="2" t="inlineStr"/>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="n">
+        <v>621</v>
+      </c>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9000-0758</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>Bombom</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G622" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H622" s="2" t="inlineStr"/>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="n">
+        <v>622</v>
+      </c>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8046-0243</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>Gus Hanif</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="F623" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G623" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H623" s="2" t="inlineStr"/>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="n">
+        <v>623</v>
+      </c>
+      <c r="B624" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6563-5693</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Tarmin</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G624" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H624" s="2" t="inlineStr"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="n">
+        <v>624</v>
+      </c>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-1474-6404</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>Isyaa</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>21:51</t>
+        </is>
+      </c>
+      <c r="F625" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G625" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H625" s="2" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="n">
+        <v>625</v>
+      </c>
+      <c r="B626" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8885-6943</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>Destiana</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>23:33</t>
+        </is>
+      </c>
+      <c r="F626" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G626" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H626" s="2" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="n">
+        <v>626</v>
+      </c>
+      <c r="B627" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C627" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5534-9690</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>Ahdar</t>
+        </is>
+      </c>
+      <c r="E627" s="2" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="F627" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dengan awalan: saya taya harga dulu)</t>
+        </is>
+      </c>
+      <c r="G627" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H627" s="2" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="n">
+        <v>627</v>
+      </c>
+      <c r="B628" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C628" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-535-667</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>kamalpaser1970</t>
+        </is>
+      </c>
+      <c r="E628" s="2" t="inlineStr">
+        <is>
+          <t>06:07</t>
+        </is>
+      </c>
+      <c r="F628" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G628" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H628" s="2" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="n">
+        <v>628</v>
+      </c>
+      <c r="B629" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C629" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-6733-2133</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>danuparpum</t>
+        </is>
+      </c>
+      <c r="E629" s="2" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="F629" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G629" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H629" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 51 of leads WA (13-14, 17-18 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H629"/>
+  <dimension ref="A1:H644"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -23330,6 +23330,542 @@
       </c>
       <c r="H629" s="2" t="inlineStr"/>
     </row>
+    <row r="630">
+      <c r="A630" s="2" t="n">
+        <v>629</v>
+      </c>
+      <c r="B630" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C630" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8174-7743</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>UMAR</t>
+        </is>
+      </c>
+      <c r="E630" s="2" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="F630" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Kalau untuk rush gr adakah</t>
+        </is>
+      </c>
+      <c r="G630" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H630" s="2" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="n">
+        <v>630</v>
+      </c>
+      <c r="B631" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C631" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6536-8355</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>Ferdananta Tarigan</t>
+        </is>
+      </c>
+      <c r="E631" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="F631" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G631" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H631" s="2" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="n">
+        <v>631</v>
+      </c>
+      <c r="B632" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C632" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-1058-3998</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>faiha aziza</t>
+        </is>
+      </c>
+      <c r="E632" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="F632" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G632" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H632" s="2" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="n">
+        <v>632</v>
+      </c>
+      <c r="B633" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C633" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3335-4036</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>Dominggus@Punk</t>
+        </is>
+      </c>
+      <c r="E633" s="2" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="F633" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G633" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H633" s="2" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="n">
+        <v>633</v>
+      </c>
+      <c r="B634" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C634" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-0163-072</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>Lili</t>
+        </is>
+      </c>
+      <c r="E634" s="2" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="F634" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G634" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H634" s="2" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="n">
+        <v>634</v>
+      </c>
+      <c r="B635" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C635" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4975-0745</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>suwandydandy79</t>
+        </is>
+      </c>
+      <c r="E635" s="2" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="F635" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil efpansa ada kah</t>
+        </is>
+      </c>
+      <c r="G635" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H635" s="2" t="inlineStr"/>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="n">
+        <v>635</v>
+      </c>
+      <c r="B636" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C636" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1828-4699</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>Edy S</t>
+        </is>
+      </c>
+      <c r="E636" s="2" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="F636" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G636" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H636" s="2" t="inlineStr"/>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="n">
+        <v>636</v>
+      </c>
+      <c r="B637" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C637" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8825-5678</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>7€NDR¥</t>
+        </is>
+      </c>
+      <c r="E637" s="2" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="F637" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek Cover mobil Sigra</t>
+        </is>
+      </c>
+      <c r="G637" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H637" s="2" t="inlineStr"/>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="n">
+        <v>637</v>
+      </c>
+      <c r="B638" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C638" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6206-6090</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>annesmanalu9</t>
+        </is>
+      </c>
+      <c r="E638" s="2" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="F638" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G638" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H638" s="2" t="inlineStr"/>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="n">
+        <v>638</v>
+      </c>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3761-2816</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>Amj</t>
+        </is>
+      </c>
+      <c r="E639" s="2" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F639" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G639" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H639" s="2" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="n">
+        <v>639</v>
+      </c>
+      <c r="B640" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C640" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6930-472</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>~ Faisal Dj, SP</t>
+        </is>
+      </c>
+      <c r="E640" s="2" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="F640" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G640" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H640" s="2" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="B641" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C641" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-4648-3287</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>50 / 50</t>
+        </is>
+      </c>
+      <c r="E641" s="2" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="F641" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G641" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H641" s="2" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="n">
+        <v>641</v>
+      </c>
+      <c r="B642" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C642" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4017-7798</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>Musrifan ARMY 99_1</t>
+        </is>
+      </c>
+      <c r="E642" s="2" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="F642" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G642" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H642" s="2" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="n">
+        <v>642</v>
+      </c>
+      <c r="B643" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C643" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9832-4222</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr"/>
+      <c r="E643" s="2" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="F643" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G643" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H643" s="2" t="inlineStr"/>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="n">
+        <v>643</v>
+      </c>
+      <c r="B644" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C644" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3775-9445</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>Indar</t>
+        </is>
+      </c>
+      <c r="E644" s="2" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="F644" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G644" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H644" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 52 of leads WA (4, 16-17 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H644"/>
+  <dimension ref="A1:H658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -23866,6 +23866,506 @@
       </c>
       <c r="H644" s="2" t="inlineStr"/>
     </row>
+    <row r="645">
+      <c r="A645" s="2" t="n">
+        <v>644</v>
+      </c>
+      <c r="B645" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C645" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3125-7236</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>Sodikin</t>
+        </is>
+      </c>
+      <c r="E645" s="2" t="inlineStr">
+        <is>
+          <t>01:47</t>
+        </is>
+      </c>
+      <c r="F645" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G645" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H645" s="2" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="n">
+        <v>645</v>
+      </c>
+      <c r="B646" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C646" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-4841-1618</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr"/>
+      <c r="E646" s="2" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="F646" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G646" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H646" s="2" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="n">
+        <v>646</v>
+      </c>
+      <c r="B647" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C647" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-5359-1000</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>FarhanA</t>
+        </is>
+      </c>
+      <c r="E647" s="2" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="F647" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G647" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H647" s="2" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="n">
+        <v>647</v>
+      </c>
+      <c r="B648" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C648" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6763-7323</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>Mulya Ayang</t>
+        </is>
+      </c>
+      <c r="E648" s="2" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="F648" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G648" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H648" s="2" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="n">
+        <v>648</v>
+      </c>
+      <c r="B649" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C649" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6280-0212</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>tonggohon ham</t>
+        </is>
+      </c>
+      <c r="E649" s="2" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="F649" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G649" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H649" s="2" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="n">
+        <v>649</v>
+      </c>
+      <c r="B650" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C650" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1394-5773</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>RK</t>
+        </is>
+      </c>
+      <c r="E650" s="2" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="F650" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G650" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H650" s="2" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="B651" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C651" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-1556-7910</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>arifin123yusuf@gmail.com</t>
+        </is>
+      </c>
+      <c r="E651" s="2" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="F651" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G651" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H651" s="2" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="n">
+        <v>651</v>
+      </c>
+      <c r="B652" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C652" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9988-7310</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>Hj.lina karno</t>
+        </is>
+      </c>
+      <c r="E652" s="2" t="inlineStr">
+        <is>
+          <t>13:09</t>
+        </is>
+      </c>
+      <c r="F652" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G652" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H652" s="2" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="n">
+        <v>652</v>
+      </c>
+      <c r="B653" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4359-6678</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>Lestari</t>
+        </is>
+      </c>
+      <c r="E653" s="2" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="F653" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G653" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H653" s="2" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="n">
+        <v>653</v>
+      </c>
+      <c r="B654" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C654" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-6749-0298</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>ademaulinda40</t>
+        </is>
+      </c>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="F654" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek harga</t>
+        </is>
+      </c>
+      <c r="G654" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H654" s="2" t="inlineStr"/>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="n">
+        <v>654</v>
+      </c>
+      <c r="B655" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9818-2707</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>Deverly Malonda</t>
+        </is>
+      </c>
+      <c r="E655" s="2" t="inlineStr">
+        <is>
+          <t>05:04</t>
+        </is>
+      </c>
+      <c r="F655" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G655" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H655" s="2" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="n">
+        <v>655</v>
+      </c>
+      <c r="B656" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4020-1003</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>Oike Makalew</t>
+        </is>
+      </c>
+      <c r="E656" s="2" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="F656" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G656" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H656" s="2" t="inlineStr"/>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="n">
+        <v>656</v>
+      </c>
+      <c r="B657" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>+62 882-7179-4800</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>cece</t>
+        </is>
+      </c>
+      <c r="E657" s="2" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="F657" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G657" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H657" s="2" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="n">
+        <v>657</v>
+      </c>
+      <c r="B658" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C658" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6108-2767</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>komang</t>
+        </is>
+      </c>
+      <c r="E658" s="2" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F658" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G658" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H658" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 53 of leads WA (5, 10, 14, 16-17 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H658"/>
+  <dimension ref="A1:H672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -24366,6 +24366,510 @@
       </c>
       <c r="H658" s="2" t="inlineStr"/>
     </row>
+    <row r="659">
+      <c r="A659" s="2" t="n">
+        <v>658</v>
+      </c>
+      <c r="B659" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C659" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5566-2097</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>Il Aunaka</t>
+        </is>
+      </c>
+      <c r="E659" s="2" t="inlineStr">
+        <is>
+          <t>09:47</t>
+        </is>
+      </c>
+      <c r="F659" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G659" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H659" s="2" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="n">
+        <v>659</v>
+      </c>
+      <c r="B660" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7982-3956</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>putranipah02</t>
+        </is>
+      </c>
+      <c r="E660" s="2" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="F660" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G660" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H660" s="2" t="inlineStr"/>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="B661" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2013-4071</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>Desi</t>
+        </is>
+      </c>
+      <c r="E661" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G661" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H661" s="2" t="inlineStr"/>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="n">
+        <v>661</v>
+      </c>
+      <c r="B662" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5564-9097</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>M. HARUM</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
+          <t>18:19</t>
+        </is>
+      </c>
+      <c r="F662" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dikirim ulang 22:58) Cek harga Cover Mobil</t>
+        </is>
+      </c>
+      <c r="G662" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H662" s="2" t="inlineStr"/>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="B663" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C663" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8602-2558</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>Oding</t>
+        </is>
+      </c>
+      <c r="E663" s="2" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="F663" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G663" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H663" s="2" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="n">
+        <v>663</v>
+      </c>
+      <c r="B664" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C664" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-9197-1134</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>Scotty Bali (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E664" s="2" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="F664" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G664" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H664" s="2" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="n">
+        <v>664</v>
+      </c>
+      <c r="B665" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C665" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9208-9757</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>Elia Ramadhani❤️Bu Aziz</t>
+        </is>
+      </c>
+      <c r="E665" s="2" t="inlineStr">
+        <is>
+          <t>09:46</t>
+        </is>
+      </c>
+      <c r="F665" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G665" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H665" s="2" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="n">
+        <v>665</v>
+      </c>
+      <c r="B666" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C666" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-2000-5676</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>A.Hassan (AHS)</t>
+        </is>
+      </c>
+      <c r="E666" s="2" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="F666" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G666" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H666" s="2" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="n">
+        <v>666</v>
+      </c>
+      <c r="B667" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C667" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1997-043</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>Fendy</t>
+        </is>
+      </c>
+      <c r="E667" s="2" t="inlineStr">
+        <is>
+          <t>12:26</t>
+        </is>
+      </c>
+      <c r="F667" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G667" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H667" s="2" t="inlineStr"/>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="n">
+        <v>667</v>
+      </c>
+      <c r="B668" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C668" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3495-4898</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>Daffas Hadi</t>
+        </is>
+      </c>
+      <c r="E668" s="2" t="inlineStr">
+        <is>
+          <t>04:28</t>
+        </is>
+      </c>
+      <c r="F668" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G668" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H668" s="2" t="inlineStr"/>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="n">
+        <v>668</v>
+      </c>
+      <c r="B669" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C669" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7314-4618</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>Zulpikar</t>
+        </is>
+      </c>
+      <c r="E669" s="2" t="inlineStr">
+        <is>
+          <t>03:04</t>
+        </is>
+      </c>
+      <c r="F669" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G669" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H669" s="2" t="inlineStr"/>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="n">
+        <v>669</v>
+      </c>
+      <c r="B670" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C670" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7772-3888</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>A Hery A</t>
+        </is>
+      </c>
+      <c r="E670" s="2" t="inlineStr">
+        <is>
+          <t>00:12</t>
+        </is>
+      </c>
+      <c r="F670" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mobil Veloz 2023?</t>
+        </is>
+      </c>
+      <c r="G670" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H670" s="2" t="inlineStr"/>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
+        <v>670</v>
+      </c>
+      <c r="B671" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C671" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5868-2368</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>Khoi M</t>
+        </is>
+      </c>
+      <c r="E671" s="2" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="F671" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G671" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H671" s="2" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="B672" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C672" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5338-1105</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>TARO ADA TARO GAU</t>
+        </is>
+      </c>
+      <c r="E672" s="2" t="inlineStr">
+        <is>
+          <t>12:26</t>
+        </is>
+      </c>
+      <c r="F672" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G672" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H672" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 54 of leads WA (2, 16-17 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H672"/>
+  <dimension ref="A1:H687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -24870,6 +24870,546 @@
       </c>
       <c r="H672" s="2" t="inlineStr"/>
     </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
+        <v>672</v>
+      </c>
+      <c r="B673" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C673" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-4200-2592</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>AF.4634.3.max</t>
+        </is>
+      </c>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="F673" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brp harga ny</t>
+        </is>
+      </c>
+      <c r="G673" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H673" s="2" t="inlineStr"/>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
+        <v>673</v>
+      </c>
+      <c r="B674" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C674" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-1533-9731</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>Ida Samida</t>
+        </is>
+      </c>
+      <c r="E674" s="2" t="inlineStr">
+        <is>
+          <t>02:55</t>
+        </is>
+      </c>
+      <c r="F674" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga kak untuk Avansa</t>
+        </is>
+      </c>
+      <c r="G674" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H674" s="2" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
+        <v>674</v>
+      </c>
+      <c r="B675" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C675" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-6512-1326</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>Juwa1009</t>
+        </is>
+      </c>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>05:06</t>
+        </is>
+      </c>
+      <c r="F675" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G675" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H675" s="2" t="inlineStr"/>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
+        <v>675</v>
+      </c>
+      <c r="B676" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C676" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3206-4555</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>Lutfi Jepara</t>
+        </is>
+      </c>
+      <c r="E676" s="2" t="inlineStr">
+        <is>
+          <t>23:35</t>
+        </is>
+      </c>
+      <c r="F676" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G676" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H676" s="2" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
+        <v>676</v>
+      </c>
+      <c r="B677" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C677" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4933-8643</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>Bismillahirrahmanirrahim</t>
+        </is>
+      </c>
+      <c r="E677" s="2" t="inlineStr">
+        <is>
+          <t>05:21</t>
+        </is>
+      </c>
+      <c r="F677" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G677" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H677" s="2" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
+        <v>677</v>
+      </c>
+      <c r="B678" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C678" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3333-9210</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>Akhmad Saikhu</t>
+        </is>
+      </c>
+      <c r="E678" s="2" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="F678" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G678" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H678" s="2" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
+        <v>678</v>
+      </c>
+      <c r="B679" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C679" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7210-5137</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>JB</t>
+        </is>
+      </c>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>07:16</t>
+        </is>
+      </c>
+      <c r="F679" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G679" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H679" s="2" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
+        <v>679</v>
+      </c>
+      <c r="B680" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C680" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3941-2850</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>skono6318</t>
+        </is>
+      </c>
+      <c r="E680" s="2" t="inlineStr">
+        <is>
+          <t>06:10</t>
+        </is>
+      </c>
+      <c r="F680" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dikirim ulang)</t>
+        </is>
+      </c>
+      <c r="G680" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H680" s="2" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="B681" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C681" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-631-198</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>Parulian Hasudungan</t>
+        </is>
+      </c>
+      <c r="E681" s="2" t="inlineStr">
+        <is>
+          <t>04:14</t>
+        </is>
+      </c>
+      <c r="F681" s="2" t="inlineStr">
+        <is>
+          <t>Halo (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G681" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H681" s="2" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="n">
+        <v>681</v>
+      </c>
+      <c r="B682" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C682" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5536-6920</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>🤝</t>
+        </is>
+      </c>
+      <c r="E682" s="2" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="F682" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G682" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H682" s="2" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
+        <v>682</v>
+      </c>
+      <c r="B683" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C683" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3536-4913</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>Mama Muhamad Alvino</t>
+        </is>
+      </c>
+      <c r="E683" s="2" t="inlineStr">
+        <is>
+          <t>00:02</t>
+        </is>
+      </c>
+      <c r="F683" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G683" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H683" s="2" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
+        <v>683</v>
+      </c>
+      <c r="B684" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C684" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2567-4138</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>❤️Naw Wul❤️</t>
+        </is>
+      </c>
+      <c r="E684" s="2" t="inlineStr">
+        <is>
+          <t>23:24</t>
+        </is>
+      </c>
+      <c r="F684" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G684" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H684" s="2" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
+        <v>684</v>
+      </c>
+      <c r="B685" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C685" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4198-1024</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>pak tris</t>
+        </is>
+      </c>
+      <c r="E685" s="2" t="inlineStr">
+        <is>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="F685" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G685" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H685" s="2" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
+        <v>685</v>
+      </c>
+      <c r="B686" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C686" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-2049-9978</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>Mu,min Jaebah</t>
+        </is>
+      </c>
+      <c r="E686" s="2" t="inlineStr">
+        <is>
+          <t>23:16</t>
+        </is>
+      </c>
+      <c r="F686" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G686" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H686" s="2" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="n">
+        <v>686</v>
+      </c>
+      <c r="B687" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C687" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1601-966</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>mahfudbasyar</t>
+        </is>
+      </c>
+      <c r="E687" s="2" t="inlineStr">
+        <is>
+          <t>22:59</t>
+        </is>
+      </c>
+      <c r="F687" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G687" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H687" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 55 of leads WA (16 Sept 2026), pass 700 total
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H687"/>
+  <dimension ref="A1:H701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -25410,6 +25410,510 @@
       </c>
       <c r="H687" s="2" t="inlineStr"/>
     </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
+        <v>687</v>
+      </c>
+      <c r="B688" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C688" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4984-3104</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>eliaspaledungeliyas</t>
+        </is>
+      </c>
+      <c r="E688" s="2" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="F688" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare berapa harganya</t>
+        </is>
+      </c>
+      <c r="G688" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H688" s="2" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
+        <v>688</v>
+      </c>
+      <c r="B689" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-2691-4829</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>🙏</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>21:29</t>
+        </is>
+      </c>
+      <c r="F689" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek hg</t>
+        </is>
+      </c>
+      <c r="G689" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H689" s="2" t="inlineStr"/>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
+        <v>689</v>
+      </c>
+      <c r="B690" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C690" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-5405-6412</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>edimanedi19</t>
+        </is>
+      </c>
+      <c r="E690" s="2" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="F690" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G690" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H690" s="2" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
+        <v>690</v>
+      </c>
+      <c r="B691" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8512-4935</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>E-Natsir</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="F691" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G691" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H691" s="2" t="inlineStr"/>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="B692" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C692" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3782-7887</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>borapullubenyamin</t>
+        </is>
+      </c>
+      <c r="E692" s="2" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="F692" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G692" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H692" s="2" t="inlineStr"/>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
+        <v>692</v>
+      </c>
+      <c r="B693" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6573-0551</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>Azhar</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="F693" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare utk motor ada nggak</t>
+        </is>
+      </c>
+      <c r="G693" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H693" s="2" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="n">
+        <v>693</v>
+      </c>
+      <c r="B694" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C694" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2319-2963</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>Subagiyo</t>
+        </is>
+      </c>
+      <c r="E694" s="2" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="F694" s="2" t="inlineStr">
+        <is>
+          <t>Harga nya berapa mas bro alo kak, Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G694" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H694" s="2" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="n">
+        <v>694</v>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9196-6699</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>happyfransisco76</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="F695" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G695" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H695" s="2" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="n">
+        <v>695</v>
+      </c>
+      <c r="B696" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9280-8977</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>Rini</t>
+        </is>
+      </c>
+      <c r="E696" s="2" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="F696" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G696" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H696" s="2" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
+        <v>696</v>
+      </c>
+      <c r="B697" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5473-0808</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>Harry</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="F697" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G697" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H697" s="2" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
+        <v>697</v>
+      </c>
+      <c r="B698" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4736-9382</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>Vitalis</t>
+        </is>
+      </c>
+      <c r="E698" s="2" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="F698" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G698" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H698" s="2" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
+        <v>698</v>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7333-3270</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>Risky Ridean</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G699" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
+        <v>699</v>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-0539-7323</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>Aryawati Kadek</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G700" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H700" s="2" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9818-4330</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>Halimbin</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="inlineStr">
+        <is>
+          <t>Mau tanya cofer mobil Expander berapa harganya pak (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G701" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 56 of leads WA (8, 15-16 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H701"/>
+  <dimension ref="A1:H715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -25914,6 +25914,517 @@
       </c>
       <c r="H701" s="2" t="inlineStr"/>
     </row>
+    <row r="702">
+      <c r="A702" s="2" t="n">
+        <v>701</v>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>+62 838-9089-0994</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>wfi (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="F702" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Bahanya tebel gak om.. yg perna saya beli tipis2 kena angin pada sobek jahitanya</t>
+        </is>
+      </c>
+      <c r="G702" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H702" s="2" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
+        <v>702</v>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>+62 897-8183-116</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>mazmos032</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa ya harga,</t>
+        </is>
+      </c>
+      <c r="G703" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="inlineStr"/>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
+        <v>703</v>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6438-3449</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>Teken Coy Nadeak</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="F704" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Buat WR-V 2025 Cek harga K</t>
+        </is>
+      </c>
+      <c r="G704" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H704" s="2" t="inlineStr"/>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="n">
+        <v>704</v>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5327-1358</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>Indrajaya</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>01:35</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G705" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="inlineStr"/>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
+        <v>705</v>
+      </c>
+      <c r="B706" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4098-3286</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>Hari sunarko 3 Dara wling</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G706" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H706" s="2" t="inlineStr"/>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="n">
+        <v>706</v>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1984-991</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>aj</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk Pajero Sport 2024</t>
+        </is>
+      </c>
+      <c r="G707" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="inlineStr"/>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="n">
+        <v>707</v>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4184-8507</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>bunda Husni</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="F708" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G708" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H708" s="2" t="inlineStr"/>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6235-7354</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>Sadiayana YG9CUO .JZ14MNZ</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga boosq</t>
+        </is>
+      </c>
+      <c r="G709" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="inlineStr"/>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
+        <v>709</v>
+      </c>
+      <c r="B710" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4582-4267</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>RUDISA</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="F710" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Itu berapa harga nya</t>
+        </is>
+      </c>
+      <c r="G710" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H710" s="2" t="inlineStr"/>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
+        <v>710</v>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5918-7960</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>Djaka</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="inlineStr">
+        <is>
+          <t>Harga utk Avanza kak (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G711" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="inlineStr"/>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
+        <v>711</v>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3857-9363</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>surpanaya26</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="F712" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G712" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H712" s="2" t="inlineStr"/>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
+        <v>712</v>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1390-0035</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>kunusabdul</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr"/>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
+        <v>713</v>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-4140-28221</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>Rizky Rejeki</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>Cover mobil grand max pick up brp (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G714" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="inlineStr"/>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-8366-161</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>Josh R (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil: byd atto 3
+Tipe Mobil: atto 3
+Tahun Mobil: 2026
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak! Ada?</t>
+        </is>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 57 of leads WA (12, 15-16 Sept 2026), pass 730 total
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H715"/>
+  <dimension ref="A1:H731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26425,6 +26425,582 @@
       </c>
       <c r="H715" s="2" t="inlineStr"/>
     </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
+        <v>715</v>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-5973-3818</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>Eful46</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Info harganya..</t>
+        </is>
+      </c>
+      <c r="G716" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="inlineStr"/>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
+        <v>716</v>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6604-4882</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>SRI SURYANI</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>21:12</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr"/>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
+        <v>717</v>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-9816-6162</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>cafe Lawang Abang/ pak D'</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga untuk Wuling confero 19</t>
+        </is>
+      </c>
+      <c r="G718" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="inlineStr"/>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="n">
+        <v>718</v>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-8486-4025</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>Nurul h</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Hrg nya brp</t>
+        </is>
+      </c>
+      <c r="G719" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="inlineStr"/>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="n">
+        <v>719</v>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3779-8798</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>PARKA iWyn</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>02:10</t>
+        </is>
+      </c>
+      <c r="F720" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G720" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H720" s="2" t="inlineStr"/>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1410-4450</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>Junaidin</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G721" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="inlineStr"/>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
+        <v>721</v>
+      </c>
+      <c r="B722" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-7413-5349</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>Sam (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E722" s="2" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="F722" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G722" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H722" s="2" t="inlineStr"/>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
+        <v>722</v>
+      </c>
+      <c r="B723" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3912-1945</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>Gun Ngo'uth</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G723" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H723" s="2" t="inlineStr"/>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
+        <v>723</v>
+      </c>
+      <c r="B724" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4044-3055</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>Wika Ampai Ikha</t>
+        </is>
+      </c>
+      <c r="E724" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="F724" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G724" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H724" s="2" t="inlineStr"/>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
+        <v>724</v>
+      </c>
+      <c r="B725" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6624-0779</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>kadekdodi83</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="F725" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga berapa</t>
+        </is>
+      </c>
+      <c r="G725" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H725" s="2" t="inlineStr"/>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
+        <v>725</v>
+      </c>
+      <c r="B726" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C726" s="2" t="inlineStr">
+        <is>
+          <t>+62 889-7067-2934</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>adolfbastian2179</t>
+        </is>
+      </c>
+      <c r="E726" s="2" t="inlineStr">
+        <is>
+          <t>23:49</t>
+        </is>
+      </c>
+      <c r="F726" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini? Mobil Honda Brio Rs .Thn 2018</t>
+        </is>
+      </c>
+      <c r="G726" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H726" s="2" t="inlineStr"/>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
+        <v>726</v>
+      </c>
+      <c r="B727" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-7431-5828</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>PRANOTO WENDY</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>00:16</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mazda CX5</t>
+        </is>
+      </c>
+      <c r="G727" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H727" s="2" t="inlineStr"/>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
+        <v>727</v>
+      </c>
+      <c r="B728" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3877-1155</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>Darma</t>
+        </is>
+      </c>
+      <c r="E728" s="2" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="F728" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G728" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H728" s="2" t="inlineStr"/>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
+        <v>728</v>
+      </c>
+      <c r="B729" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="inlineStr">
+        <is>
+          <t>+62 881-0375-30156</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>herusetiawan</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="F729" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk mobil hry prestige harga brp?</t>
+        </is>
+      </c>
+      <c r="G729" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="inlineStr"/>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
+        <v>729</v>
+      </c>
+      <c r="B730" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C730" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4298-1209</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>vpamikirang</t>
+        </is>
+      </c>
+      <c r="E730" s="2" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="F730" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G730" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H730" s="2" t="inlineStr"/>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
+        <v>730</v>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3405-8921</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>Ian 03-1</t>
+        </is>
+      </c>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="F731" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G731" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 58 of leads WA (15-16 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H731"/>
+  <dimension ref="A1:H746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -27001,6 +27001,546 @@
       </c>
       <c r="H731" s="2" t="inlineStr"/>
     </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
+        <v>731</v>
+      </c>
+      <c r="B732" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>+670 7369 0951</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>Otomotif (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E732" s="2" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="F732" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G732" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H732" s="2" t="inlineStr"/>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
+        <v>732</v>
+      </c>
+      <c r="B733" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8917-1219</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>Ghell_212</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>07:10</t>
+        </is>
+      </c>
+      <c r="F733" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G733" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="inlineStr"/>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
+        <v>733</v>
+      </c>
+      <c r="B734" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4301-4039</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>itjaid</t>
+        </is>
+      </c>
+      <c r="E734" s="2" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="F734" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G734" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H734" s="2" t="inlineStr"/>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="n">
+        <v>734</v>
+      </c>
+      <c r="B735" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-2102-0302</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>kurniawannia2802</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="F735" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G735" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="inlineStr"/>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
+        <v>735</v>
+      </c>
+      <c r="B736" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C736" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8828-4569</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>Suwardi</t>
+        </is>
+      </c>
+      <c r="E736" s="2" t="inlineStr">
+        <is>
+          <t>07:09</t>
+        </is>
+      </c>
+      <c r="F736" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G736" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H736" s="2" t="inlineStr"/>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
+        <v>736</v>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9760-3842</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>Ayah Akak</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="F737" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G737" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="inlineStr"/>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="n">
+        <v>737</v>
+      </c>
+      <c r="B738" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4528-354</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>noukekaunang2</t>
+        </is>
+      </c>
+      <c r="E738" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="F738" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G738" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H738" s="2" t="inlineStr"/>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="n">
+        <v>738</v>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1122-2532</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>rusmanjawada74</t>
+        </is>
+      </c>
+      <c r="E739" s="2" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="F739" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G739" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="inlineStr"/>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="n">
+        <v>739</v>
+      </c>
+      <c r="B740" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-7416-1793</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>Hayyun Worsnop</t>
+        </is>
+      </c>
+      <c r="E740" s="2" t="inlineStr">
+        <is>
+          <t>04:26</t>
+        </is>
+      </c>
+      <c r="F740" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G740" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H740" s="2" t="inlineStr"/>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
+        <v>740</v>
+      </c>
+      <c r="B741" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8044-1064</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>TATA SOFYET 🇧🇷🇧🇷</t>
+        </is>
+      </c>
+      <c r="E741" s="2" t="inlineStr">
+        <is>
+          <t>04:42</t>
+        </is>
+      </c>
+      <c r="F741" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G741" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
+        <v>741</v>
+      </c>
+      <c r="B742" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1141-0361</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>Maxxx</t>
+        </is>
+      </c>
+      <c r="E742" s="2" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="F742" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G742" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H742" s="2" t="inlineStr"/>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
+        <v>742</v>
+      </c>
+      <c r="B743" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5576-9792</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>Nining</t>
+        </is>
+      </c>
+      <c r="E743" s="2" t="inlineStr">
+        <is>
+          <t>05:49</t>
+        </is>
+      </c>
+      <c r="F743" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G743" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="inlineStr"/>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
+        <v>743</v>
+      </c>
+      <c r="B744" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C744" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9323-3636</t>
+        </is>
+      </c>
+      <c r="D744" s="2" t="inlineStr">
+        <is>
+          <t>DEdi Muksin</t>
+        </is>
+      </c>
+      <c r="E744" s="2" t="inlineStr">
+        <is>
+          <t>03:16</t>
+        </is>
+      </c>
+      <c r="F744" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G744" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H744" s="2" t="inlineStr"/>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="n">
+        <v>744</v>
+      </c>
+      <c r="B745" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C745" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3713-1419</t>
+        </is>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>ardha Lepa</t>
+        </is>
+      </c>
+      <c r="E745" s="2" t="inlineStr">
+        <is>
+          <t>20:49</t>
+        </is>
+      </c>
+      <c r="F745" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare,mobil grand Livina XV</t>
+        </is>
+      </c>
+      <c r="G745" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H745" s="2" t="inlineStr"/>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
+        <v>745</v>
+      </c>
+      <c r="B746" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C746" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-3887-7848</t>
+        </is>
+      </c>
+      <c r="D746" s="2" t="inlineStr">
+        <is>
+          <t>daisywidyasari71</t>
+        </is>
+      </c>
+      <c r="E746" s="2" t="inlineStr">
+        <is>
+          <t>22:14</t>
+        </is>
+      </c>
+      <c r="F746" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G746" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H746" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 59 of leads WA (2, 11, 14-15 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H746"/>
+  <dimension ref="A1:H760"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -27541,6 +27541,513 @@
       </c>
       <c r="H746" s="2" t="inlineStr"/>
     </row>
+    <row r="747">
+      <c r="A747" s="2" t="n">
+        <v>746</v>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-4094-6159</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>Jimmonk</t>
+        </is>
+      </c>
+      <c r="E747" s="2" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="F747" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G747" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H747" s="2" t="inlineStr"/>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="n">
+        <v>747</v>
+      </c>
+      <c r="B748" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1557-551</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>Reka Hardian</t>
+        </is>
+      </c>
+      <c r="E748" s="2" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="F748" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G748" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H748" s="2" t="inlineStr"/>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="B749" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4010-5277</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>Ellen S</t>
+        </is>
+      </c>
+      <c r="E749" s="2" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="F749" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G749" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H749" s="2" t="inlineStr"/>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
+        <v>749</v>
+      </c>
+      <c r="B750" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3408-129</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>TriesNo</t>
+        </is>
+      </c>
+      <c r="E750" s="2" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="F750" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G750" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H750" s="2" t="inlineStr"/>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="B751" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7959-9970</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>Bintang (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E751" s="2" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="F751" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G751" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H751" s="2" t="inlineStr"/>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="n">
+        <v>751</v>
+      </c>
+      <c r="B752" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C752" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3782-6565</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr"/>
+      <c r="E752" s="2" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="F752" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G752" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H752" s="2" t="inlineStr"/>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
+        <v>752</v>
+      </c>
+      <c r="B753" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C753" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-1333-0806</t>
+        </is>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>Dharie</t>
+        </is>
+      </c>
+      <c r="E753" s="2" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="F753" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brio brp</t>
+        </is>
+      </c>
+      <c r="G753" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H753" s="2" t="inlineStr"/>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
+        <v>753</v>
+      </c>
+      <c r="B754" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C754" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-309-699</t>
+        </is>
+      </c>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>Tommy</t>
+        </is>
+      </c>
+      <c r="E754" s="2" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="F754" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ini semi outdoor .yg utk outdoor ada</t>
+        </is>
+      </c>
+      <c r="G754" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H754" s="2" t="inlineStr"/>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
+        <v>754</v>
+      </c>
+      <c r="B755" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C755" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3553-7431</t>
+        </is>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>gibranangkringan</t>
+        </is>
+      </c>
+      <c r="E755" s="2" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="F755" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G755" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H755" s="2" t="inlineStr"/>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="B756" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4671-4199</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>Abdul Wakhid</t>
+        </is>
+      </c>
+      <c r="E756" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F756" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G756" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H756" s="2" t="inlineStr"/>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
+        <v>756</v>
+      </c>
+      <c r="B757" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C757" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1850-4601</t>
+        </is>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>Mamat Soengenep Madura</t>
+        </is>
+      </c>
+      <c r="E757" s="2" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="F757" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dikirim ulang 19:48)</t>
+        </is>
+      </c>
+      <c r="G757" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H757" s="2" t="inlineStr"/>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
+        <v>757</v>
+      </c>
+      <c r="B758" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C758" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6823-8057</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Novrizal</t>
+        </is>
+      </c>
+      <c r="E758" s="2" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="F758" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G758" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H758" s="2" t="inlineStr"/>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="B759" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-2349-6862</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>M45 3DY</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="F759" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G759" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H759" s="2" t="inlineStr"/>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="n">
+        <v>759</v>
+      </c>
+      <c r="B760" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C760" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7155-906</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>Herry Ariady</t>
+        </is>
+      </c>
+      <c r="E760" s="2" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="F760" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G760" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H760" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 60 of leads WA (6, 12-15 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H760"/>
+  <dimension ref="A1:H775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -28048,6 +28048,553 @@
       </c>
       <c r="H760" s="2" t="inlineStr"/>
     </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="B761" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-4720-2642</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>Edi icoet</t>
+        </is>
+      </c>
+      <c r="E761" s="2" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="F761" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga brapa</t>
+        </is>
+      </c>
+      <c r="G761" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H761" s="2" t="inlineStr"/>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
+        <v>761</v>
+      </c>
+      <c r="B762" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C762" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-665-042</t>
+        </is>
+      </c>
+      <c r="D762" s="2" t="inlineStr">
+        <is>
+          <t>Muhammad Idrus</t>
+        </is>
+      </c>
+      <c r="E762" s="2" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="F762" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G762" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H762" s="2" t="inlineStr"/>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
+        <v>762</v>
+      </c>
+      <c r="B763" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C763" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8774-1689</t>
+        </is>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>Oky setiawan</t>
+        </is>
+      </c>
+      <c r="E763" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="F763" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G763" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H763" s="2" t="inlineStr"/>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="B764" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C764" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9319-4391</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>nizam_fita</t>
+        </is>
+      </c>
+      <c r="E764" s="2" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="F764" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G764" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H764" s="2" t="inlineStr"/>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
+        <v>764</v>
+      </c>
+      <c r="B765" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9977-1464</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>SILVER QUIN.</t>
+        </is>
+      </c>
+      <c r="E765" s="2" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="F765" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek harga</t>
+        </is>
+      </c>
+      <c r="G765" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H765" s="2" t="inlineStr"/>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
+        <v>765</v>
+      </c>
+      <c r="B766" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-2817-8377</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>Bima Satriya</t>
+        </is>
+      </c>
+      <c r="E766" s="2" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="F766" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G766" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H766" s="2" t="inlineStr"/>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="n">
+        <v>766</v>
+      </c>
+      <c r="B767" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C767" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3906-7418</t>
+        </is>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>Made Tiding</t>
+        </is>
+      </c>
+      <c r="E767" s="2" t="inlineStr">
+        <is>
+          <t>03:32</t>
+        </is>
+      </c>
+      <c r="F767" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk jazz ada ngk</t>
+        </is>
+      </c>
+      <c r="G767" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H767" s="2" t="inlineStr"/>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
+        <v>767</v>
+      </c>
+      <c r="B768" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8832-5809</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>Aisya</t>
+        </is>
+      </c>
+      <c r="E768" s="2" t="inlineStr">
+        <is>
+          <t>02:38</t>
+        </is>
+      </c>
+      <c r="F768" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G768" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H768" s="2" t="inlineStr"/>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="B769" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3452-9011</t>
+        </is>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>Hartanta Silvi</t>
+        </is>
+      </c>
+      <c r="E769" s="2" t="inlineStr">
+        <is>
+          <t>10:23</t>
+        </is>
+      </c>
+      <c r="F769" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G769" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H769" s="2" t="inlineStr"/>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
+        <v>769</v>
+      </c>
+      <c r="B770" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C770" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-5677-9713</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>nyomansuweca62i</t>
+        </is>
+      </c>
+      <c r="E770" s="2" t="inlineStr">
+        <is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="F770" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G770" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H770" s="2" t="inlineStr"/>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="B771" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C771" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8833-5331</t>
+        </is>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>kabulwahyudi</t>
+        </is>
+      </c>
+      <c r="E771" s="2" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="F771" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G771" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H771" s="2" t="inlineStr"/>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="n">
+        <v>771</v>
+      </c>
+      <c r="B772" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3586-906</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>Charles Umboh (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E772" s="2" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="F772" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dikirim ulang)</t>
+        </is>
+      </c>
+      <c r="G772" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H772" s="2" t="inlineStr"/>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="n">
+        <v>772</v>
+      </c>
+      <c r="B773" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C773" s="2" t="inlineStr">
+        <is>
+          <t>+62 881-0277-83993</t>
+        </is>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>JOHN</t>
+        </is>
+      </c>
+      <c r="E773" s="2" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="F773" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare harga BRP dgnmodilexpander ada pak</t>
+        </is>
+      </c>
+      <c r="G773" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H773" s="2" t="inlineStr"/>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="B774" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C774" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1206-3609</t>
+        </is>
+      </c>
+      <c r="D774" s="2" t="inlineStr">
+        <is>
+          <t>Stevanus</t>
+        </is>
+      </c>
+      <c r="E774" s="2" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="F774" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G774" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H774" s="2" t="inlineStr"/>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="B775" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C775" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5098-335</t>
+        </is>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>Yulius</t>
+        </is>
+      </c>
+      <c r="E775" s="2" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="F775" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G775" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H775" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 61 of leads WA (1, 4, 14-15 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H775"/>
+  <dimension ref="A1:H789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -28595,6 +28595,510 @@
       </c>
       <c r="H775" s="2" t="inlineStr"/>
     </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
+        <v>775</v>
+      </c>
+      <c r="B776" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C776" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9298-173</t>
+        </is>
+      </c>
+      <c r="D776" s="2" t="inlineStr">
+        <is>
+          <t>salim m hasan</t>
+        </is>
+      </c>
+      <c r="E776" s="2" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F776" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G776" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H776" s="2" t="inlineStr"/>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="n">
+        <v>776</v>
+      </c>
+      <c r="B777" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="inlineStr">
+        <is>
+          <t>+62 888-0254-9836</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>Mahyadi</t>
+        </is>
+      </c>
+      <c r="E777" s="2" t="inlineStr">
+        <is>
+          <t>18:13</t>
+        </is>
+      </c>
+      <c r="F777" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G777" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H777" s="2" t="inlineStr"/>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
+        <v>777</v>
+      </c>
+      <c r="B778" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C778" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8788-2199</t>
+        </is>
+      </c>
+      <c r="D778" s="2" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="E778" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="F778" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G778" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H778" s="2" t="inlineStr"/>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="B779" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C779" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-6512-2524</t>
+        </is>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>Ida Bagus Widnyana</t>
+        </is>
+      </c>
+      <c r="E779" s="2" t="inlineStr">
+        <is>
+          <t>03:43</t>
+        </is>
+      </c>
+      <c r="F779" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G779" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H779" s="2" t="inlineStr"/>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
+        <v>779</v>
+      </c>
+      <c r="B780" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C780" s="2" t="inlineStr">
+        <is>
+          <t>+62 881-6700-312</t>
+        </is>
+      </c>
+      <c r="D780" s="2" t="inlineStr">
+        <is>
+          <t>ontoseno</t>
+        </is>
+      </c>
+      <c r="E780" s="2" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="F780" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G780" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H780" s="2" t="inlineStr"/>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
+        <v>780</v>
+      </c>
+      <c r="B781" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C781" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8985-8677</t>
+        </is>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>sahreza pahlepi</t>
+        </is>
+      </c>
+      <c r="E781" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F781" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G781" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H781" s="2" t="inlineStr"/>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="n">
+        <v>781</v>
+      </c>
+      <c r="B782" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C782" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2669-0934</t>
+        </is>
+      </c>
+      <c r="D782" s="2" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="E782" s="2" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="F782" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G782" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H782" s="2" t="inlineStr"/>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
+        <v>782</v>
+      </c>
+      <c r="B783" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C783" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-3822-1844</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>GT</t>
+        </is>
+      </c>
+      <c r="E783" s="2" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="F783" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G783" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H783" s="2" t="inlineStr"/>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="n">
+        <v>783</v>
+      </c>
+      <c r="B784" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9866-9866</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>H.Agus.S.Mudjarab,SH.</t>
+        </is>
+      </c>
+      <c r="E784" s="2" t="inlineStr">
+        <is>
+          <t>00:01</t>
+        </is>
+      </c>
+      <c r="F784" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G784" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H784" s="2" t="inlineStr"/>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
+        <v>784</v>
+      </c>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9702-8580</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>Hans Tenine</t>
+        </is>
+      </c>
+      <c r="E785" s="2" t="inlineStr">
+        <is>
+          <t>03:07</t>
+        </is>
+      </c>
+      <c r="F785" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G785" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H785" s="2" t="inlineStr"/>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="n">
+        <v>785</v>
+      </c>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4777-7583</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>Delta 2002</t>
+        </is>
+      </c>
+      <c r="E786" s="2" t="inlineStr">
+        <is>
+          <t>23:51</t>
+        </is>
+      </c>
+      <c r="F786" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G786" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H786" s="2" t="inlineStr"/>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
+        <v>786</v>
+      </c>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3744-1601</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>Made Sukana</t>
+        </is>
+      </c>
+      <c r="E787" s="2" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="F787" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G787" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H787" s="2" t="inlineStr"/>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="n">
+        <v>787</v>
+      </c>
+      <c r="B788" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-5303-8941</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>Nurhikma Auliya</t>
+        </is>
+      </c>
+      <c r="E788" s="2" t="inlineStr">
+        <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="F788" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G788" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H788" s="2" t="inlineStr"/>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
+        <v>788</v>
+      </c>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-0866-6429</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>D@v!d</t>
+        </is>
+      </c>
+      <c r="E789" s="2" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="F789" s="2" t="inlineStr">
+        <is>
+          <t>Hrga (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G789" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H789" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 62 of leads WA (4, 10, 12-15 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H789"/>
+  <dimension ref="A1:H804"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29099,6 +29099,546 @@
       </c>
       <c r="H789" s="2" t="inlineStr"/>
     </row>
+    <row r="790">
+      <c r="A790" s="2" t="n">
+        <v>789</v>
+      </c>
+      <c r="B790" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C790" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3354-9936</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>Gendut Supardi</t>
+        </is>
+      </c>
+      <c r="E790" s="2" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="F790" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare harga berapa</t>
+        </is>
+      </c>
+      <c r="G790" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H790" s="2" t="inlineStr"/>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="n">
+        <v>790</v>
+      </c>
+      <c r="B791" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C791" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4048-1865</t>
+        </is>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>Danankchan</t>
+        </is>
+      </c>
+      <c r="E791" s="2" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="F791" s="2" t="inlineStr">
+        <is>
+          <t>Untuk mobil kijang th 93 berapa ka (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G791" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H791" s="2" t="inlineStr"/>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="n">
+        <v>791</v>
+      </c>
+      <c r="B792" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C792" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2254-3418</t>
+        </is>
+      </c>
+      <c r="D792" s="2" t="inlineStr">
+        <is>
+          <t>Titus</t>
+        </is>
+      </c>
+      <c r="E792" s="2" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="F792" s="2" t="inlineStr">
+        <is>
+          <t>Sore mba, mau cari utk kijang innova 2008 mba (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G792" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H792" s="2" t="inlineStr"/>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="n">
+        <v>792</v>
+      </c>
+      <c r="B793" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C793" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9127-1344</t>
+        </is>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>fitrandahidayatullah</t>
+        </is>
+      </c>
+      <c r="E793" s="2" t="inlineStr">
+        <is>
+          <t>14:49</t>
+        </is>
+      </c>
+      <c r="F793" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G793" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H793" s="2" t="inlineStr"/>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="n">
+        <v>793</v>
+      </c>
+      <c r="B794" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C794" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3022-246</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>Sayogo</t>
+        </is>
+      </c>
+      <c r="E794" s="2" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="F794" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G794" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H794" s="2" t="inlineStr"/>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="n">
+        <v>794</v>
+      </c>
+      <c r="B795" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C795" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4046-3873</t>
+        </is>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>Anto</t>
+        </is>
+      </c>
+      <c r="E795" s="2" t="inlineStr">
+        <is>
+          <t>01:56</t>
+        </is>
+      </c>
+      <c r="F795" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Link toped plz</t>
+        </is>
+      </c>
+      <c r="G795" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H795" s="2" t="inlineStr"/>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="n">
+        <v>795</v>
+      </c>
+      <c r="B796" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C796" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2211-3494</t>
+        </is>
+      </c>
+      <c r="D796" s="2" t="inlineStr">
+        <is>
+          <t>💞Hana💞</t>
+        </is>
+      </c>
+      <c r="E796" s="2" t="inlineStr">
+        <is>
+          <t>16:19</t>
+        </is>
+      </c>
+      <c r="F796" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga brapa?</t>
+        </is>
+      </c>
+      <c r="G796" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H796" s="2" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="n">
+        <v>796</v>
+      </c>
+      <c r="B797" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C797" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6427-4065</t>
+        </is>
+      </c>
+      <c r="D797" s="2" t="inlineStr">
+        <is>
+          <t>Mr Sinabutar</t>
+        </is>
+      </c>
+      <c r="E797" s="2" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="F797" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare untuk Calya/Sigra</t>
+        </is>
+      </c>
+      <c r="G797" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H797" s="2" t="inlineStr"/>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="n">
+        <v>797</v>
+      </c>
+      <c r="B798" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-2796-0440</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>Herdian Fajar Ramathan</t>
+        </is>
+      </c>
+      <c r="E798" s="2" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="F798" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G798" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H798" s="2" t="inlineStr"/>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="n">
+        <v>798</v>
+      </c>
+      <c r="B799" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C799" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7431-9485</t>
+        </is>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>Aidatina</t>
+        </is>
+      </c>
+      <c r="E799" s="2" t="inlineStr">
+        <is>
+          <t>15:32</t>
+        </is>
+      </c>
+      <c r="F799" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G799" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H799" s="2" t="inlineStr"/>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="n">
+        <v>799</v>
+      </c>
+      <c r="B800" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C800" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8178-7899</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>HM.Rifai</t>
+        </is>
+      </c>
+      <c r="E800" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F800" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G800" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H800" s="2" t="inlineStr"/>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-3290-7581</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="E801" s="2" t="inlineStr">
+        <is>
+          <t>05:58</t>
+        </is>
+      </c>
+      <c r="F801" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G801" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H801" s="2" t="inlineStr"/>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="n">
+        <v>801</v>
+      </c>
+      <c r="B802" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C802" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-2819-007</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>Santoso_constantine</t>
+        </is>
+      </c>
+      <c r="E802" s="2" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="F802" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G802" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H802" s="2" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="n">
+        <v>802</v>
+      </c>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8199-7826</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>khairulamrizal846</t>
+        </is>
+      </c>
+      <c r="E803" s="2" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="F803" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G803" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H803" s="2" t="inlineStr"/>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="n">
+        <v>803</v>
+      </c>
+      <c r="B804" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C804" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2987-4667</t>
+        </is>
+      </c>
+      <c r="D804" s="2" t="inlineStr">
+        <is>
+          <t>Andy Wiryatama</t>
+        </is>
+      </c>
+      <c r="E804" s="2" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="F804" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga brpa kak?</t>
+        </is>
+      </c>
+      <c r="G804" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H804" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 63 of leads WA (12-14 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H804"/>
+  <dimension ref="A1:H820"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -29639,6 +29639,589 @@
       </c>
       <c r="H804" s="2" t="inlineStr"/>
     </row>
+    <row r="805">
+      <c r="A805" s="2" t="n">
+        <v>804</v>
+      </c>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-2391-7624</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>Nurhadi Didi</t>
+        </is>
+      </c>
+      <c r="E805" s="2" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="F805" s="2" t="inlineStr">
+        <is>
+          <t>Dimana lokasi toko nya mba Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G805" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H805" s="2" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="n">
+        <v>805</v>
+      </c>
+      <c r="B806" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-9921-9782</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>Echa Salon</t>
+        </is>
+      </c>
+      <c r="E806" s="2" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="F806" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G806" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H806" s="2" t="inlineStr"/>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="n">
+        <v>806</v>
+      </c>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-0021-1208</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>Nining Widowati</t>
+        </is>
+      </c>
+      <c r="E807" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="F807" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G807" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H807" s="2" t="inlineStr"/>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="n">
+        <v>807</v>
+      </c>
+      <c r="B808" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7803-8511</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>Mariana Girsang</t>
+        </is>
+      </c>
+      <c r="E808" s="2" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="F808" s="2" t="inlineStr">
+        <is>
+          <t>Mau tanya harga nya berapa (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G808" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H808" s="2" t="inlineStr"/>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="n">
+        <v>808</v>
+      </c>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-3870-7963</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>Soni</t>
+        </is>
+      </c>
+      <c r="E809" s="2" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="F809" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G809" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H809" s="2" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
+        <v>809</v>
+      </c>
+      <c r="B810" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C810" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-8935-5599</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>Heri Bertus</t>
+        </is>
+      </c>
+      <c r="E810" s="2" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="F810" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada untuk ayla</t>
+        </is>
+      </c>
+      <c r="G810" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H810" s="2" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
+        <v>810</v>
+      </c>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8617-0510</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>Indra ctb Jakpus</t>
+        </is>
+      </c>
+      <c r="E811" s="2" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="F811" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G811" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H811" s="2" t="inlineStr"/>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="n">
+        <v>811</v>
+      </c>
+      <c r="B812" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C812" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-8006-64286</t>
+        </is>
+      </c>
+      <c r="D812" s="2" t="inlineStr">
+        <is>
+          <t>Hj Heriana</t>
+        </is>
+      </c>
+      <c r="E812" s="2" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="F812" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G812" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H812" s="2" t="inlineStr"/>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="n">
+        <v>812</v>
+      </c>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9374-8354</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>mbok sri cmplok bdg</t>
+        </is>
+      </c>
+      <c r="E813" s="2" t="inlineStr">
+        <is>
+          <t>05:50</t>
+        </is>
+      </c>
+      <c r="F813" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Mf kak klou untuk Inova rebon. Cek</t>
+        </is>
+      </c>
+      <c r="G813" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H813" s="2" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="n">
+        <v>813</v>
+      </c>
+      <c r="B814" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C814" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-8422-8835</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E814" s="2" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="F814" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G814" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H814" s="2" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="n">
+        <v>814</v>
+      </c>
+      <c r="B815" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C815" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-5238-9588</t>
+        </is>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>Alithadira</t>
+        </is>
+      </c>
+      <c r="E815" s="2" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="F815" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G815" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H815" s="2" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="n">
+        <v>815</v>
+      </c>
+      <c r="B816" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C816" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3786-0189</t>
+        </is>
+      </c>
+      <c r="D816" s="2" t="inlineStr">
+        <is>
+          <t>Sunjsun</t>
+        </is>
+      </c>
+      <c r="E816" s="2" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="F816" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G816" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H816" s="2" t="inlineStr"/>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="n">
+        <v>816</v>
+      </c>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-2791-8424</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>arodi</t>
+        </is>
+      </c>
+      <c r="E817" s="2" t="inlineStr">
+        <is>
+          <t>06:07</t>
+        </is>
+      </c>
+      <c r="F817" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G817" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H817" s="2" t="inlineStr"/>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="n">
+        <v>817</v>
+      </c>
+      <c r="B818" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C818" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-3026-944</t>
+        </is>
+      </c>
+      <c r="D818" s="2" t="inlineStr">
+        <is>
+          <t>Afrizal</t>
+        </is>
+      </c>
+      <c r="E818" s="2" t="inlineStr">
+        <is>
+          <t>08:58</t>
+        </is>
+      </c>
+      <c r="F818" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G818" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H818" s="2" t="inlineStr"/>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="n">
+        <v>818</v>
+      </c>
+      <c r="B819" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C819" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-7516-3276</t>
+        </is>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>Bunda Gio❤️❤️❤️</t>
+        </is>
+      </c>
+      <c r="E819" s="2" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="F819" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Bole cek harga</t>
+        </is>
+      </c>
+      <c r="G819" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H819" s="2" t="inlineStr"/>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="n">
+        <v>819</v>
+      </c>
+      <c r="B820" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C820" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4381-3579</t>
+        </is>
+      </c>
+      <c r="D820" s="2" t="inlineStr">
+        <is>
+          <t>Haris Daeng Nappa</t>
+        </is>
+      </c>
+      <c r="E820" s="2" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="F820" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Bisa COD</t>
+        </is>
+      </c>
+      <c r="G820" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H820" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 64 of leads WA (12-13 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H820"/>
+  <dimension ref="A1:H836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -30222,6 +30222,582 @@
       </c>
       <c r="H820" s="2" t="inlineStr"/>
     </row>
+    <row r="821">
+      <c r="A821" s="2" t="n">
+        <v>820</v>
+      </c>
+      <c r="B821" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C821" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9937-1990</t>
+        </is>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>Dede</t>
+        </is>
+      </c>
+      <c r="E821" s="2" t="inlineStr">
+        <is>
+          <t>06:16</t>
+        </is>
+      </c>
+      <c r="F821" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G821" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H821" s="2" t="inlineStr"/>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="n">
+        <v>821</v>
+      </c>
+      <c r="B822" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C822" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-8657-7335</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>Cliff Jonathan</t>
+        </is>
+      </c>
+      <c r="E822" s="2" t="inlineStr">
+        <is>
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="F822" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G822" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H822" s="2" t="inlineStr"/>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="n">
+        <v>822</v>
+      </c>
+      <c r="B823" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="inlineStr">
+        <is>
+          <t>+62 889-7118-0500</t>
+        </is>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>jelabut</t>
+        </is>
+      </c>
+      <c r="E823" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="F823" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G823" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H823" s="2" t="inlineStr"/>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="n">
+        <v>823</v>
+      </c>
+      <c r="B824" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C824" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3729-5998</t>
+        </is>
+      </c>
+      <c r="D824" s="2" t="inlineStr">
+        <is>
+          <t>Sevi oktores</t>
+        </is>
+      </c>
+      <c r="E824" s="2" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="F824" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G824" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H824" s="2" t="inlineStr"/>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="n">
+        <v>824</v>
+      </c>
+      <c r="B825" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4714-1531</t>
+        </is>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>Hotmian</t>
+        </is>
+      </c>
+      <c r="E825" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="F825" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G825" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H825" s="2" t="inlineStr"/>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="n">
+        <v>825</v>
+      </c>
+      <c r="B826" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C826" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2557-6198</t>
+        </is>
+      </c>
+      <c r="D826" s="2" t="inlineStr">
+        <is>
+          <t>Sugiarti</t>
+        </is>
+      </c>
+      <c r="E826" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="F826" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G826" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H826" s="2" t="inlineStr"/>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="n">
+        <v>826</v>
+      </c>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-6688-1010</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>WW</t>
+        </is>
+      </c>
+      <c r="E827" s="2" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="F827" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G827" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="inlineStr"/>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="n">
+        <v>827</v>
+      </c>
+      <c r="B828" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-4894-353</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>Ary Sulistiyowaty</t>
+        </is>
+      </c>
+      <c r="E828" s="2" t="inlineStr">
+        <is>
+          <t>08:07</t>
+        </is>
+      </c>
+      <c r="F828" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G828" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H828" s="2" t="inlineStr"/>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="n">
+        <v>828</v>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-9131-921</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>Marcelo Iskandar Chang</t>
+        </is>
+      </c>
+      <c r="E829" s="2" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="F829" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G829" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="inlineStr"/>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="n">
+        <v>829</v>
+      </c>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7708-0711</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>Soemardi</t>
+        </is>
+      </c>
+      <c r="E830" s="2" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="F830" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G830" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H830" s="2" t="inlineStr"/>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="n">
+        <v>830</v>
+      </c>
+      <c r="B831" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C831" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3707-4336</t>
+        </is>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>Dwi Harsono</t>
+        </is>
+      </c>
+      <c r="E831" s="2" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="F831" s="2" t="inlineStr">
+        <is>
+          <t>Hrg cover selimut carry futura minibus (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G831" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H831" s="2" t="inlineStr"/>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="n">
+        <v>831</v>
+      </c>
+      <c r="B832" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C832" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8873-4999</t>
+        </is>
+      </c>
+      <c r="D832" s="2" t="inlineStr">
+        <is>
+          <t>tulussitorus</t>
+        </is>
+      </c>
+      <c r="E832" s="2" t="inlineStr">
+        <is>
+          <t>04:16</t>
+        </is>
+      </c>
+      <c r="F832" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G832" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H832" s="2" t="inlineStr"/>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="n">
+        <v>832</v>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-5555-0232</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>Mud Mada</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="inlineStr">
+        <is>
+          <t>06:49</t>
+        </is>
+      </c>
+      <c r="F833" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G833" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H833" s="2" t="inlineStr"/>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="n">
+        <v>833</v>
+      </c>
+      <c r="B834" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3559-0890</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>Procurement Team Bagasanti dan Luxlo (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E834" s="2" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="F834" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Can I get more info on this?</t>
+        </is>
+      </c>
+      <c r="G834" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H834" s="2" t="inlineStr"/>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="n">
+        <v>834</v>
+      </c>
+      <c r="B835" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9562-4799</t>
+        </is>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>Rezeki Agung</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="inlineStr">
+        <is>
+          <t>06:54</t>
+        </is>
+      </c>
+      <c r="F835" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G835" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H835" s="2" t="inlineStr"/>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="n">
+        <v>835</v>
+      </c>
+      <c r="B836" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C836" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6179-8355</t>
+        </is>
+      </c>
+      <c r="D836" s="2" t="inlineStr">
+        <is>
+          <t>Las</t>
+        </is>
+      </c>
+      <c r="E836" s="2" t="inlineStr">
+        <is>
+          <t>07:53</t>
+        </is>
+      </c>
+      <c r="F836" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G836" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H836" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 65 of leads WA (6, 12-14 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H836"/>
+  <dimension ref="A1:H851"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -30798,6 +30798,546 @@
       </c>
       <c r="H836" s="2" t="inlineStr"/>
     </row>
+    <row r="837">
+      <c r="A837" s="2" t="n">
+        <v>836</v>
+      </c>
+      <c r="B837" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C837" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3921-0496</t>
+        </is>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>Emy Fangidae</t>
+        </is>
+      </c>
+      <c r="E837" s="2" t="inlineStr">
+        <is>
+          <t>00:04</t>
+        </is>
+      </c>
+      <c r="F837" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G837" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H837" s="2" t="inlineStr"/>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="n">
+        <v>837</v>
+      </c>
+      <c r="B838" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C838" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-5521-7980</t>
+        </is>
+      </c>
+      <c r="D838" s="2" t="inlineStr">
+        <is>
+          <t>Gogoh Sulaksono</t>
+        </is>
+      </c>
+      <c r="E838" s="2" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="F838" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G838" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H838" s="2" t="inlineStr"/>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="n">
+        <v>838</v>
+      </c>
+      <c r="B839" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C839" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3628-9493</t>
+        </is>
+      </c>
+      <c r="D839" s="2" t="inlineStr">
+        <is>
+          <t>urbanus</t>
+        </is>
+      </c>
+      <c r="E839" s="2" t="inlineStr">
+        <is>
+          <t>06:18</t>
+        </is>
+      </c>
+      <c r="F839" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G839" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H839" s="2" t="inlineStr"/>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="n">
+        <v>839</v>
+      </c>
+      <c r="B840" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C840" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2345-7550</t>
+        </is>
+      </c>
+      <c r="D840" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E840" s="2" t="inlineStr">
+        <is>
+          <t>02:33</t>
+        </is>
+      </c>
+      <c r="F840" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G840" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H840" s="2" t="inlineStr"/>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="n">
+        <v>840</v>
+      </c>
+      <c r="B841" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C841" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4268-7107</t>
+        </is>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E841" s="2" t="inlineStr">
+        <is>
+          <t>02:26</t>
+        </is>
+      </c>
+      <c r="F841" s="2" t="inlineStr">
+        <is>
+          <t>Halbo kak, saya ingin berapa duit Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G841" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H841" s="2" t="inlineStr"/>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="n">
+        <v>841</v>
+      </c>
+      <c r="B842" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C842" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-0840-9108</t>
+        </is>
+      </c>
+      <c r="D842" s="2" t="inlineStr">
+        <is>
+          <t>Ni luh Suartami</t>
+        </is>
+      </c>
+      <c r="E842" s="2" t="inlineStr">
+        <is>
+          <t>21:57</t>
+        </is>
+      </c>
+      <c r="F842" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G842" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H842" s="2" t="inlineStr"/>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="n">
+        <v>842</v>
+      </c>
+      <c r="B843" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C843" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-4772-6915</t>
+        </is>
+      </c>
+      <c r="D843" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E843" s="2" t="inlineStr">
+        <is>
+          <t>01:19</t>
+        </is>
+      </c>
+      <c r="F843" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G843" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H843" s="2" t="inlineStr"/>
+    </row>
+    <row r="844">
+      <c r="A844" s="2" t="n">
+        <v>843</v>
+      </c>
+      <c r="B844" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C844" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-4981-6725</t>
+        </is>
+      </c>
+      <c r="D844" s="2" t="inlineStr">
+        <is>
+          <t>hasim</t>
+        </is>
+      </c>
+      <c r="E844" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="F844" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G844" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H844" s="2" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" s="2" t="n">
+        <v>844</v>
+      </c>
+      <c r="B845" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C845" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5466-4575</t>
+        </is>
+      </c>
+      <c r="D845" s="2" t="inlineStr">
+        <is>
+          <t>~A_R</t>
+        </is>
+      </c>
+      <c r="E845" s="2" t="inlineStr">
+        <is>
+          <t>04:52</t>
+        </is>
+      </c>
+      <c r="F845" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G845" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H845" s="2" t="inlineStr"/>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="n">
+        <v>845</v>
+      </c>
+      <c r="B846" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C846" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2978-5830</t>
+        </is>
+      </c>
+      <c r="D846" s="2" t="inlineStr">
+        <is>
+          <t>Anward</t>
+        </is>
+      </c>
+      <c r="E846" s="2" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="F846" s="2" t="inlineStr">
+        <is>
+          <t>Untuk luxio (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G846" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H846" s="2" t="inlineStr"/>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="n">
+        <v>846</v>
+      </c>
+      <c r="B847" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C847" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1858-8033</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>Elmar A. Kono</t>
+        </is>
+      </c>
+      <c r="E847" s="2" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="F847" s="2" t="inlineStr">
+        <is>
+          <t>Hello! Brp harga cover utk mercy 300E W124 THN 1992 (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G847" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H847" s="2" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="n">
+        <v>847</v>
+      </c>
+      <c r="B848" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C848" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2347-0380</t>
+        </is>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>ISTIE QOMAH</t>
+        </is>
+      </c>
+      <c r="E848" s="2" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="F848" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G848" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H848" s="2" t="inlineStr"/>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="n">
+        <v>848</v>
+      </c>
+      <c r="B849" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C849" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9490-3403</t>
+        </is>
+      </c>
+      <c r="D849" s="2" t="inlineStr">
+        <is>
+          <t>julpan pasarib</t>
+        </is>
+      </c>
+      <c r="E849" s="2" t="inlineStr">
+        <is>
+          <t>17:29</t>
+        </is>
+      </c>
+      <c r="F849" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G849" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H849" s="2" t="inlineStr"/>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="n">
+        <v>849</v>
+      </c>
+      <c r="B850" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C850" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-3361-2229</t>
+        </is>
+      </c>
+      <c r="D850" s="2" t="inlineStr">
+        <is>
+          <t>kalian gak tau</t>
+        </is>
+      </c>
+      <c r="E850" s="2" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="F850" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G850" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H850" s="2" t="inlineStr"/>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="n">
+        <v>850</v>
+      </c>
+      <c r="B851" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C851" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3869-9746</t>
+        </is>
+      </c>
+      <c r="D851" s="2" t="inlineStr">
+        <is>
+          <t>Ayuera</t>
+        </is>
+      </c>
+      <c r="E851" s="2" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="F851" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G851" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H851" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 66 of leads WA (1, 11-12 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H851"/>
+  <dimension ref="A1:H866"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -31338,6 +31338,574 @@
       </c>
       <c r="H851" s="2" t="inlineStr"/>
     </row>
+    <row r="852">
+      <c r="A852" s="2" t="n">
+        <v>851</v>
+      </c>
+      <c r="B852" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C852" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3698-7574</t>
+        </is>
+      </c>
+      <c r="D852" s="2" t="inlineStr">
+        <is>
+          <t>150_1970012022025211003</t>
+        </is>
+      </c>
+      <c r="E852" s="2" t="inlineStr">
+        <is>
+          <t>20:09</t>
+        </is>
+      </c>
+      <c r="F852" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare UNDERCOVER XENIA 2012</t>
+        </is>
+      </c>
+      <c r="G852" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H852" s="2" t="inlineStr"/>
+    </row>
+    <row r="853">
+      <c r="A853" s="2" t="n">
+        <v>852</v>
+      </c>
+      <c r="B853" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C853" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-2930-7398</t>
+        </is>
+      </c>
+      <c r="D853" s="2" t="inlineStr">
+        <is>
+          <t>Agusiki</t>
+        </is>
+      </c>
+      <c r="E853" s="2" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="F853" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utk megaa caryy ada mba</t>
+        </is>
+      </c>
+      <c r="G853" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H853" s="2" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="n">
+        <v>853</v>
+      </c>
+      <c r="B854" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C854" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4544-3303</t>
+        </is>
+      </c>
+      <c r="D854" s="2" t="inlineStr">
+        <is>
+          <t>Tri Laniri</t>
+        </is>
+      </c>
+      <c r="E854" s="2" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="F854" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G854" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H854" s="2" t="inlineStr"/>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="n">
+        <v>854</v>
+      </c>
+      <c r="B855" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C855" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2106-6836</t>
+        </is>
+      </c>
+      <c r="D855" s="2" t="inlineStr">
+        <is>
+          <t>Prasetia</t>
+        </is>
+      </c>
+      <c r="E855" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="F855" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G855" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H855" s="2" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="n">
+        <v>855</v>
+      </c>
+      <c r="B856" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C856" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5533-002</t>
+        </is>
+      </c>
+      <c r="D856" s="2" t="inlineStr">
+        <is>
+          <t>YUNALDI</t>
+        </is>
+      </c>
+      <c r="E856" s="2" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="F856" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Info harganya.</t>
+        </is>
+      </c>
+      <c r="G856" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H856" s="2" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="n">
+        <v>856</v>
+      </c>
+      <c r="B857" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C857" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9641-0393</t>
+        </is>
+      </c>
+      <c r="D857" s="2" t="inlineStr">
+        <is>
+          <t>jafarsalii091</t>
+        </is>
+      </c>
+      <c r="E857" s="2" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="F857" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G857" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H857" s="2" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" s="2" t="n">
+        <v>857</v>
+      </c>
+      <c r="B858" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C858" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-7842-9072</t>
+        </is>
+      </c>
+      <c r="D858" s="2" t="inlineStr">
+        <is>
+          <t>yayunalfianto</t>
+        </is>
+      </c>
+      <c r="E858" s="2" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="F858" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G858" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H858" s="2" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="n">
+        <v>858</v>
+      </c>
+      <c r="B859" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C859" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-3655-7558</t>
+        </is>
+      </c>
+      <c r="D859" s="2" t="inlineStr">
+        <is>
+          <t>デニール</t>
+        </is>
+      </c>
+      <c r="E859" s="2" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="F859" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G859" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H859" s="2" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" s="2" t="n">
+        <v>859</v>
+      </c>
+      <c r="B860" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C860" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-7867-7645</t>
+        </is>
+      </c>
+      <c r="D860" s="2" t="inlineStr">
+        <is>
+          <t>Zakiyan</t>
+        </is>
+      </c>
+      <c r="E860" s="2" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="F860" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G860" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H860" s="2" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" s="2" t="n">
+        <v>860</v>
+      </c>
+      <c r="B861" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C861" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4023-5484</t>
+        </is>
+      </c>
+      <c r="D861" s="2" t="inlineStr">
+        <is>
+          <t>Acc</t>
+        </is>
+      </c>
+      <c r="E861" s="2" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="F861" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G861" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H861" s="2" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
+        <v>861</v>
+      </c>
+      <c r="B862" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C862" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-4977-9314</t>
+        </is>
+      </c>
+      <c r="D862" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E862" s="2" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="F862" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G862" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H862" s="2" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="n">
+        <v>862</v>
+      </c>
+      <c r="B863" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C863" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-2571-4276</t>
+        </is>
+      </c>
+      <c r="D863" s="2" t="inlineStr">
+        <is>
+          <t>Adit</t>
+        </is>
+      </c>
+      <c r="E863" s="2" t="inlineStr">
+        <is>
+          <t>05:56</t>
+        </is>
+      </c>
+      <c r="F863" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G863" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H863" s="2" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="n">
+        <v>863</v>
+      </c>
+      <c r="B864" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C864" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-3758-5441</t>
+        </is>
+      </c>
+      <c r="D864" s="2" t="inlineStr">
+        <is>
+          <t>Amar Furnitur</t>
+        </is>
+      </c>
+      <c r="E864" s="2" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="F864" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G864" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H864" s="2" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="n">
+        <v>864</v>
+      </c>
+      <c r="B865" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C865" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4238-0832</t>
+        </is>
+      </c>
+      <c r="D865" s="2" t="inlineStr">
+        <is>
+          <t>Andi Hasmawati</t>
+        </is>
+      </c>
+      <c r="E865" s="2" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="F865" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak!</t>
+        </is>
+      </c>
+      <c r="G865" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H865" s="2" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" s="2" t="n">
+        <v>865</v>
+      </c>
+      <c r="B866" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C866" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6019-4891</t>
+        </is>
+      </c>
+      <c r="D866" s="2" t="inlineStr">
+        <is>
+          <t>Hendry</t>
+        </is>
+      </c>
+      <c r="E866" s="2" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="F866" s="2" t="inlineStr">
+        <is>
+          <t>Halo Admin Undercover! Saya mau order Cover Mobil.
+Merk Mobil:
+Tipe Mobil:
+Tahun Mobil:
+Nama Penerima:
+Alamat Penerima:
+Tipe Cover: (Reguler/Exclusive)
+Tolong bantu cek harga dan stocknya ya Kak! Hailo</t>
+        </is>
+      </c>
+      <c r="G866" s="2" t="inlineStr">
+        <is>
+          <t>Landing Page V2</t>
+        </is>
+      </c>
+      <c r="H866" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 67 of leads WA (19-21 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H866"/>
+  <dimension ref="A1:H879"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -31906,6 +31906,474 @@
       </c>
       <c r="H866" s="2" t="inlineStr"/>
     </row>
+    <row r="867">
+      <c r="A867" s="2" t="n">
+        <v>866</v>
+      </c>
+      <c r="B867" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C867" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5287-7889</t>
+        </is>
+      </c>
+      <c r="D867" s="2" t="inlineStr">
+        <is>
+          <t>lianafalia74</t>
+        </is>
+      </c>
+      <c r="E867" s="2" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="F867" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G867" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H867" s="2" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="n">
+        <v>867</v>
+      </c>
+      <c r="B868" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C868" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-8383-4972</t>
+        </is>
+      </c>
+      <c r="D868" s="2" t="inlineStr">
+        <is>
+          <t>Tbn (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E868" s="2" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="F868" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G868" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H868" s="2" t="inlineStr"/>
+    </row>
+    <row r="869">
+      <c r="A869" s="2" t="n">
+        <v>868</v>
+      </c>
+      <c r="B869" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C869" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-8865-2340</t>
+        </is>
+      </c>
+      <c r="D869" s="2" t="inlineStr">
+        <is>
+          <t>lainnya (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E869" s="2" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="F869" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G869" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H869" s="2" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" s="2" t="n">
+        <v>869</v>
+      </c>
+      <c r="B870" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C870" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4112-6880</t>
+        </is>
+      </c>
+      <c r="D870" s="2" t="inlineStr">
+        <is>
+          <t>Jumadi Ati</t>
+        </is>
+      </c>
+      <c r="E870" s="2" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="F870" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G870" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H870" s="2" t="inlineStr"/>
+    </row>
+    <row r="871">
+      <c r="A871" s="2" t="n">
+        <v>870</v>
+      </c>
+      <c r="B871" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C871" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-6057-4688</t>
+        </is>
+      </c>
+      <c r="D871" s="2" t="inlineStr">
+        <is>
+          <t>TBN</t>
+        </is>
+      </c>
+      <c r="E871" s="2" t="inlineStr">
+        <is>
+          <t>14:09</t>
+        </is>
+      </c>
+      <c r="F871" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G871" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H871" s="2" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" s="2" t="n">
+        <v>871</v>
+      </c>
+      <c r="B872" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C872" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-7415-6087</t>
+        </is>
+      </c>
+      <c r="D872" s="2" t="inlineStr">
+        <is>
+          <t>Radithia</t>
+        </is>
+      </c>
+      <c r="E872" s="2" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="F872" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G872" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H872" s="2" t="inlineStr"/>
+    </row>
+    <row r="873">
+      <c r="A873" s="2" t="n">
+        <v>872</v>
+      </c>
+      <c r="B873" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C873" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4635-0101</t>
+        </is>
+      </c>
+      <c r="D873" s="2" t="inlineStr">
+        <is>
+          <t>Kurinati</t>
+        </is>
+      </c>
+      <c r="E873" s="2" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="F873" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga utk type kend honda brio</t>
+        </is>
+      </c>
+      <c r="G873" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H873" s="2" t="inlineStr"/>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="n">
+        <v>873</v>
+      </c>
+      <c r="B874" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C874" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9380-3380</t>
+        </is>
+      </c>
+      <c r="D874" s="2" t="inlineStr">
+        <is>
+          <t>djoasinhie</t>
+        </is>
+      </c>
+      <c r="E874" s="2" t="inlineStr">
+        <is>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="F874" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Harga</t>
+        </is>
+      </c>
+      <c r="G874" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H874" s="2" t="inlineStr"/>
+    </row>
+    <row r="875">
+      <c r="A875" s="2" t="n">
+        <v>874</v>
+      </c>
+      <c r="B875" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C875" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9070-3602</t>
+        </is>
+      </c>
+      <c r="D875" s="2" t="inlineStr">
+        <is>
+          <t>Senoajie</t>
+        </is>
+      </c>
+      <c r="E875" s="2" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="F875" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G875" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H875" s="2" t="inlineStr"/>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="n">
+        <v>875</v>
+      </c>
+      <c r="B876" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C876" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8575-2300</t>
+        </is>
+      </c>
+      <c r="D876" s="2" t="inlineStr">
+        <is>
+          <t>Jon Barita</t>
+        </is>
+      </c>
+      <c r="E876" s="2" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="F876" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G876" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H876" s="2" t="inlineStr"/>
+    </row>
+    <row r="877">
+      <c r="A877" s="2" t="n">
+        <v>876</v>
+      </c>
+      <c r="B877" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C877" s="2" t="inlineStr">
+        <is>
+          <t>+62 816-393-266</t>
+        </is>
+      </c>
+      <c r="D877" s="2" t="inlineStr">
+        <is>
+          <t>Sa Ryoko</t>
+        </is>
+      </c>
+      <c r="E877" s="2" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="F877" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G877" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H877" s="2" t="inlineStr"/>
+    </row>
+    <row r="878">
+      <c r="A878" s="2" t="n">
+        <v>877</v>
+      </c>
+      <c r="B878" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C878" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5699-2789</t>
+        </is>
+      </c>
+      <c r="D878" s="2" t="inlineStr">
+        <is>
+          <t>rahmatmokogonta</t>
+        </is>
+      </c>
+      <c r="E878" s="2" t="inlineStr">
+        <is>
+          <t>10:23</t>
+        </is>
+      </c>
+      <c r="F878" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G878" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H878" s="2" t="inlineStr"/>
+    </row>
+    <row r="879">
+      <c r="A879" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="B879" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C879" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4054-1848</t>
+        </is>
+      </c>
+      <c r="D879" s="2" t="inlineStr">
+        <is>
+          <t>wiwinalansar</t>
+        </is>
+      </c>
+      <c r="E879" s="2" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="F879" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G879" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H879" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 67 of leads WA (10, 15, 20-21 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H879"/>
+  <dimension ref="A1:H895"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -32374,6 +32374,578 @@
       </c>
       <c r="H879" s="2" t="inlineStr"/>
     </row>
+    <row r="880">
+      <c r="A880" s="2" t="n">
+        <v>879</v>
+      </c>
+      <c r="B880" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C880" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5462-2284</t>
+        </is>
+      </c>
+      <c r="D880" s="2" t="inlineStr">
+        <is>
+          <t>Nanu</t>
+        </is>
+      </c>
+      <c r="E880" s="2" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="F880" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G880" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H880" s="2" t="inlineStr"/>
+    </row>
+    <row r="881">
+      <c r="A881" s="2" t="n">
+        <v>880</v>
+      </c>
+      <c r="B881" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C881" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4600-4117</t>
+        </is>
+      </c>
+      <c r="D881" s="2" t="inlineStr">
+        <is>
+          <t>Nona Mura ❤️</t>
+        </is>
+      </c>
+      <c r="E881" s="2" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="F881" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G881" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H881" s="2" t="inlineStr"/>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="n">
+        <v>881</v>
+      </c>
+      <c r="B882" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C882" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5253-5782</t>
+        </is>
+      </c>
+      <c r="D882" s="2" t="inlineStr">
+        <is>
+          <t>Rarafi09💙</t>
+        </is>
+      </c>
+      <c r="E882" s="2" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F882" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G882" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H882" s="2" t="inlineStr"/>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="n">
+        <v>882</v>
+      </c>
+      <c r="B883" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C883" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-2818-9350</t>
+        </is>
+      </c>
+      <c r="D883" s="2" t="inlineStr">
+        <is>
+          <t>Suriani Malaka</t>
+        </is>
+      </c>
+      <c r="E883" s="2" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="F883" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare cek harga</t>
+        </is>
+      </c>
+      <c r="G883" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H883" s="2" t="inlineStr"/>
+    </row>
+    <row r="884">
+      <c r="A884" s="2" t="n">
+        <v>883</v>
+      </c>
+      <c r="B884" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C884" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-6239-0701</t>
+        </is>
+      </c>
+      <c r="D884" s="2" t="inlineStr">
+        <is>
+          <t>rzher (akun bisnis)</t>
+        </is>
+      </c>
+      <c r="E884" s="2" t="inlineStr">
+        <is>
+          <t>17:42</t>
+        </is>
+      </c>
+      <c r="F884" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G884" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H884" s="2" t="inlineStr"/>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="n">
+        <v>884</v>
+      </c>
+      <c r="B885" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C885" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-2525-4408</t>
+        </is>
+      </c>
+      <c r="D885" s="2" t="inlineStr">
+        <is>
+          <t>Dion</t>
+        </is>
+      </c>
+      <c r="E885" s="2" t="inlineStr">
+        <is>
+          <t>17:42</t>
+        </is>
+      </c>
+      <c r="F885" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G885" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H885" s="2" t="inlineStr"/>
+    </row>
+    <row r="886">
+      <c r="A886" s="2" t="n">
+        <v>885</v>
+      </c>
+      <c r="B886" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C886" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7803-5072</t>
+        </is>
+      </c>
+      <c r="D886" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E886" s="2" t="inlineStr">
+        <is>
+          <t>16:19</t>
+        </is>
+      </c>
+      <c r="F886" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G886" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H886" s="2" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" s="2" t="n">
+        <v>886</v>
+      </c>
+      <c r="B887" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C887" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3702-0766</t>
+        </is>
+      </c>
+      <c r="D887" s="2" t="inlineStr">
+        <is>
+          <t>Rini</t>
+        </is>
+      </c>
+      <c r="E887" s="2" t="inlineStr">
+        <is>
+          <t>17:06</t>
+        </is>
+      </c>
+      <c r="F887" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G887" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H887" s="2" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="B888" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C888" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4294-9515</t>
+        </is>
+      </c>
+      <c r="D888" s="2" t="inlineStr">
+        <is>
+          <t>djarwisalwis</t>
+        </is>
+      </c>
+      <c r="E888" s="2" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="F888" s="2" t="inlineStr">
+        <is>
+          <t>Berapa harganya. (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G888" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H888" s="2" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" s="2" t="n">
+        <v>888</v>
+      </c>
+      <c r="B889" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C889" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8742-5655</t>
+        </is>
+      </c>
+      <c r="D889" s="2" t="inlineStr"/>
+      <c r="E889" s="2" t="inlineStr">
+        <is>
+          <t>06:49</t>
+        </is>
+      </c>
+      <c r="F889" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G889" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H889" s="2" t="inlineStr"/>
+    </row>
+    <row r="890">
+      <c r="A890" s="2" t="n">
+        <v>889</v>
+      </c>
+      <c r="B890" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C890" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9957-7808</t>
+        </is>
+      </c>
+      <c r="D890" s="2" t="inlineStr">
+        <is>
+          <t>Kukuh</t>
+        </is>
+      </c>
+      <c r="E890" s="2" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="F890" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G890" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H890" s="2" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" s="2" t="n">
+        <v>890</v>
+      </c>
+      <c r="B891" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C891" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7351-6137</t>
+        </is>
+      </c>
+      <c r="D891" s="2" t="inlineStr">
+        <is>
+          <t>divadily</t>
+        </is>
+      </c>
+      <c r="E891" s="2" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="F891" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G891" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H891" s="2" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" s="2" t="n">
+        <v>891</v>
+      </c>
+      <c r="B892" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C892" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4216-0528</t>
+        </is>
+      </c>
+      <c r="D892" s="2" t="inlineStr">
+        <is>
+          <t>jufrispdmm69@gmail.com</t>
+        </is>
+      </c>
+      <c r="E892" s="2" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="F892" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G892" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H892" s="2" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" s="2" t="n">
+        <v>892</v>
+      </c>
+      <c r="B893" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C893" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7979-8970</t>
+        </is>
+      </c>
+      <c r="D893" s="2" t="inlineStr">
+        <is>
+          <t>Purwanto</t>
+        </is>
+      </c>
+      <c r="E893" s="2" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="F893" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G893" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H893" s="2" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" s="2" t="n">
+        <v>893</v>
+      </c>
+      <c r="B894" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C894" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7753-7433</t>
+        </is>
+      </c>
+      <c r="D894" s="2" t="inlineStr">
+        <is>
+          <t>Imam</t>
+        </is>
+      </c>
+      <c r="E894" s="2" t="inlineStr">
+        <is>
+          <t>00:37</t>
+        </is>
+      </c>
+      <c r="F894" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G894" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H894" s="2" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" s="2" t="n">
+        <v>894</v>
+      </c>
+      <c r="B895" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C895" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-5328-5571</t>
+        </is>
+      </c>
+      <c r="D895" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E895" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="F895" s="2" t="inlineStr">
+        <is>
+          <t>cek arga bos (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G895" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H895" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 68 of leads WA (6, 12, 19-21 Sept 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01557kCSXmpK1ujmS3edppio
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H895"/>
+  <dimension ref="A1:H910"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -32946,6 +32946,546 @@
       </c>
       <c r="H895" s="2" t="inlineStr"/>
     </row>
+    <row r="896">
+      <c r="A896" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="B896" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C896" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4430-4458</t>
+        </is>
+      </c>
+      <c r="D896" s="2" t="inlineStr">
+        <is>
+          <t>Y2FD</t>
+        </is>
+      </c>
+      <c r="E896" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F896" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G896" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H896" s="2" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" s="2" t="n">
+        <v>896</v>
+      </c>
+      <c r="B897" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C897" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6013-4460</t>
+        </is>
+      </c>
+      <c r="D897" s="2" t="inlineStr">
+        <is>
+          <t>edi muliyono24</t>
+        </is>
+      </c>
+      <c r="E897" s="2" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="F897" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G897" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H897" s="2" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" s="2" t="n">
+        <v>897</v>
+      </c>
+      <c r="B898" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C898" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-8432-5433</t>
+        </is>
+      </c>
+      <c r="D898" s="2" t="inlineStr">
+        <is>
+          <t>Akang</t>
+        </is>
+      </c>
+      <c r="E898" s="2" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="F898" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G898" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H898" s="2" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="B899" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C899" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7637-0179</t>
+        </is>
+      </c>
+      <c r="D899" s="2" t="inlineStr">
+        <is>
+          <t>Inggit Urang Biaso</t>
+        </is>
+      </c>
+      <c r="E899" s="2" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="F899" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Ada cover avanza veloz 1,5 tahun 2017</t>
+        </is>
+      </c>
+      <c r="G899" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H899" s="2" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" s="2" t="n">
+        <v>899</v>
+      </c>
+      <c r="B900" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C900" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4709-7205</t>
+        </is>
+      </c>
+      <c r="D900" s="2" t="inlineStr">
+        <is>
+          <t>Titin Suleman</t>
+        </is>
+      </c>
+      <c r="E900" s="2" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="F900" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Brp harganya</t>
+        </is>
+      </c>
+      <c r="G900" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H900" s="2" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="B901" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C901" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4234-9410</t>
+        </is>
+      </c>
+      <c r="D901" s="2" t="inlineStr">
+        <is>
+          <t>Arif Paria</t>
+        </is>
+      </c>
+      <c r="E901" s="2" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="F901" s="2" t="inlineStr">
+        <is>
+          <t>Cover mobil brv (tidak pakai CTA template)</t>
+        </is>
+      </c>
+      <c r="G901" s="2" t="inlineStr">
+        <is>
+          <t>Whatsapp</t>
+        </is>
+      </c>
+      <c r="H901" s="2" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" s="2" t="n">
+        <v>901</v>
+      </c>
+      <c r="B902" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C902" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4182-5613</t>
+        </is>
+      </c>
+      <c r="D902" s="2" t="inlineStr">
+        <is>
+          <t>odix</t>
+        </is>
+      </c>
+      <c r="E902" s="2" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="F902" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G902" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H902" s="2" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" s="2" t="n">
+        <v>902</v>
+      </c>
+      <c r="B903" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C903" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7020-5601</t>
+        </is>
+      </c>
+      <c r="D903" s="2" t="inlineStr">
+        <is>
+          <t>netri hanthoni</t>
+        </is>
+      </c>
+      <c r="E903" s="2" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="F903" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G903" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H903" s="2" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" s="2" t="n">
+        <v>903</v>
+      </c>
+      <c r="B904" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C904" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-9544-0497</t>
+        </is>
+      </c>
+      <c r="D904" s="2" t="inlineStr">
+        <is>
+          <t>Alif&amp;Alby</t>
+        </is>
+      </c>
+      <c r="E904" s="2" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="F904" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Berapa hargax</t>
+        </is>
+      </c>
+      <c r="G904" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H904" s="2" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B905" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C905" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-5228-2781</t>
+        </is>
+      </c>
+      <c r="D905" s="2" t="inlineStr">
+        <is>
+          <t>Juni</t>
+        </is>
+      </c>
+      <c r="E905" s="2" t="inlineStr">
+        <is>
+          <t>06:29</t>
+        </is>
+      </c>
+      <c r="F905" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare buat mbil Toyota Rush gr spotr ada</t>
+        </is>
+      </c>
+      <c r="G905" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H905" s="2" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" s="2" t="n">
+        <v>905</v>
+      </c>
+      <c r="B906" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C906" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3912-5799</t>
+        </is>
+      </c>
+      <c r="D906" s="2" t="inlineStr">
+        <is>
+          <t>Saudagar Sewi</t>
+        </is>
+      </c>
+      <c r="E906" s="2" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="F906" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G906" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H906" s="2" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" s="2" t="n">
+        <v>906</v>
+      </c>
+      <c r="B907" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C907" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-5303-6043</t>
+        </is>
+      </c>
+      <c r="D907" s="2" t="inlineStr">
+        <is>
+          <t>Mhammad fhmi.</t>
+        </is>
+      </c>
+      <c r="E907" s="2" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="F907" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G907" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H907" s="2" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" s="2" t="n">
+        <v>907</v>
+      </c>
+      <c r="B908" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C908" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8432-6806</t>
+        </is>
+      </c>
+      <c r="D908" s="2" t="inlineStr">
+        <is>
+          <t>Rinaa</t>
+        </is>
+      </c>
+      <c r="E908" s="2" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="F908" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare (dikirim ulang)</t>
+        </is>
+      </c>
+      <c r="G908" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H908" s="2" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" s="2" t="n">
+        <v>908</v>
+      </c>
+      <c r="B909" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C909" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9993-4355</t>
+        </is>
+      </c>
+      <c r="D909" s="2" t="inlineStr">
+        <is>
+          <t>MANGKURAJIN502</t>
+        </is>
+      </c>
+      <c r="E909" s="2" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="F909" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G909" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H909" s="2" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" s="2" t="n">
+        <v>909</v>
+      </c>
+      <c r="B910" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C910" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-1704-5108</t>
+        </is>
+      </c>
+      <c r="D910" s="2" t="inlineStr">
+        <is>
+          <t>Whendy_17</t>
+        </is>
+      </c>
+      <c r="E910" s="2" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="F910" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G910" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H910" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add batch 69 of leads WA (4, 7-8, 10, 15-24 Sept 2026)
114 new leads across 3 agent-extracted batches, 0 duplicates found.
</commit_message>
<xml_diff>
--- a/data/leads_wa.xlsx
+++ b/data/leads_wa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H910"/>
+  <dimension ref="A1:H1024"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -33486,6 +33486,4106 @@
       </c>
       <c r="H910" s="2" t="inlineStr"/>
     </row>
+    <row r="911">
+      <c r="A911" s="2" t="n">
+        <v>910</v>
+      </c>
+      <c r="B911" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C911" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-0878-0792</t>
+        </is>
+      </c>
+      <c r="D911" s="2" t="inlineStr">
+        <is>
+          <t>Suhendi</t>
+        </is>
+      </c>
+      <c r="E911" s="2" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="F911" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G911" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H911" s="2" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" s="2" t="n">
+        <v>911</v>
+      </c>
+      <c r="B912" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C912" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4608-6888</t>
+        </is>
+      </c>
+      <c r="D912" s="2" t="inlineStr">
+        <is>
+          <t>Diana Adjam</t>
+        </is>
+      </c>
+      <c r="E912" s="2" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="F912" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G912" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H912" s="2" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" s="2" t="n">
+        <v>912</v>
+      </c>
+      <c r="B913" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C913" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1321-5343</t>
+        </is>
+      </c>
+      <c r="D913" s="2" t="inlineStr">
+        <is>
+          <t>Zeri Irawan</t>
+        </is>
+      </c>
+      <c r="E913" s="2" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="F913" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G913" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H913" s="2" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" s="2" t="n">
+        <v>913</v>
+      </c>
+      <c r="B914" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C914" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9947-8590</t>
+        </is>
+      </c>
+      <c r="D914" s="2" t="inlineStr">
+        <is>
+          <t>athaya dan arsy</t>
+        </is>
+      </c>
+      <c r="E914" s="2" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="F914" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G914" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H914" s="2" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" s="2" t="n">
+        <v>914</v>
+      </c>
+      <c r="B915" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C915" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9993-0457</t>
+        </is>
+      </c>
+      <c r="D915" s="2" t="inlineStr">
+        <is>
+          <t>grahasandhicoliving</t>
+        </is>
+      </c>
+      <c r="E915" s="2" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="F915" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G915" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H915" s="2" t="inlineStr"/>
+    </row>
+    <row r="916">
+      <c r="A916" s="2" t="n">
+        <v>915</v>
+      </c>
+      <c r="B916" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C916" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-9271-9084</t>
+        </is>
+      </c>
+      <c r="D916" s="2" t="inlineStr">
+        <is>
+          <t>Kadek Ar</t>
+        </is>
+      </c>
+      <c r="E916" s="2" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="F916" s="2" t="inlineStr">
+        <is>
+          <t>Hallo ut Daihatsu Sigra 25 ada kak ? Harga ?</t>
+        </is>
+      </c>
+      <c r="G916" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H916" s="2" t="inlineStr"/>
+    </row>
+    <row r="917">
+      <c r="A917" s="2" t="n">
+        <v>916</v>
+      </c>
+      <c r="B917" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C917" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4170-5788</t>
+        </is>
+      </c>
+      <c r="D917" s="2" t="inlineStr">
+        <is>
+          <t>Sadra Genjing</t>
+        </is>
+      </c>
+      <c r="E917" s="2" t="inlineStr">
+        <is>
+          <t>01:52</t>
+        </is>
+      </c>
+      <c r="F917" s="2" t="inlineStr">
+        <is>
+          <t>Pesan sarung jok mobil</t>
+        </is>
+      </c>
+      <c r="G917" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H917" s="2" t="inlineStr"/>
+    </row>
+    <row r="918">
+      <c r="A918" s="2" t="n">
+        <v>917</v>
+      </c>
+      <c r="B918" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C918" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-7671-8744</t>
+        </is>
+      </c>
+      <c r="D918" s="2" t="inlineStr">
+        <is>
+          <t>Ts Jaya Listrik</t>
+        </is>
+      </c>
+      <c r="E918" s="2" t="inlineStr">
+        <is>
+          <t>11:16</t>
+        </is>
+      </c>
+      <c r="F918" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G918" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H918" s="2" t="inlineStr"/>
+    </row>
+    <row r="919">
+      <c r="A919" s="2" t="n">
+        <v>918</v>
+      </c>
+      <c r="B919" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C919" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-3195-3789</t>
+        </is>
+      </c>
+      <c r="D919" s="2" t="inlineStr">
+        <is>
+          <t>Bunda Tati</t>
+        </is>
+      </c>
+      <c r="E919" s="2" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="F919" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G919" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H919" s="2" t="inlineStr"/>
+    </row>
+    <row r="920">
+      <c r="A920" s="2" t="n">
+        <v>919</v>
+      </c>
+      <c r="B920" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C920" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7624-6913</t>
+        </is>
+      </c>
+      <c r="D920" s="2" t="inlineStr">
+        <is>
+          <t>Ummu Sufyan</t>
+        </is>
+      </c>
+      <c r="E920" s="2" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="F920" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G920" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H920" s="2" t="inlineStr"/>
+    </row>
+    <row r="921">
+      <c r="A921" s="2" t="n">
+        <v>920</v>
+      </c>
+      <c r="B921" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C921" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-9843-4898</t>
+        </is>
+      </c>
+      <c r="D921" s="2" t="inlineStr">
+        <is>
+          <t>Jevita</t>
+        </is>
+      </c>
+      <c r="E921" s="2" t="inlineStr">
+        <is>
+          <t>23:37</t>
+        </is>
+      </c>
+      <c r="F921" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G921" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H921" s="2" t="inlineStr"/>
+    </row>
+    <row r="922">
+      <c r="A922" s="2" t="n">
+        <v>921</v>
+      </c>
+      <c r="B922" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C922" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-4095-4749</t>
+        </is>
+      </c>
+      <c r="D922" s="2" t="inlineStr">
+        <is>
+          <t>Hamba Allah</t>
+        </is>
+      </c>
+      <c r="E922" s="2" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="F922" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Info harga</t>
+        </is>
+      </c>
+      <c r="G922" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H922" s="2" t="inlineStr"/>
+    </row>
+    <row r="923">
+      <c r="A923" s="2" t="n">
+        <v>922</v>
+      </c>
+      <c r="B923" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C923" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-9407-8386</t>
+        </is>
+      </c>
+      <c r="D923" s="2" t="inlineStr">
+        <is>
+          <t>Pakmanboby</t>
+        </is>
+      </c>
+      <c r="E923" s="2" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="F923" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G923" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H923" s="2" t="inlineStr"/>
+    </row>
+    <row r="924">
+      <c r="A924" s="2" t="n">
+        <v>923</v>
+      </c>
+      <c r="B924" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C924" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-5023-2888</t>
+        </is>
+      </c>
+      <c r="D924" s="2" t="inlineStr">
+        <is>
+          <t>ludaehanduran</t>
+        </is>
+      </c>
+      <c r="E924" s="2" t="inlineStr">
+        <is>
+          <t>06:46</t>
+        </is>
+      </c>
+      <c r="F924" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G924" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H924" s="2" t="inlineStr"/>
+    </row>
+    <row r="925">
+      <c r="A925" s="2" t="n">
+        <v>924</v>
+      </c>
+      <c r="B925" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C925" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1443-4513</t>
+        </is>
+      </c>
+      <c r="D925" s="2" t="inlineStr">
+        <is>
+          <t>@b</t>
+        </is>
+      </c>
+      <c r="E925" s="2" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="F925" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G925" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H925" s="2" t="inlineStr"/>
+    </row>
+    <row r="926">
+      <c r="A926" s="2" t="n">
+        <v>925</v>
+      </c>
+      <c r="B926" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C926" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8952-0370</t>
+        </is>
+      </c>
+      <c r="D926" s="2" t="inlineStr">
+        <is>
+          <t>Ran</t>
+        </is>
+      </c>
+      <c r="E926" s="2" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="F926" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G926" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H926" s="2" t="inlineStr"/>
+    </row>
+    <row r="927">
+      <c r="A927" s="2" t="n">
+        <v>926</v>
+      </c>
+      <c r="B927" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C927" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4001-8063</t>
+        </is>
+      </c>
+      <c r="D927" s="2" t="inlineStr">
+        <is>
+          <t>Richard Posumah</t>
+        </is>
+      </c>
+      <c r="E927" s="2" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="F927" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G927" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H927" s="2" t="inlineStr"/>
+    </row>
+    <row r="928">
+      <c r="A928" s="2" t="n">
+        <v>927</v>
+      </c>
+      <c r="B928" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C928" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-3058-8732</t>
+        </is>
+      </c>
+      <c r="D928" s="2" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="E928" s="2" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="F928" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G928" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H928" s="2" t="inlineStr"/>
+    </row>
+    <row r="929">
+      <c r="A929" s="2" t="n">
+        <v>928</v>
+      </c>
+      <c r="B929" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C929" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6822-4599</t>
+        </is>
+      </c>
+      <c r="D929" s="2" t="inlineStr">
+        <is>
+          <t>defriyanto</t>
+        </is>
+      </c>
+      <c r="E929" s="2" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="F929" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G929" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H929" s="2" t="inlineStr"/>
+    </row>
+    <row r="930">
+      <c r="A930" s="2" t="n">
+        <v>929</v>
+      </c>
+      <c r="B930" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C930" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9594-0689</t>
+        </is>
+      </c>
+      <c r="D930" s="2" t="inlineStr">
+        <is>
+          <t>Ayah Razqashiqa</t>
+        </is>
+      </c>
+      <c r="E930" s="2" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="F930" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G930" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H930" s="2" t="inlineStr"/>
+    </row>
+    <row r="931">
+      <c r="A931" s="2" t="n">
+        <v>930</v>
+      </c>
+      <c r="B931" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C931" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-0331-6644</t>
+        </is>
+      </c>
+      <c r="D931" s="2" t="inlineStr">
+        <is>
+          <t>mnoordiansyah</t>
+        </is>
+      </c>
+      <c r="E931" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="F931" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G931" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H931" s="2" t="inlineStr"/>
+    </row>
+    <row r="932">
+      <c r="A932" s="2" t="n">
+        <v>931</v>
+      </c>
+      <c r="B932" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C932" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-2352-9723</t>
+        </is>
+      </c>
+      <c r="D932" s="2" t="inlineStr">
+        <is>
+          <t>hellyke29</t>
+        </is>
+      </c>
+      <c r="E932" s="2" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="F932" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G932" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H932" s="2" t="inlineStr"/>
+    </row>
+    <row r="933">
+      <c r="A933" s="2" t="n">
+        <v>932</v>
+      </c>
+      <c r="B933" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C933" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-5962-4440</t>
+        </is>
+      </c>
+      <c r="D933" s="2" t="inlineStr">
+        <is>
+          <t>Zacky Andrian Iqbal</t>
+        </is>
+      </c>
+      <c r="E933" s="2" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="F933" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G933" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H933" s="2" t="inlineStr"/>
+    </row>
+    <row r="934">
+      <c r="A934" s="2" t="n">
+        <v>933</v>
+      </c>
+      <c r="B934" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C934" s="2" t="inlineStr">
+        <is>
+          <t>+62 817-355-309</t>
+        </is>
+      </c>
+      <c r="D934" s="2" t="inlineStr">
+        <is>
+          <t>IKAstawan</t>
+        </is>
+      </c>
+      <c r="E934" s="2" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="F934" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk mobil Mobilio th 2014</t>
+        </is>
+      </c>
+      <c r="G934" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H934" s="2" t="inlineStr"/>
+    </row>
+    <row r="935">
+      <c r="A935" s="2" t="n">
+        <v>934</v>
+      </c>
+      <c r="B935" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C935" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-8982-5335</t>
+        </is>
+      </c>
+      <c r="D935" s="2" t="inlineStr">
+        <is>
+          <t>Rubie</t>
+        </is>
+      </c>
+      <c r="E935" s="2" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="F935" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G935" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H935" s="2" t="inlineStr"/>
+    </row>
+    <row r="936">
+      <c r="A936" s="2" t="n">
+        <v>935</v>
+      </c>
+      <c r="B936" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C936" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-2524-4491</t>
+        </is>
+      </c>
+      <c r="D936" s="2" t="inlineStr">
+        <is>
+          <t>aprisarfan</t>
+        </is>
+      </c>
+      <c r="E936" s="2" t="inlineStr">
+        <is>
+          <t>04:43</t>
+        </is>
+      </c>
+      <c r="F936" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G936" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H936" s="2" t="inlineStr"/>
+    </row>
+    <row r="937">
+      <c r="A937" s="2" t="n">
+        <v>936</v>
+      </c>
+      <c r="B937" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C937" s="2" t="inlineStr">
+        <is>
+          <t>+62 818-556-990</t>
+        </is>
+      </c>
+      <c r="D937" s="2" t="inlineStr">
+        <is>
+          <t>Wa-One</t>
+        </is>
+      </c>
+      <c r="E937" s="2" t="inlineStr">
+        <is>
+          <t>03:33</t>
+        </is>
+      </c>
+      <c r="F937" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G937" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H937" s="2" t="inlineStr"/>
+    </row>
+    <row r="938">
+      <c r="A938" s="2" t="n">
+        <v>937</v>
+      </c>
+      <c r="B938" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C938" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-1210-3471</t>
+        </is>
+      </c>
+      <c r="D938" s="2" t="inlineStr">
+        <is>
+          <t>Embun Hendrodjati</t>
+        </is>
+      </c>
+      <c r="E938" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="F938" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G938" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H938" s="2" t="inlineStr"/>
+    </row>
+    <row r="939">
+      <c r="A939" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="B939" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C939" s="2" t="inlineStr">
+        <is>
+          <t>+62 831-3510-2328</t>
+        </is>
+      </c>
+      <c r="D939" s="2" t="inlineStr">
+        <is>
+          <t>Mengetik....</t>
+        </is>
+      </c>
+      <c r="E939" s="2" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="F939" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G939" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H939" s="2" t="inlineStr"/>
+    </row>
+    <row r="940">
+      <c r="A940" s="2" t="n">
+        <v>939</v>
+      </c>
+      <c r="B940" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C940" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1070-8926</t>
+        </is>
+      </c>
+      <c r="D940" s="2" t="inlineStr">
+        <is>
+          <t>Jess</t>
+        </is>
+      </c>
+      <c r="E940" s="2" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="F940" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Selamat pagi Bapak Ibu Untk toyota inovasi zenix ada Pak?</t>
+        </is>
+      </c>
+      <c r="G940" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H940" s="2" t="inlineStr"/>
+    </row>
+    <row r="941">
+      <c r="A941" s="2" t="n">
+        <v>940</v>
+      </c>
+      <c r="B941" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C941" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-2666-5551</t>
+        </is>
+      </c>
+      <c r="D941" s="2" t="inlineStr">
+        <is>
+          <t>Erwin BRT</t>
+        </is>
+      </c>
+      <c r="E941" s="2" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="F941" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utuk ayla berapa merah</t>
+        </is>
+      </c>
+      <c r="G941" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H941" s="2" t="inlineStr"/>
+    </row>
+    <row r="942">
+      <c r="A942" s="2" t="n">
+        <v>941</v>
+      </c>
+      <c r="B942" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C942" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9890-1514</t>
+        </is>
+      </c>
+      <c r="D942" s="2" t="inlineStr">
+        <is>
+          <t>CAM</t>
+        </is>
+      </c>
+      <c r="E942" s="2" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="F942" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G942" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H942" s="2" t="inlineStr"/>
+    </row>
+    <row r="943">
+      <c r="A943" s="2" t="n">
+        <v>942</v>
+      </c>
+      <c r="B943" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C943" s="2" t="inlineStr">
+        <is>
+          <t>+62 819-2459-224</t>
+        </is>
+      </c>
+      <c r="D943" s="2" t="inlineStr">
+        <is>
+          <t>marvin</t>
+        </is>
+      </c>
+      <c r="E943" s="2" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="F943" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G943" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H943" s="2" t="inlineStr"/>
+    </row>
+    <row r="944">
+      <c r="A944" s="2" t="n">
+        <v>943</v>
+      </c>
+      <c r="B944" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C944" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7407-4660</t>
+        </is>
+      </c>
+      <c r="D944" s="2" t="inlineStr">
+        <is>
+          <t>Yandri Ardianto</t>
+        </is>
+      </c>
+      <c r="E944" s="2" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="F944" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G944" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H944" s="2" t="inlineStr"/>
+    </row>
+    <row r="945">
+      <c r="A945" s="2" t="n">
+        <v>944</v>
+      </c>
+      <c r="B945" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C945" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-9414-0248</t>
+        </is>
+      </c>
+      <c r="D945" s="2" t="inlineStr">
+        <is>
+          <t>Mangku Ardika</t>
+        </is>
+      </c>
+      <c r="E945" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="F945" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G945" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H945" s="2" t="inlineStr"/>
+    </row>
+    <row r="946">
+      <c r="A946" s="2" t="n">
+        <v>945</v>
+      </c>
+      <c r="B946" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C946" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-1440-1778</t>
+        </is>
+      </c>
+      <c r="D946" s="2" t="inlineStr">
+        <is>
+          <t>I KETUT BUDI YASA</t>
+        </is>
+      </c>
+      <c r="E946" s="2" t="inlineStr"/>
+      <c r="F946" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G946" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H946" s="2" t="inlineStr"/>
+    </row>
+    <row r="947">
+      <c r="A947" s="2" t="n">
+        <v>946</v>
+      </c>
+      <c r="B947" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C947" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1663-348</t>
+        </is>
+      </c>
+      <c r="D947" s="2" t="inlineStr">
+        <is>
+          <t>M Raihan Lutfiansyah</t>
+        </is>
+      </c>
+      <c r="E947" s="2" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="F947" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G947" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H947" s="2" t="inlineStr"/>
+    </row>
+    <row r="948">
+      <c r="A948" s="2" t="n">
+        <v>947</v>
+      </c>
+      <c r="B948" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C948" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-2260-9899</t>
+        </is>
+      </c>
+      <c r="D948" s="2" t="inlineStr">
+        <is>
+          <t>Bismilah</t>
+        </is>
+      </c>
+      <c r="E948" s="2" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="F948" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G948" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H948" s="2" t="inlineStr"/>
+    </row>
+    <row r="949">
+      <c r="A949" s="2" t="n">
+        <v>948</v>
+      </c>
+      <c r="B949" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C949" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-7574-0390</t>
+        </is>
+      </c>
+      <c r="D949" s="2" t="inlineStr">
+        <is>
+          <t>Adi</t>
+        </is>
+      </c>
+      <c r="E949" s="2" t="inlineStr">
+        <is>
+          <t>17:49</t>
+        </is>
+      </c>
+      <c r="F949" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Cek hrg cover Ras 2020</t>
+        </is>
+      </c>
+      <c r="G949" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H949" s="2" t="inlineStr"/>
+    </row>
+    <row r="950">
+      <c r="A950" s="2" t="n">
+        <v>949</v>
+      </c>
+      <c r="B950" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C950" s="2" t="inlineStr">
+        <is>
+          <t>+62 856-4584-7048</t>
+        </is>
+      </c>
+      <c r="D950" s="2" t="inlineStr">
+        <is>
+          <t>Juni Prasetyo</t>
+        </is>
+      </c>
+      <c r="E950" s="2" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="F950" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G950" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H950" s="2" t="inlineStr"/>
+    </row>
+    <row r="951">
+      <c r="A951" s="2" t="n">
+        <v>950</v>
+      </c>
+      <c r="B951" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C951" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1665-0808</t>
+        </is>
+      </c>
+      <c r="D951" s="2" t="inlineStr">
+        <is>
+          <t>Eko Andrianto, S.E., M.M.</t>
+        </is>
+      </c>
+      <c r="E951" s="2" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="F951" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G951" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H951" s="2" t="inlineStr"/>
+    </row>
+    <row r="952">
+      <c r="A952" s="2" t="n">
+        <v>951</v>
+      </c>
+      <c r="B952" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C952" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9660-4484</t>
+        </is>
+      </c>
+      <c r="D952" s="2" t="inlineStr">
+        <is>
+          <t>Ama Samuel</t>
+        </is>
+      </c>
+      <c r="E952" s="2" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="F952" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G952" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H952" s="2" t="inlineStr"/>
+    </row>
+    <row r="953">
+      <c r="A953" s="2" t="n">
+        <v>952</v>
+      </c>
+      <c r="B953" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C953" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7441-2241</t>
+        </is>
+      </c>
+      <c r="D953" s="2" t="inlineStr">
+        <is>
+          <t>heri siahyudi</t>
+        </is>
+      </c>
+      <c r="E953" s="2" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="F953" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G953" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H953" s="2" t="inlineStr"/>
+    </row>
+    <row r="954">
+      <c r="A954" s="2" t="n">
+        <v>953</v>
+      </c>
+      <c r="B954" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C954" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4809-9427</t>
+        </is>
+      </c>
+      <c r="D954" s="2" t="inlineStr">
+        <is>
+          <t>Pangeran Helmi</t>
+        </is>
+      </c>
+      <c r="E954" s="2" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="F954" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G954" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H954" s="2" t="inlineStr"/>
+    </row>
+    <row r="955">
+      <c r="A955" s="2" t="n">
+        <v>954</v>
+      </c>
+      <c r="B955" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C955" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4651-9945</t>
+        </is>
+      </c>
+      <c r="D955" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Connor</t>
+        </is>
+      </c>
+      <c r="E955" s="2" t="inlineStr">
+        <is>
+          <t>00:36</t>
+        </is>
+      </c>
+      <c r="F955" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G955" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H955" s="2" t="inlineStr"/>
+    </row>
+    <row r="956">
+      <c r="A956" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="B956" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C956" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3566-1875</t>
+        </is>
+      </c>
+      <c r="D956" s="2" t="inlineStr">
+        <is>
+          <t>Eko Meinanto</t>
+        </is>
+      </c>
+      <c r="E956" s="2" t="inlineStr">
+        <is>
+          <t>18:18</t>
+        </is>
+      </c>
+      <c r="F956" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G956" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H956" s="2" t="inlineStr"/>
+    </row>
+    <row r="957">
+      <c r="A957" s="2" t="n">
+        <v>956</v>
+      </c>
+      <c r="B957" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C957" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-2548-3888</t>
+        </is>
+      </c>
+      <c r="D957" s="2" t="inlineStr">
+        <is>
+          <t>Bahroin Erwin</t>
+        </is>
+      </c>
+      <c r="E957" s="2" t="inlineStr">
+        <is>
+          <t>05:41</t>
+        </is>
+      </c>
+      <c r="F957" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G957" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H957" s="2" t="inlineStr"/>
+    </row>
+    <row r="958">
+      <c r="A958" s="2" t="n">
+        <v>957</v>
+      </c>
+      <c r="B958" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C958" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3926-7710</t>
+        </is>
+      </c>
+      <c r="D958" s="2" t="inlineStr">
+        <is>
+          <t>Agus Losor</t>
+        </is>
+      </c>
+      <c r="E958" s="2" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="F958" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G958" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H958" s="2" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="B959" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C959" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-3803-726</t>
+        </is>
+      </c>
+      <c r="D959" s="2" t="inlineStr">
+        <is>
+          <t>Uncle Joni</t>
+        </is>
+      </c>
+      <c r="E959" s="2" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="F959" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk mobil Avanza 2010</t>
+        </is>
+      </c>
+      <c r="G959" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H959" s="2" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" s="2" t="n">
+        <v>959</v>
+      </c>
+      <c r="B960" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C960" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-8546-2222</t>
+        </is>
+      </c>
+      <c r="D960" s="2" t="inlineStr">
+        <is>
+          <t>Nagin OKE!!</t>
+        </is>
+      </c>
+      <c r="E960" s="2" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="F960" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G960" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H960" s="2" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="B961" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C961" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1313-9252</t>
+        </is>
+      </c>
+      <c r="D961" s="2" t="inlineStr">
+        <is>
+          <t>Budi Hartanto</t>
+        </is>
+      </c>
+      <c r="E961" s="2" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="F961" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G961" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H961" s="2" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" s="2" t="n">
+        <v>961</v>
+      </c>
+      <c r="B962" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C962" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-8296-3190</t>
+        </is>
+      </c>
+      <c r="D962" s="2" t="inlineStr">
+        <is>
+          <t>Emil</t>
+        </is>
+      </c>
+      <c r="E962" s="2" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="F962" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Utk toyota fortuner 2025</t>
+        </is>
+      </c>
+      <c r="G962" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H962" s="2" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="B963" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C963" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4104-0849</t>
+        </is>
+      </c>
+      <c r="D963" s="2" t="inlineStr">
+        <is>
+          <t>Hendrik A Mayor</t>
+        </is>
+      </c>
+      <c r="E963" s="2" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="F963" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G963" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H963" s="2" t="inlineStr"/>
+    </row>
+    <row r="964">
+      <c r="A964" s="2" t="n">
+        <v>963</v>
+      </c>
+      <c r="B964" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C964" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-1571-8193</t>
+        </is>
+      </c>
+      <c r="D964" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E964" s="2" t="inlineStr">
+        <is>
+          <t>09:39</t>
+        </is>
+      </c>
+      <c r="F964" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare Untuk honda accord cielo 94 ada...?</t>
+        </is>
+      </c>
+      <c r="G964" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H964" s="2" t="inlineStr"/>
+    </row>
+    <row r="965">
+      <c r="A965" s="2" t="n">
+        <v>964</v>
+      </c>
+      <c r="B965" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C965" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-9061-9495</t>
+        </is>
+      </c>
+      <c r="D965" s="2" t="inlineStr">
+        <is>
+          <t>Vera</t>
+        </is>
+      </c>
+      <c r="E965" s="2" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="F965" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G965" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H965" s="2" t="inlineStr"/>
+    </row>
+    <row r="966">
+      <c r="A966" s="2" t="n">
+        <v>965</v>
+      </c>
+      <c r="B966" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C966" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-4420-8528</t>
+        </is>
+      </c>
+      <c r="D966" s="2" t="inlineStr">
+        <is>
+          <t>Putra zhelebes</t>
+        </is>
+      </c>
+      <c r="E966" s="2" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="F966" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G966" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H966" s="2" t="inlineStr"/>
+    </row>
+    <row r="967">
+      <c r="A967" s="2" t="n">
+        <v>966</v>
+      </c>
+      <c r="B967" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C967" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-2692-5483</t>
+        </is>
+      </c>
+      <c r="D967" s="2" t="inlineStr">
+        <is>
+          <t>Bpk Britnay.Travel Weemat</t>
+        </is>
+      </c>
+      <c r="E967" s="2" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="F967" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G967" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H967" s="2" t="inlineStr"/>
+    </row>
+    <row r="968">
+      <c r="A968" s="2" t="n">
+        <v>967</v>
+      </c>
+      <c r="B968" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C968" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-6714-4356</t>
+        </is>
+      </c>
+      <c r="D968" s="2" t="inlineStr">
+        <is>
+          <t>mangkuputraperasan</t>
+        </is>
+      </c>
+      <c r="E968" s="2" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="F968" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G968" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H968" s="2" t="inlineStr"/>
+    </row>
+    <row r="969">
+      <c r="A969" s="2" t="n">
+        <v>968</v>
+      </c>
+      <c r="B969" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C969" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-2456-3199</t>
+        </is>
+      </c>
+      <c r="D969" s="2" t="inlineStr">
+        <is>
+          <t>Agus Sae</t>
+        </is>
+      </c>
+      <c r="E969" s="2" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="F969" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G969" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H969" s="2" t="inlineStr"/>
+    </row>
+    <row r="970">
+      <c r="A970" s="2" t="n">
+        <v>969</v>
+      </c>
+      <c r="B970" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C970" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7344-7015</t>
+        </is>
+      </c>
+      <c r="D970" s="2" t="inlineStr">
+        <is>
+          <t>mamy key'na</t>
+        </is>
+      </c>
+      <c r="E970" s="2" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="F970" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G970" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H970" s="2" t="inlineStr"/>
+    </row>
+    <row r="971">
+      <c r="A971" s="2" t="n">
+        <v>970</v>
+      </c>
+      <c r="B971" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C971" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-6300-771</t>
+        </is>
+      </c>
+      <c r="D971" s="2" t="inlineStr">
+        <is>
+          <t>saparuddin</t>
+        </is>
+      </c>
+      <c r="E971" s="2" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="F971" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G971" s="2" t="inlineStr">
+        <is>
+          <t>Meta - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H971" s="2" t="inlineStr"/>
+    </row>
+    <row r="972">
+      <c r="A972" s="2" t="n">
+        <v>971</v>
+      </c>
+      <c r="B972" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C972" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-1940-7181</t>
+        </is>
+      </c>
+      <c r="D972" s="2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="E972" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="F972" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G972" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H972" s="2" t="inlineStr"/>
+    </row>
+    <row r="973">
+      <c r="A973" s="2" t="n">
+        <v>972</v>
+      </c>
+      <c r="B973" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C973" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9999-4084</t>
+        </is>
+      </c>
+      <c r="D973" s="2" t="inlineStr">
+        <is>
+          <t>NOBODY</t>
+        </is>
+      </c>
+      <c r="E973" s="2" t="inlineStr">
+        <is>
+          <t>04:27</t>
+        </is>
+      </c>
+      <c r="F973" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G973" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H973" s="2" t="inlineStr"/>
+    </row>
+    <row r="974">
+      <c r="A974" s="2" t="n">
+        <v>973</v>
+      </c>
+      <c r="B974" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C974" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-2417-9704</t>
+        </is>
+      </c>
+      <c r="D974" s="2" t="inlineStr">
+        <is>
+          <t>M. Ali Maulana</t>
+        </is>
+      </c>
+      <c r="E974" s="2" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="F974" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G974" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H974" s="2" t="inlineStr"/>
+    </row>
+    <row r="975">
+      <c r="A975" s="2" t="n">
+        <v>974</v>
+      </c>
+      <c r="B975" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C975" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-7565-733</t>
+        </is>
+      </c>
+      <c r="D975" s="2" t="inlineStr">
+        <is>
+          <t>abdul Wahid/Andri putra</t>
+        </is>
+      </c>
+      <c r="E975" s="2" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="F975" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G975" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H975" s="2" t="inlineStr"/>
+    </row>
+    <row r="976">
+      <c r="A976" s="2" t="n">
+        <v>975</v>
+      </c>
+      <c r="B976" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C976" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4720-0900</t>
+        </is>
+      </c>
+      <c r="D976" s="2" t="inlineStr">
+        <is>
+          <t>silablasius13@gmail.com</t>
+        </is>
+      </c>
+      <c r="E976" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F976" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G976" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H976" s="2" t="inlineStr"/>
+    </row>
+    <row r="977">
+      <c r="A977" s="2" t="n">
+        <v>976</v>
+      </c>
+      <c r="B977" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C977" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4467-4853</t>
+        </is>
+      </c>
+      <c r="D977" s="2" t="inlineStr">
+        <is>
+          <t>Ronny</t>
+        </is>
+      </c>
+      <c r="E977" s="2" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="F977" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G977" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H977" s="2" t="inlineStr"/>
+    </row>
+    <row r="978">
+      <c r="A978" s="2" t="n">
+        <v>977</v>
+      </c>
+      <c r="B978" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C978" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9505-1373</t>
+        </is>
+      </c>
+      <c r="D978" s="2" t="inlineStr">
+        <is>
+          <t>Abidin</t>
+        </is>
+      </c>
+      <c r="E978" s="2" t="inlineStr">
+        <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="F978" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G978" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H978" s="2" t="inlineStr"/>
+    </row>
+    <row r="979">
+      <c r="A979" s="2" t="n">
+        <v>978</v>
+      </c>
+      <c r="B979" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C979" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-7127-4147</t>
+        </is>
+      </c>
+      <c r="D979" s="2" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="E979" s="2" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="F979" s="2" t="inlineStr">
+        <is>
+          <t>cover untuk mobil Avanza tpeE berapa ya kak</t>
+        </is>
+      </c>
+      <c r="G979" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H979" s="2" t="inlineStr"/>
+    </row>
+    <row r="980">
+      <c r="A980" s="2" t="n">
+        <v>979</v>
+      </c>
+      <c r="B980" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C980" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-4800-1433</t>
+        </is>
+      </c>
+      <c r="D980" s="2" t="inlineStr">
+        <is>
+          <t>(emoji)</t>
+        </is>
+      </c>
+      <c r="E980" s="2" t="inlineStr">
+        <is>
+          <t>06:43</t>
+        </is>
+      </c>
+      <c r="F980" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G980" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H980" s="2" t="inlineStr"/>
+    </row>
+    <row r="981">
+      <c r="A981" s="2" t="n">
+        <v>980</v>
+      </c>
+      <c r="B981" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C981" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-1619-9714</t>
+        </is>
+      </c>
+      <c r="D981" s="2" t="inlineStr">
+        <is>
+          <t>Lettu Suyatno Nano</t>
+        </is>
+      </c>
+      <c r="E981" s="2" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="F981" s="2" t="inlineStr">
+        <is>
+          <t>Autocare</t>
+        </is>
+      </c>
+      <c r="G981" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H981" s="2" t="inlineStr"/>
+    </row>
+    <row r="982">
+      <c r="A982" s="2" t="n">
+        <v>981</v>
+      </c>
+      <c r="B982" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C982" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-9292-7774</t>
+        </is>
+      </c>
+      <c r="D982" s="2" t="inlineStr">
+        <is>
+          <t>Erica</t>
+        </is>
+      </c>
+      <c r="E982" s="2" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="F982" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G982" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H982" s="2" t="inlineStr"/>
+    </row>
+    <row r="983">
+      <c r="A983" s="2" t="n">
+        <v>982</v>
+      </c>
+      <c r="B983" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C983" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-4576-0840</t>
+        </is>
+      </c>
+      <c r="D983" s="2" t="inlineStr">
+        <is>
+          <t>Papa Kamayaa</t>
+        </is>
+      </c>
+      <c r="E983" s="2" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="F983" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G983" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H983" s="2" t="inlineStr"/>
+    </row>
+    <row r="984">
+      <c r="A984" s="2" t="n">
+        <v>983</v>
+      </c>
+      <c r="B984" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C984" s="2" t="inlineStr">
+        <is>
+          <t>+62 878-0984-8019</t>
+        </is>
+      </c>
+      <c r="D984" s="2" t="inlineStr">
+        <is>
+          <t>Pudin</t>
+        </is>
+      </c>
+      <c r="E984" s="2" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="F984" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G984" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H984" s="2" t="inlineStr"/>
+    </row>
+    <row r="985">
+      <c r="A985" s="2" t="n">
+        <v>984</v>
+      </c>
+      <c r="B985" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C985" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4719-1111</t>
+        </is>
+      </c>
+      <c r="D985" s="2" t="inlineStr">
+        <is>
+          <t>Antonius Marten</t>
+        </is>
+      </c>
+      <c r="E985" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="F985" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G985" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H985" s="2" t="inlineStr"/>
+    </row>
+    <row r="986">
+      <c r="A986" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="B986" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C986" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4312-4729</t>
+        </is>
+      </c>
+      <c r="D986" s="2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="E986" s="2" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="F986" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G986" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H986" s="2" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" s="2" t="n">
+        <v>986</v>
+      </c>
+      <c r="B987" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C987" s="2" t="inlineStr">
+        <is>
+          <t>+62 896-3109-5891</t>
+        </is>
+      </c>
+      <c r="D987" s="2" t="inlineStr">
+        <is>
+          <t>Raappaarr</t>
+        </is>
+      </c>
+      <c r="E987" s="2" t="inlineStr">
+        <is>
+          <t>00:52</t>
+        </is>
+      </c>
+      <c r="F987" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G987" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H987" s="2" t="inlineStr"/>
+    </row>
+    <row r="988">
+      <c r="A988" s="2" t="n">
+        <v>987</v>
+      </c>
+      <c r="B988" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C988" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-1802-5188</t>
+        </is>
+      </c>
+      <c r="D988" s="2" t="inlineStr">
+        <is>
+          <t>Franky Merentek</t>
+        </is>
+      </c>
+      <c r="E988" s="2" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="F988" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G988" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H988" s="2" t="inlineStr"/>
+    </row>
+    <row r="989">
+      <c r="A989" s="2" t="n">
+        <v>988</v>
+      </c>
+      <c r="B989" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C989" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-3773-3772</t>
+        </is>
+      </c>
+      <c r="D989" s="2" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
+      <c r="E989" s="2" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="F989" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G989" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H989" s="2" t="inlineStr"/>
+    </row>
+    <row r="990">
+      <c r="A990" s="2" t="n">
+        <v>989</v>
+      </c>
+      <c r="B990" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C990" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-6837-2596</t>
+        </is>
+      </c>
+      <c r="D990" s="2" t="inlineStr">
+        <is>
+          <t>Riga</t>
+        </is>
+      </c>
+      <c r="E990" s="2" t="inlineStr">
+        <is>
+          <t>23:36</t>
+        </is>
+      </c>
+      <c r="F990" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G990" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H990" s="2" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="n">
+        <v>990</v>
+      </c>
+      <c r="B991" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C991" s="2" t="inlineStr">
+        <is>
+          <t>+62 815-2435-6028</t>
+        </is>
+      </c>
+      <c r="D991" s="2" t="inlineStr">
+        <is>
+          <t>Lubis</t>
+        </is>
+      </c>
+      <c r="E991" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="F991" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G991" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H991" s="2" t="inlineStr"/>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>991</v>
+      </c>
+      <c r="B992" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C992" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-3241-3736</t>
+        </is>
+      </c>
+      <c r="D992" s="2" t="inlineStr">
+        <is>
+          <t>Irf4n s4nj4ya</t>
+        </is>
+      </c>
+      <c r="E992" s="2" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="F992" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G992" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H992" s="2" t="inlineStr"/>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="n">
+        <v>992</v>
+      </c>
+      <c r="B993" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C993" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-5662-2597</t>
+        </is>
+      </c>
+      <c r="D993" s="2" t="inlineStr">
+        <is>
+          <t>Zhem</t>
+        </is>
+      </c>
+      <c r="E993" s="2" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
+      <c r="F993" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G993" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H993" s="2" t="inlineStr"/>
+    </row>
+    <row r="994">
+      <c r="A994" s="2" t="n">
+        <v>993</v>
+      </c>
+      <c r="B994" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C994" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-2906-8479</t>
+        </is>
+      </c>
+      <c r="D994" s="2" t="inlineStr">
+        <is>
+          <t>Saeful Bahri</t>
+        </is>
+      </c>
+      <c r="E994" s="2" t="inlineStr">
+        <is>
+          <t>07:04</t>
+        </is>
+      </c>
+      <c r="F994" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G994" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H994" s="2" t="inlineStr"/>
+    </row>
+    <row r="995">
+      <c r="A995" s="2" t="n">
+        <v>994</v>
+      </c>
+      <c r="B995" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C995" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-8365-1981</t>
+        </is>
+      </c>
+      <c r="D995" s="2" t="inlineStr">
+        <is>
+          <t>irsan Rosyidi AbG</t>
+        </is>
+      </c>
+      <c r="E995" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="F995" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G995" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H995" s="2" t="inlineStr"/>
+    </row>
+    <row r="996">
+      <c r="A996" s="2" t="n">
+        <v>995</v>
+      </c>
+      <c r="B996" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C996" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-1460-1539</t>
+        </is>
+      </c>
+      <c r="D996" s="2" t="inlineStr">
+        <is>
+          <t>m.rohim</t>
+        </is>
+      </c>
+      <c r="E996" s="2" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="F996" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G996" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H996" s="2" t="inlineStr"/>
+    </row>
+    <row r="997">
+      <c r="A997" s="2" t="n">
+        <v>996</v>
+      </c>
+      <c r="B997" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C997" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-1964-9294</t>
+        </is>
+      </c>
+      <c r="D997" s="2" t="inlineStr">
+        <is>
+          <t>mak edo</t>
+        </is>
+      </c>
+      <c r="E997" s="2" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="F997" s="2" t="inlineStr">
+        <is>
+          <t>berapa sista,,</t>
+        </is>
+      </c>
+      <c r="G997" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H997" s="2" t="inlineStr"/>
+    </row>
+    <row r="998">
+      <c r="A998" s="2" t="n">
+        <v>997</v>
+      </c>
+      <c r="B998" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C998" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-3804-2340</t>
+        </is>
+      </c>
+      <c r="D998" s="2" t="inlineStr">
+        <is>
+          <t>n89053282</t>
+        </is>
+      </c>
+      <c r="E998" s="2" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="F998" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G998" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H998" s="2" t="inlineStr"/>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="B999" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C999" s="2" t="inlineStr">
+        <is>
+          <t>+62 851-1997-1565</t>
+        </is>
+      </c>
+      <c r="D999" s="2" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="E999" s="2" t="inlineStr">
+        <is>
+          <t>04:46</t>
+        </is>
+      </c>
+      <c r="F999" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G999" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H999" s="2" t="inlineStr"/>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="n">
+        <v>999</v>
+      </c>
+      <c r="B1000" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1000" s="2" t="inlineStr">
+        <is>
+          <t>+62 877-7808-0172</t>
+        </is>
+      </c>
+      <c r="D1000" s="2" t="inlineStr">
+        <is>
+          <t>aloysiusfkwenang</t>
+        </is>
+      </c>
+      <c r="E1000" s="2" t="inlineStr">
+        <is>
+          <t>05:46</t>
+        </is>
+      </c>
+      <c r="F1000" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1000" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1000" s="2" t="inlineStr"/>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B1001" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1001" s="2" t="inlineStr">
+        <is>
+          <t>+62 853-4150-1953</t>
+        </is>
+      </c>
+      <c r="D1001" s="2" t="inlineStr">
+        <is>
+          <t>Tamsil Hasbullah</t>
+        </is>
+      </c>
+      <c r="E1001" s="2" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="F1001" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1001" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1001" s="2" t="inlineStr"/>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B1002" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1002" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-3535-6766</t>
+        </is>
+      </c>
+      <c r="D1002" s="2" t="inlineStr">
+        <is>
+          <t>Rasit</t>
+        </is>
+      </c>
+      <c r="E1002" s="2" t="inlineStr">
+        <is>
+          <t>02:09</t>
+        </is>
+      </c>
+      <c r="F1002" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1002" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1002" s="2" t="inlineStr"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B1003" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1003" s="2" t="inlineStr">
+        <is>
+          <t>+62 811-1333-888</t>
+        </is>
+      </c>
+      <c r="D1003" s="2" t="inlineStr">
+        <is>
+          <t>H JAUW</t>
+        </is>
+      </c>
+      <c r="E1003" s="2" t="inlineStr">
+        <is>
+          <t>04:40</t>
+        </is>
+      </c>
+      <c r="F1003" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1003" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1003" s="2" t="inlineStr"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="2" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B1004" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1004" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-1233-9541</t>
+        </is>
+      </c>
+      <c r="D1004" s="2" t="inlineStr">
+        <is>
+          <t>agussinging</t>
+        </is>
+      </c>
+      <c r="E1004" s="2" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="F1004" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1004" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1004" s="2" t="inlineStr"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B1005" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1005" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-7685-1024</t>
+        </is>
+      </c>
+      <c r="D1005" s="2" t="inlineStr">
+        <is>
+          <t>H.Suherman</t>
+        </is>
+      </c>
+      <c r="E1005" s="2" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="F1005" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1005" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1005" s="2" t="inlineStr"/>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B1006" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1006" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4060-5103</t>
+        </is>
+      </c>
+      <c r="D1006" s="2" t="inlineStr">
+        <is>
+          <t>Suyib</t>
+        </is>
+      </c>
+      <c r="E1006" s="2" t="inlineStr">
+        <is>
+          <t>21:48</t>
+        </is>
+      </c>
+      <c r="F1006" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1006" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1006" s="2" t="inlineStr"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B1007" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1007" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-6655-6225</t>
+        </is>
+      </c>
+      <c r="D1007" s="2" t="inlineStr">
+        <is>
+          <t>Fincy Annisa</t>
+        </is>
+      </c>
+      <c r="E1007" s="2" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="F1007" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1007" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1007" s="2" t="inlineStr"/>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B1008" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1008" s="2" t="inlineStr">
+        <is>
+          <t>+62 859-6034-6391</t>
+        </is>
+      </c>
+      <c r="D1008" s="2" t="inlineStr">
+        <is>
+          <t>SACHO NATA KANEMOCHI</t>
+        </is>
+      </c>
+      <c r="E1008" s="2" t="inlineStr">
+        <is>
+          <t>20:09</t>
+        </is>
+      </c>
+      <c r="F1008" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1008" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1008" s="2" t="inlineStr"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="2" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B1009" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1009" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-3984-6995</t>
+        </is>
+      </c>
+      <c r="D1009" s="2" t="inlineStr">
+        <is>
+          <t>L.Usman Jayadi</t>
+        </is>
+      </c>
+      <c r="E1009" s="2" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="F1009" s="2" t="inlineStr">
+        <is>
+          <t>Kalau utk Avanza New all brp harganya</t>
+        </is>
+      </c>
+      <c r="G1009" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1009" s="2" t="inlineStr"/>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B1010" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1010" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-4497-8496</t>
+        </is>
+      </c>
+      <c r="D1010" s="2" t="inlineStr">
+        <is>
+          <t>martinusangkat123</t>
+        </is>
+      </c>
+      <c r="E1010" s="2" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="F1010" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1010" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1010" s="2" t="inlineStr"/>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="2" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B1011" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1011" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4827-1569</t>
+        </is>
+      </c>
+      <c r="D1011" s="2" t="inlineStr">
+        <is>
+          <t>ARMY 99-1</t>
+        </is>
+      </c>
+      <c r="E1011" s="2" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="F1011" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1011" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1011" s="2" t="inlineStr"/>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="2" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B1012" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1012" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-9090-4042</t>
+        </is>
+      </c>
+      <c r="D1012" s="2" t="inlineStr">
+        <is>
+          <t>Mahreza Pradana</t>
+        </is>
+      </c>
+      <c r="E1012" s="2" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="F1012" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1012" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1012" s="2" t="inlineStr"/>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="2" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B1013" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1013" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-4494-9392</t>
+        </is>
+      </c>
+      <c r="D1013" s="2" t="inlineStr">
+        <is>
+          <t>Helenarlef</t>
+        </is>
+      </c>
+      <c r="E1013" s="2" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="F1013" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1013" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1013" s="2" t="inlineStr"/>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="2" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B1014" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C1014" s="2" t="inlineStr">
+        <is>
+          <t>+62 852-4121-0866</t>
+        </is>
+      </c>
+      <c r="D1014" s="2" t="inlineStr">
+        <is>
+          <t>Wyn Baliasa</t>
+        </is>
+      </c>
+      <c r="E1014" s="2" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="F1014" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1014" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1014" s="2" t="inlineStr"/>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="2" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B1015" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C1015" s="2" t="inlineStr">
+        <is>
+          <t>+62 813-7556-0642</t>
+        </is>
+      </c>
+      <c r="D1015" s="2" t="inlineStr">
+        <is>
+          <t>Rubiati Pane</t>
+        </is>
+      </c>
+      <c r="E1015" s="2" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="F1015" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1015" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1015" s="2" t="inlineStr"/>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="2" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B1016" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C1016" s="2" t="inlineStr">
+        <is>
+          <t>+62 812-9523-3417</t>
+        </is>
+      </c>
+      <c r="D1016" s="2" t="inlineStr">
+        <is>
+          <t>Peri .Qapi</t>
+        </is>
+      </c>
+      <c r="E1016" s="2" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="F1016" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1016" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1016" s="2" t="inlineStr"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="2" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B1017" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1017" s="2" t="inlineStr">
+        <is>
+          <t>+62 823-9642-9700</t>
+        </is>
+      </c>
+      <c r="D1017" s="2" t="inlineStr">
+        <is>
+          <t>Mustafa</t>
+        </is>
+      </c>
+      <c r="E1017" s="2" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="F1017" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare hrg BRP yaa</t>
+        </is>
+      </c>
+      <c r="G1017" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1017" s="2" t="inlineStr"/>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="2" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B1018" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1018" s="2" t="inlineStr">
+        <is>
+          <t>+62 822-4011-6201</t>
+        </is>
+      </c>
+      <c r="D1018" s="2" t="inlineStr">
+        <is>
+          <t>ayah Riyen</t>
+        </is>
+      </c>
+      <c r="E1018" s="2" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="F1018" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1018" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1018" s="2" t="inlineStr"/>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="2" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B1019" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C1019" s="2" t="inlineStr">
+        <is>
+          <t>+62 821-7676-4872</t>
+        </is>
+      </c>
+      <c r="D1019" s="2" t="inlineStr">
+        <is>
+          <t>Carianto</t>
+        </is>
+      </c>
+      <c r="E1019" s="2" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="F1019" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1019" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1019" s="2" t="inlineStr"/>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="2" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B1020" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1020" s="2" t="inlineStr">
+        <is>
+          <t>+62 898-9392-444</t>
+        </is>
+      </c>
+      <c r="D1020" s="2" t="inlineStr">
+        <is>
+          <t>Gema Bemi Azhar</t>
+        </is>
+      </c>
+      <c r="E1020" s="2" t="inlineStr">
+        <is>
+          <t>17:27</t>
+        </is>
+      </c>
+      <c r="F1020" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1020" s="2" t="inlineStr">
+        <is>
+          <t>Instagram - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1020" s="2" t="inlineStr"/>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="2" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B1021" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1021" s="2" t="inlineStr">
+        <is>
+          <t>+62 857-1740-2927</t>
+        </is>
+      </c>
+      <c r="D1021" s="2" t="inlineStr">
+        <is>
+          <t>Thimangjaya</t>
+        </is>
+      </c>
+      <c r="E1021" s="2" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="F1021" s="2" t="inlineStr">
+        <is>
+          <t>Halo! Bisakah saya mendapatkan info selengkapnya tentang ini?</t>
+        </is>
+      </c>
+      <c r="G1021" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp (Video)</t>
+        </is>
+      </c>
+      <c r="H1021" s="2" t="inlineStr"/>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="2" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B1022" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1022" s="2" t="inlineStr">
+        <is>
+          <t>+62 888-1851-778</t>
+        </is>
+      </c>
+      <c r="D1022" s="2" t="inlineStr">
+        <is>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="E1022" s="2" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="F1022" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1022" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1022" s="2" t="inlineStr"/>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="2" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B1023" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1023" s="2" t="inlineStr">
+        <is>
+          <t>+62 895-1437-3920</t>
+        </is>
+      </c>
+      <c r="D1023" s="2" t="inlineStr">
+        <is>
+          <t>Agus</t>
+        </is>
+      </c>
+      <c r="E1023" s="2" t="inlineStr">
+        <is>
+          <t>10:23</t>
+        </is>
+      </c>
+      <c r="F1023" s="2" t="inlineStr">
+        <is>
+          <t>Halo kak, saya ingin cek Stok &amp; Promo Cover Reguler Undercover Autocare</t>
+        </is>
+      </c>
+      <c r="G1023" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1023" s="2" t="inlineStr"/>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="2" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B1024" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C1024" s="2" t="inlineStr">
+        <is>
+          <t>+62 858-0122-3317</t>
+        </is>
+      </c>
+      <c r="D1024" s="2" t="inlineStr">
+        <is>
+          <t>Han han</t>
+        </is>
+      </c>
+      <c r="E1024" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="F1024" s="2" t="inlineStr">
+        <is>
+          <t>Kak mau tanya kalau caver untuk mobil avanza 2010 berapa harganya</t>
+        </is>
+      </c>
+      <c r="G1024" s="2" t="inlineStr">
+        <is>
+          <t>Facebook - Whatsapp</t>
+        </is>
+      </c>
+      <c r="H1024" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>